<commit_message>
fix(lib): RS.MI-1.1 correction on cyfun 2023
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
+++ b/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="cff_meta" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="cff_content" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="implementation_groups_meta" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="implementation_groups_content" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cff_meta" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cff_content" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="implementation_groups_meta" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="implementation_groups_content" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -124,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -201,6 +203,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,7 +604,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -611,10 +614,8 @@
           <t>publication_date</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2025-06-18 00:00:00</t>
-        </is>
+      <c r="B4" s="30" t="n">
+        <v>46255</v>
       </c>
     </row>
     <row r="5">
@@ -948,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M351"/>
+  <dimension ref="A1:M347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1052,8 +1053,6 @@
           <t>IDENTIFIER (ID)</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" s="7" t="inlineStr">
         <is>
           <t>IDENTIFICEREN (ID)</t>
@@ -1089,7 +1088,6 @@
           <t>Les données, le personnel, les dispositifs, les systèmes et les installations qui permettent à l'organisation d'atteindre ses objectifs opérationnels sont identifiés et gérés en fonction de leur importance relative par rapport aux objectifs de l'organisation et à sa stratégie en matière de risques.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" s="11" t="inlineStr">
         <is>
           <t>Vermogensbeheer</t>
@@ -1120,7 +1118,6 @@
           <t>Les dispositifs et systèmes physiques utilisés dans l'organisation sont inventoriés.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="L4" s="16" t="inlineStr">
         <is>
           <t>Inventarisatie van de binnen de organisatie gebruikte fysieke apparaten en systemen.</t>
@@ -1364,7 +1361,6 @@
           <t>Les plateformes et applications logicielles utilisées au sein de l'organisation sont inventoriées.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="L9" s="16" t="inlineStr">
         <is>
           <t>Inventarisatie van de binnen de organisatie gebruikte softwareplatforms en - toepassingen.</t>
@@ -1658,7 +1654,6 @@
           <t>La communication organisationnelle et les flux de données sont schématisés.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="L15" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve"> De organisatorische communicatie- en gegevensstromen worden in kaart gebracht.</t>
@@ -1858,7 +1853,6 @@
           <t xml:space="preserve"> Les systèmes d'information externes sont catalogués.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="L19" s="16" t="inlineStr">
         <is>
           <t>Externe informatiesystemen worden gecatalogiseerd.</t>
@@ -1990,7 +1984,6 @@
           <t>Les ressources sont organisées par ordre de priorité en fonction de leur classification, de leur criticité et de leur valeur opérationnelle.</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="L22" s="16" t="inlineStr">
         <is>
           <t>Middelen worden geprioriteerd op basis van hun classificatie, kriticiteit en bedrijfswaarde.</t>
@@ -2099,7 +2092,6 @@
           <t>Les rôles, responsabilités et pouvoirs en matière de cybersécurité pour l'ensemble du personnel et les parties prenantes tierces (par exemple, les fournisseurs, les clients, les partenaires) sont établis.</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
       <c r="L24" s="16" t="inlineStr">
         <is>
           <t>Rollen, verantwoordelijkheden en bevoegdheden op het gebied van informatie- en cyberbeveiliging worden vastgesteld voor het gehele personeel en belanghebbenden van derden.</t>
@@ -2244,7 +2236,6 @@
           <t>La mission, les objectifs, les parties prenantes et les activités de l'organisation sont compris et classés par ordre de priorité ; ces informations sont utilisées pour définir les rôles, les responsabilités et les décisions en matière de gestion des risques liés à la cybersécurité.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" s="11" t="inlineStr">
         <is>
           <t>Bedrijfsomgeving</t>
@@ -2275,7 +2266,6 @@
           <t>Le rôle de l'organisation dans la chaîne d'approvisionnement est identifié et communiqué.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="L28" s="16" t="inlineStr">
         <is>
           <t>De rol van de organisatie in de toeleveringsketen wordt vastgesteld en gecommuniceerd.</t>
@@ -2403,7 +2393,6 @@
           <t>La place de l'organisation dans les infrastructures critiques et son secteur d'activité est identifiée et communiquée.</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="L31" s="16" t="inlineStr">
         <is>
           <t>De plaats van de organisatie in de kritieke infrastructuur en haar bedrijfstak wordt vastgesteld en gecommuniceerd.</t>
@@ -2554,7 +2543,6 @@
           <t>Les dépendances et les fonctions critiques pour la prestation des services critiques sont établies.</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="L35" s="16" t="inlineStr">
         <is>
           <t>Afhankelijkheden en kritieke functies voor de levering van kritieke diensten zijn vastgesteld.</t>
@@ -2630,7 +2618,6 @@
           <t>Les exigences en matière de résilience pour soutenir la prestation de services essentiels sont établies pour tous les états de fonctionnement (par exemple, en cas de contrainte/attaque, pendant le rétablissement, les opérations normales).</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="L37" s="16" t="inlineStr">
         <is>
           <t>Voor alle operationele staten (bv. onder dwang/aanval, tijdens herstel, normale operaties) worden vereisten vastgesteld met betrekking tot weerbaarheid ter ondersteuning van de levering van kritieke diensten.</t>
@@ -2824,7 +2811,6 @@
           <t>Les politiques, procédures et processus de gestion et de suivi des exigences réglementaires, juridiques, environnementales et opérationnelles de l'organisation sont compris et contribuent à la gestion du risque de cybersécurité.</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" s="11" t="inlineStr">
         <is>
           <t>Bestuur</t>
@@ -2855,7 +2841,6 @@
           <t>La politique de cybersécurité de l'organisation est établie et communiquée .</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
       <c r="L42" s="16" t="inlineStr">
         <is>
           <t>Het cyberbeveiligingsbeleid van de organisatie wordt vastgesteld en gecommuniceerd.</t>
@@ -2995,7 +2980,6 @@
           <t>Les exigences légales et réglementaires concernant la cybersécurité, y compris les obligations en matière de vie privée et de libertés civiles, sont comprises et gérées .</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
       <c r="L45" s="16" t="inlineStr">
         <is>
           <t>Wettelijke en regelgevende voorschriften inzake cyberbeveiliging, met inbegrip van verplichtingen inzake privacy en burgerlijke vrijheden, worden begrepen en beheerd.</t>
@@ -3124,7 +3108,6 @@
           <t>Les processus de gouvernance et de gestion des risques traitent les risques de cybersécurité .</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
       <c r="L48" s="16" t="inlineStr">
         <is>
           <t>Governance- en risicobeheerprocessen adresseren risico's met betrekking tot cyberbeveiliging.</t>
@@ -3260,7 +3243,6 @@
           <t>L'organisation comprend le risque de cybersécurité pour les opérations de l'organisation (y compris la mission, les fonctions, l'image ou la réputation), ses actifs et les individus.</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" s="11" t="inlineStr">
         <is>
           <t>Risicobeoordeling</t>
@@ -3291,7 +3273,6 @@
           <t xml:space="preserve"> Les vulnérabilités des actifs sont identifiées et documentées.</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
       <c r="L52" s="16" t="inlineStr">
         <is>
           <t>Kwetsbaarheden van activa worden vastgesteld en gedocumenteerd.</t>
@@ -3475,7 +3456,6 @@
           <t>Les renseignements sur les cybermenaces sont reçus de forums de partage d'informations et de sources.</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
       <c r="L56" s="16" t="inlineStr">
         <is>
           <t>Informatie over cyberdreigingen wordt ontvangen van fora en bronnen voor informatie-uitwisseling.</t>
@@ -3601,7 +3581,6 @@
           <t>Les menaces, les vulnérabilités, les probabilités et les impacts sont utilisés pour déterminer les risques.</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
       <c r="L59" s="16" t="inlineStr">
         <is>
           <t>Bedreigingen, kwetsbaarheden, waarschijnlijkheden en gevolgen worden gebruikt om het risico te bepalen.</t>
@@ -3784,7 +3763,6 @@
           <t>Les réponses aux risques sont identifiées et classées par ordre de priorité.</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
       <c r="L63" s="16" t="inlineStr">
         <is>
           <t>Respons op risico’s worden vastgesteld en geprioriteerd.</t>
@@ -3879,7 +3857,6 @@
           <t>Les priorités, contraintes, tolérances au risque et hypothèses de l'organisation sont établies et utilisées pour soutenir les décisions relatives au risque opérationnel.</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
       <c r="K65" s="11" t="inlineStr">
         <is>
           <t>Risicobeheer</t>
@@ -3910,7 +3887,6 @@
           <t>Les processus de gestion des risques sont établis, gérés et acceptés par les parties prenantes de l’organisation.</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
       <c r="L66" s="16" t="inlineStr">
         <is>
           <t>Risicobeheerprocessen worden vastgesteld, beheerd en goedgekeurd door belanghebbenden in de organisatie.</t>
@@ -3986,7 +3962,6 @@
           <t>La tolérance de l'organisation au risque est déterminée et clairement exprimée.</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
       <c r="L68" s="16" t="inlineStr">
         <is>
           <t>De risicotolerantie van de organisatie wordt bepaald en duidelijk uitgedrukt.</t>
@@ -4062,7 +4037,6 @@
           <t>La détermination de la tolérance au risque de l'organisation est éclairée par son rôle dans l'infrastructure critique et l'analyse des risques spécifiques au secteur.</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
       <c r="L70" s="16" t="inlineStr">
         <is>
           <t>De organisatie bepaalt haar risicotolerantie op basis van haar rol in de analyse van kritieke infrastructuur en sectorspecifieke risico's.</t>
@@ -4148,7 +4122,6 @@
           <t>Les priorités, les contraintes, les tolérances au risque et les hypothèses de l'organisation sont établies et utilisées pour soutenir les décisions liées à la gestion des risques de la chaîne d'approvisionnement. L'organisation a établi et mis en œuvre les processus pour identifier, évaluer et gérer les risques liés à la chaîne d'approvisionnement.</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
       <c r="K72" s="11" t="inlineStr">
         <is>
           <t>Risicobeheer van de toeleveringsketen</t>
@@ -4179,7 +4152,6 @@
           <t>Les processus de gestion des risques liés à la chaîne d'approvisionnement sont identifiés, établis, évalués, gérés et acceptés par les parties prenantes de l'organisation.</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
       <c r="L73" s="16" t="inlineStr">
         <is>
           <t>De processen voor het beheer van cyberrisico's in de toeleveringsketen worden geïdentificeerd, vastgesteld, beoordeeld, beheerd en goedgekeurd door de belanghebbenden van de organisatie.</t>
@@ -4255,7 +4227,6 @@
           <t>Les fournisseurs et les partenaires tiers de systèmes d'information, de composants et de services sont identifiés, classés par ordre de priorité et évalués à l'aide d'un processus d'évaluation des risques de la cyberchaîne d’approvisionnement.</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
       <c r="L75" s="16" t="inlineStr">
         <is>
           <t>Leveranciers en externe partners van informatiesystemen, componenten en diensten worden geïdentificeerd, geprioriteerd en beoordeeld met behulp van een risicobeoordelingsproces voor de cybertoeleveringsketen.</t>
@@ -4381,7 +4352,6 @@
           <t>Les contrats avec les fournisseurs et les partenaires tiers sont utilisés pour mettre en œuvre des mesures appropriées conçues pour atteindre les objectifs du programme de cybersécurité et du plan de gestion des risques de la chaîne d'approvisionnement de l'organisation.</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
       <c r="L78" s="16" t="inlineStr">
         <is>
           <t>Contracten met leveranciers en externe partners worden gebruikt om passende maatregelen te implementeren, die dermate zijn ontworpen opdat wordt beantwoord aan de doelstellingen van het cyberbeveiligingsprogramma van de organisatie en haar cyber risicobeheersplan voor de toeleveringsketen.</t>
@@ -4563,7 +4533,6 @@
           <t>Les fournisseurs et les partenaires tiers sont régulièrement évalués à l'aide d'audits, de résultats de tests ou d'autres formes d'évaluation pour confirmer qu'ils respectent leurs obligations contractuelles.</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
       <c r="L82" s="16" t="inlineStr">
         <is>
           <t>Leveranciers en externe partners worden routinematig beoordeeld aan de hand van audits, testresultaten of andere vormen van evaluaties om te bevestigen dat zij aan hun contractuele verplichtingen voldoen.</t>
@@ -4689,7 +4658,6 @@
           <t>La planification et les tests de réponse et de rétablissement sont effectués avec les fournisseurs et les prestataires tiers.</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
       <c r="L85" s="16" t="inlineStr">
         <is>
           <t>Respons- en herstelplanning en tests worden uitgevoerd met leveranciers en derde partijen.</t>
@@ -4815,7 +4783,6 @@
           <t>PROTEGER (PR)</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
       <c r="K88" s="7" t="inlineStr">
         <is>
           <t>BESCHERMEN (PR)</t>
@@ -4851,7 +4818,6 @@
           <t>L'accès aux actifs physiques et logiques et aux installations associées est limité aux utilisateurs, processus et dispositifs autorisés, et est géré en fonction du risque évalué d'accès non autorisé aux activités et transactions autorisées.</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" s="11" t="inlineStr">
         <is>
           <t>Identiteitsbeheer, authenticatie en toegangscontrole</t>
@@ -4882,7 +4848,6 @@
           <t>Les identités et les identifiants sont émis, gérés, vérifiés, révoqués et audités pour les dispositifs, utilisateurs et processus autorisés.</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
       <c r="L90" s="16" t="inlineStr">
         <is>
           <t>Identiteiten en referenties (“credentials”) worden afgegeven, beheerd, geverifieerd, ingetrokken en gecontroleerd voor geautoriseerde apparaten, gebruikers en processen.</t>
@@ -5194,7 +5159,6 @@
           <t>L'accès physique aux actifs est géré et protégé.</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
       <c r="L96" s="16" t="inlineStr">
         <is>
           <t>De fysieke toegang tot activa wordt beheerd en beschermd.</t>
@@ -5449,7 +5413,6 @@
           <t>L'accès à distance est géré.</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
       <c r="L101" s="16" t="inlineStr">
         <is>
           <t>De toegang op afstand wordt beheerd.</t>
@@ -5755,7 +5718,6 @@
           <t>Les permissions et autorisations d'accès sont gérées en intégrant les principes du moindre privilège et de la séparation des tâches.</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
       <c r="L107" s="16" t="inlineStr">
         <is>
           <t>De toegangsrechten en machtigingen worden beheerd, met inachtneming van de beginselen van "least privilege" en scheiding van taken.</t>
@@ -6283,7 +6245,6 @@
           <t>L'intégrité du réseau (séparation du réseau, segmentation du réseau...) est protégée.</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
       <c r="L117" s="16" t="inlineStr">
         <is>
           <t>Netwerkintegriteit (netwerksegregatie, netwerksegmentatie...) wordt beschermd.</t>
@@ -6654,7 +6615,6 @@
           <t>Les identités sont prouvées et liées aux identifiants et présentées dans les interactions.</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
       <c r="L124" s="16" t="inlineStr">
         <is>
           <t>Identiteiten worden aangetoond en verbonden aan referenties (“credentials”) en bevestigd in interacties.</t>
@@ -6780,7 +6740,6 @@
           <t>Les utilisateurs, les appareils et les autres actifs sont authentifiés (par exemple, à un seul facteur, à plusieurs facteurs) en fonction du risque de la transaction (par exemple, les risques pour la sécurité et la confidentialité des individus et d’autres risques organisationnels)</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr"/>
       <c r="L127" s="16" t="inlineStr">
         <is>
           <t>Identiteiten worden aangetoond en verbonden aan referenties (“credentials”) en bevestigd in interacties.</t>
@@ -6866,7 +6825,6 @@
           <t>Le personnel et les partenaires de l'organisation reçoivent une formation de sensibilisation à la cybersécurité et sont formés à l'exécution de leurs tâches et responsabilités liées à la cybersécurité, conformément aux politiques, procédures et accords connexes.</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr"/>
       <c r="K129" s="11" t="inlineStr">
         <is>
           <t>Bewustmaking en opleiding</t>
@@ -6897,7 +6855,6 @@
           <t>Tous les utilisateurs sont informés et entrainés.</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr"/>
       <c r="L130" s="16" t="inlineStr">
         <is>
           <t>Alle gebruikers worden geïnformeerd en opgeleid.</t>
@@ -7091,7 +7048,6 @@
           <t xml:space="preserve"> Les utilisateurs privilégiés comprennent leurs rôles et leurs responsabilités.</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr"/>
       <c r="L134" s="16" t="inlineStr">
         <is>
           <t>Geprivilegieerde gebruikers begrijpen hun rollen en verantwoordelijkheden.</t>
@@ -7167,7 +7123,6 @@
           <t>Les parties prenantes tierces (par exemple, les fournisseurs, les clients, les partenaires) comprennent leurs rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
       <c r="L136" s="16" t="inlineStr">
         <is>
           <t>Belanghebbenden van derden (bijv. leveranciers, klanten, partners) begrijpen hun rol en verantwoordelijkheden.</t>
@@ -7393,7 +7348,6 @@
           <t>Les cadres supérieurs comprennent leurs rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
       <c r="L141" s="16" t="inlineStr">
         <is>
           <t>Hogere leidinggevenden begrijpen hun taken en verantwoordelijkheden.</t>
@@ -7469,7 +7423,6 @@
           <t>Le personnel de la sécurité physique et de la cybersécurité comprend ses rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr"/>
       <c r="L143" s="16" t="inlineStr">
         <is>
           <t>Fysiek en cyberbeveiligingspersoneel begrijpt hun rollen en verantwoordelijkheden.</t>
@@ -7555,7 +7508,6 @@
           <t>Les informations et les enregistrements (données) sont gérés conformément à la stratégie de l'organisation en matière de risques afin de protéger la confidentialité, l'intégrité et la disponibilité des informations.</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
       <c r="K145" s="12" t="inlineStr">
         <is>
           <t>Gegevensbeveiliging</t>
@@ -7586,7 +7538,6 @@
           <t>Les données au repos sont protégées.</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
       <c r="L146" s="15" t="inlineStr">
         <is>
           <t>Data in rust is beschermd.</t>
@@ -7674,7 +7625,6 @@
           <t>Les données en transit sont protégées.</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
       <c r="L148" s="16" t="inlineStr">
         <is>
           <t>Data-in-transitie is beschermd.</t>
@@ -7751,7 +7701,6 @@
           <t>Les actifs sont gérés de manière formelle tout au long de leur retrait, de leur transfert et de leur mise à disposition.</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
       <c r="L150" s="16" t="inlineStr">
         <is>
           <t>Activa worden formeel beheerd gedurende de verhuizing, overdracht en verwijdering.</t>
@@ -7986,7 +7935,6 @@
           <t>Une capacité adéquate pour assurer la disponibilité est maintenue.</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
       <c r="L155" s="16" t="inlineStr">
         <is>
           <t>Voldoende capaciteit om de beschikbaarheid te waarborgen.</t>
@@ -8162,7 +8110,6 @@
           <t>Les protections contre les fuites de données sont mises en œuvre.</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
       <c r="L159" s="16" t="inlineStr">
         <is>
           <t>Beveiligingen tegen datalekken worden geïmplementeerd.</t>
@@ -8241,7 +8188,6 @@
           <t>Des mécanismes de vérification de l'intégrité sont utilisés pour vérifier l'intégrité des logiciels, des microprogrammes et des informations.</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr"/>
       <c r="L161" s="16" t="inlineStr">
         <is>
           <t>Integriteitscontrolemechanismen worden gebruikt om de integriteit van software, firmware en informatie te controleren.</t>
@@ -8417,7 +8363,6 @@
           <t>L'environnement ou les environnements de développement et de test sont séparés de l'environnement de production.</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr"/>
       <c r="L165" s="16" t="inlineStr">
         <is>
           <t>De ontwikkelings- en testomgeving(en) zijn gescheiden van de productieomgeving.</t>
@@ -8497,7 +8442,6 @@
           <t>Les mécanismes de contrôle d'intégrité sont utilisés pour vérifier l'intégrité du matériel.</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr"/>
       <c r="L167" s="16" t="inlineStr">
         <is>
           <t>Integriteitscontrolemechanismen worden gebruikt om de integriteit van de hardware te verifiëren.</t>
@@ -8633,7 +8577,6 @@
           <t>Les politiques de sécurité (qui traitent de l'objectif, de la portée, des rôles, des responsabilités, de l'engagement de la direction et de la coordination entre les entités organisationnelles), les processus et les procédures sont maintenus et utilisés pour gérer la protection des systèmes d'information et des actifs.</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr"/>
       <c r="K170" s="11" t="inlineStr">
         <is>
           <t>Informatiebeschermingsprocessen en - procedures</t>
@@ -8664,7 +8607,6 @@
           <t>Une configuration de base des systèmes de contrôle des technologies de l'information/de l'industrie est créée et maintenue en intégrant les principes de sécurité.</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr"/>
       <c r="L171" s="16" t="inlineStr">
         <is>
           <t>Er wordt een basisconfiguratie van informatietechnologie/industriële controlesystemen gecreëerd en onderhouden, waarin de beveiligingsbeginselen zijn verwerkt .</t>
@@ -8798,7 +8740,6 @@
           <t>Un cycle de vie du développement des systèmes pour gérer les systèmes est mis en œuvre .</t>
         </is>
       </c>
-      <c r="J174" t="inlineStr"/>
       <c r="L174" s="16" t="inlineStr">
         <is>
           <t>Een levenscyclus voor systeemontwikkeling om systemen te beheren wordt geïmplementeerd.</t>
@@ -8942,7 +8883,6 @@
           <t>Des processus de contrôle des changements de configuration sont en place.</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr"/>
       <c r="L177" s="16" t="inlineStr">
         <is>
           <t>Er zijn processen voor het beheer van configuratiewijzigingen aanwezig.</t>
@@ -9068,7 +9008,6 @@
           <t>Des sauvegardes des informations sont effectuées, maintenues et testées .</t>
         </is>
       </c>
-      <c r="J180" t="inlineStr"/>
       <c r="L180" s="16" t="inlineStr">
         <is>
           <t>Er worden back-ups van informatie gemaakt, onderhouden en getest.</t>
@@ -9356,7 +9295,6 @@
           <t>La politique et les règlements concernant l'environnement physique d'exploitation des actifs de l'organisation sont respectés.</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr"/>
       <c r="L186" s="16" t="inlineStr">
         <is>
           <t>Beleid en voorschriften met betrekking tot de fysieke bedrijfsomgeving voor bedrijfsmiddelen van de organisatie worden nageleefd .</t>
@@ -9488,7 +9426,6 @@
           <t>Les données sont détruites conformément à la politique.</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr"/>
       <c r="L189" s="16" t="inlineStr">
         <is>
           <t>Gegevens worden vernietigd overeenkomstig beleid.</t>
@@ -9629,7 +9566,6 @@
           <t>Les processus de protection sont améliorés</t>
         </is>
       </c>
-      <c r="J192" t="inlineStr"/>
       <c r="L192" s="16" t="inlineStr">
         <is>
           <t>De beschermingsprocessen worden verbeterd.</t>
@@ -9808,7 +9744,6 @@
           <t>L'efficacité des technologies de protection est partagée.</t>
         </is>
       </c>
-      <c r="J196" t="inlineStr"/>
       <c r="L196" s="16" t="inlineStr">
         <is>
           <t>De doeltreffendheid van beschermingstechnologieën wordt gedeeld.</t>
@@ -9984,7 +9919,6 @@
           <t>Des plans de réponse (réponse aux incidents et continuité des activités) et des plans de rétablissement (reprise après incident et reprise après sinistre) sont en place et gérés.</t>
         </is>
       </c>
-      <c r="J200" t="inlineStr"/>
       <c r="L200" s="16" t="inlineStr">
         <is>
           <t>Responsplannen (Incident Response en Business Continuity) en herstelplannen (Incident Recovery en Disaster Recovery) zijn aanwezig en worden beheerd.</t>
@@ -10119,7 +10053,6 @@
           <t>La cybersécurité est incluse dans les pratiques de ressources humaines (déprovisionnement, sélection du personnel...).</t>
         </is>
       </c>
-      <c r="J203" t="inlineStr"/>
       <c r="L203" s="16" t="inlineStr">
         <is>
           <t>Cyberbeveiliging is opgenomen in de personeelsbeheer (afbouwen, personeelsscreening...).</t>
@@ -10248,7 +10181,6 @@
           <t>Un plan de gestion des vulnérabilités est élaboré et mis en œuvre.</t>
         </is>
       </c>
-      <c r="J206" t="inlineStr"/>
       <c r="L206" s="16" t="inlineStr">
         <is>
           <t>Een plan voor het beheer van kwetsbaarheden wordt ontwikkeld en uitgevoerd.</t>
@@ -10337,7 +10269,6 @@
           <t>La maintenance et la réparation des composants des systèmes de contrôle et d'information industriels sont effectuées conformément aux politiques et procédures.</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr"/>
       <c r="K208" s="11" t="inlineStr">
         <is>
           <t>Onderhoud</t>
@@ -10368,7 +10299,6 @@
           <t>L'entretien et la réparation des actifs de l'organisation sont effectués et consignés, avec des outils approuvés et contrôlés.</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr"/>
       <c r="L209" s="16" t="inlineStr">
         <is>
           <t>Onderhoud en reparatie van bedrijfsmiddelen van de organisatie worden uitgevoerd en geregistreerd, met goedgekeurde en gecontroleerde gereedschappen.</t>
@@ -10754,7 +10684,6 @@
           <t>La maintenance à distance des actifs de l'organisation est approuvée, consignée et effectuée de manière à empêcher tout accès non autorisé.</t>
         </is>
       </c>
-      <c r="J217" t="inlineStr"/>
       <c r="L217" s="16" t="inlineStr">
         <is>
           <t>Onderhoud op afstand van bedrijfsmiddelen van de organisatie moet worden goedgekeurd, geregistreerd en uitgevoerd op een wijze die ongeoorloofde toegang voorkomt.</t>
@@ -10940,7 +10869,6 @@
           <t>Les solutions de sécurité technique sont gérées de manière à garantir la sécurité et la résilience des systèmes et des actifs, conformément aux politiques, procédures et accords connexes.</t>
         </is>
       </c>
-      <c r="J221" t="inlineStr"/>
       <c r="K221" s="11" t="inlineStr">
         <is>
           <t>Beschermingstechnologie</t>
@@ -10971,7 +10899,6 @@
           <t>Les enregistrements d'audit/logs sont déterminés, documentés, mis en œuvre et révisés conformément à la politique.</t>
         </is>
       </c>
-      <c r="J222" t="inlineStr"/>
       <c r="L222" s="16" t="inlineStr">
         <is>
           <t>Registraties van audits/logs worden vastgesteld, gedocumenteerd, uitgevoerd en herzien overeenkomstig beleid.</t>
@@ -11203,7 +11130,6 @@
           <t>Les supports amovibles sont protégés et leur utilisation est limitée conformément à la politique.</t>
         </is>
       </c>
-      <c r="J227" t="inlineStr"/>
       <c r="L227" s="16" t="inlineStr">
         <is>
           <t>Verwisselbare media worden beschermd en het gebruik ervan wordt beperkt overeenkomstig het beleid.</t>
@@ -11379,7 +11305,6 @@
           <t>Le principe de la moindre fonctionnalité est incorporé en configurant les systèmes de manière à ne fournir que les capacités essentielles.</t>
         </is>
       </c>
-      <c r="J231" t="inlineStr"/>
       <c r="L231" s="16" t="inlineStr">
         <is>
           <t>Het beginsel van minimale functionaliteit wordt toegepast door systemen zo te configureren dat ze alleen essentiële mogelijkheden bieden.</t>
@@ -11555,7 +11480,6 @@
           <t>Les réseaux de communication et de contrôle sont protégés.</t>
         </is>
       </c>
-      <c r="J235" t="inlineStr"/>
       <c r="L235" s="16" t="inlineStr">
         <is>
           <t>Communicatie- en besturingsnetwerken zijn beveiligd.</t>
@@ -11743,7 +11667,6 @@
           <t>DETECTER (DE)</t>
         </is>
       </c>
-      <c r="J239" t="inlineStr"/>
       <c r="K239" s="7" t="inlineStr">
         <is>
           <t>DETECTEREN (DE)</t>
@@ -11774,8 +11697,6 @@
           <t>Anomalies et événements</t>
         </is>
       </c>
-      <c r="I240" t="inlineStr"/>
-      <c r="J240" t="inlineStr"/>
       <c r="K240" s="11" t="inlineStr">
         <is>
           <t>Anomalieën en gebeurtenissen</t>
@@ -11806,7 +11727,6 @@
           <t>Une base de référence des opérations du réseau et des flux de données attendus pour les utilisateurs et les systèmes est établie et gérée.</t>
         </is>
       </c>
-      <c r="J241" t="inlineStr"/>
       <c r="L241" s="16" t="inlineStr">
         <is>
           <t>Een baseline van netwerkoperaties en verwachte gegevensstromen voor gebruikers en systemen wordt vastgesteld en beheerd.</t>
@@ -11891,7 +11811,6 @@
           <t>Les événements détectés sont analysés pour comprendre les cibles et les méthodes d’attaque.</t>
         </is>
       </c>
-      <c r="J243" t="inlineStr"/>
       <c r="L243" s="16" t="inlineStr">
         <is>
           <t>Gedetecteerde events worden geanalyseerd om inzicht te krijgen in aanvalsdoelen en -methoden.</t>
@@ -12017,7 +11936,6 @@
           <t>Les données d'événements sont collectées et corrélées à partir de sources et de capteurs multiples.</t>
         </is>
       </c>
-      <c r="J246" t="inlineStr"/>
       <c r="L246" s="16" t="inlineStr">
         <is>
           <t>Gegevens m.b.t. events worden verzameld en gecorreleerd uit meerdere bronnen en sensoren.</t>
@@ -12197,7 +12115,6 @@
           <t>L'impact des événements est déterminé.</t>
         </is>
       </c>
-      <c r="J250" t="inlineStr"/>
       <c r="L250" s="16" t="inlineStr">
         <is>
           <t>De impact van events wordt bepaald.</t>
@@ -12273,7 +12190,6 @@
           <t>Les seuils d'alerte des incidents sont établis.</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr"/>
       <c r="L252" s="16" t="inlineStr">
         <is>
           <t>Er worden alarmdrempels voor incidenten vastgesteld.</t>
@@ -12409,7 +12325,6 @@
           <t>Le système d'information et les actifs sont surveillés pour identifier les événements de cybersécurité et vérifier l'efficacité des mesures de protection.</t>
         </is>
       </c>
-      <c r="J255" t="inlineStr"/>
       <c r="K255" s="11" t="inlineStr">
         <is>
           <t>Voortdurende bewaking van de beveiliging</t>
@@ -12440,7 +12355,6 @@
           <t>Le réseau est surveillé pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
       <c r="L256" s="16" t="inlineStr">
         <is>
           <t>Het netwerk wordt gemonitord om potentiële cyberbeveiligingsevents op te sporen.</t>
@@ -12637,7 +12551,6 @@
           <t>L'environnement physique est surveillé pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J260" t="inlineStr"/>
       <c r="L260" s="16" t="inlineStr">
         <is>
           <t>De fysieke omgeving wordt bewaakt om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -12763,7 +12676,6 @@
           <t>L'activité du personnel est surveillée pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J263" t="inlineStr"/>
       <c r="L263" s="16" t="inlineStr">
         <is>
           <t>Personeelsactiviteiten worden gemonitord om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -12941,7 +12853,6 @@
           <t>Le code malveillant est détecté.</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr"/>
       <c r="L267" s="16" t="inlineStr">
         <is>
           <t>Kwaadaardige code wordt gedetecteerd.</t>
@@ -13073,7 +12984,6 @@
           <t>Un code mobile non autorisé est détecté.</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr"/>
       <c r="L270" s="16" t="inlineStr">
         <is>
           <t>Ongeoorloofde mobiele code is gedetecteerd.</t>
@@ -13152,7 +13062,6 @@
           <t>L'activité des prestataires de services externes est surveillée pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr"/>
       <c r="L272" s="16" t="inlineStr">
         <is>
           <t>De activiteit van externe dienstverleners wordt gemonitord om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -13278,7 +13187,6 @@
           <t>La surveillance du personnel, des connexions, des dispositifs et des logiciels non autorisés est effectuée.</t>
         </is>
       </c>
-      <c r="J275" t="inlineStr"/>
       <c r="L275" s="16" t="inlineStr">
         <is>
           <t>Monitoring op onbevoegd personeel, verbindingen, apparatuur en software wordt uitgevoerd.</t>
@@ -13410,7 +13318,6 @@
           <t>Les analyses de vulnérabilité sont effectuées.</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr"/>
       <c r="L278" s="16" t="inlineStr">
         <is>
           <t>Kwetsbaarheidsscans worden uitgevoerd.</t>
@@ -13546,7 +13453,6 @@
           <t>Les processus et procédures de détection sont maintenus et testés pour garantir la prise de conscience des événements anormaux.</t>
         </is>
       </c>
-      <c r="J281" t="inlineStr"/>
       <c r="K281" s="11" t="inlineStr">
         <is>
           <t>Opsporingsprocessen</t>
@@ -13577,7 +13483,6 @@
           <t>Les activités de détection sont conformes à toutes les exigences applicables.</t>
         </is>
       </c>
-      <c r="J282" t="inlineStr"/>
       <c r="L282" s="16" t="inlineStr">
         <is>
           <t>Detectie moet gebeuren conform alle toepasselijke eisen.</t>
@@ -13653,7 +13558,6 @@
           <t>Les processus de détection sont testés.</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr"/>
       <c r="L284" s="16" t="inlineStr">
         <is>
           <t>Detectieprocessen worden getest.</t>
@@ -13732,7 +13636,6 @@
           <t>Les informations relatives à la détection des événements sont communiquées.</t>
         </is>
       </c>
-      <c r="J286" t="inlineStr"/>
       <c r="L286" s="16" t="inlineStr">
         <is>
           <t>Informatie over gedetecteerde events wordt gecommuniceerd.</t>
@@ -13808,7 +13711,6 @@
           <t>Les processus de détection sont améliorés en permanence.</t>
         </is>
       </c>
-      <c r="J288" t="inlineStr"/>
       <c r="L288" s="16" t="inlineStr">
         <is>
           <t>De processen voor het detecteren van abnormale events worden voortdurend verbeterd.</t>
@@ -13937,8 +13839,6 @@
           <t>REPONDRE (RS)</t>
         </is>
       </c>
-      <c r="I291" t="inlineStr"/>
-      <c r="J291" t="inlineStr"/>
       <c r="K291" s="7" t="inlineStr">
         <is>
           <t>REAGEREN (RS)</t>
@@ -13974,7 +13874,6 @@
           <t>Les processus et procédures de réponse sont exécutés et maintenus, afin de garantir une réponse aux incidents de cybersécurité détectés.</t>
         </is>
       </c>
-      <c r="J292" t="inlineStr"/>
       <c r="K292" s="11" t="inlineStr">
         <is>
           <t>Responsplanning</t>
@@ -14005,7 +13904,6 @@
           <t xml:space="preserve"> Le plan de réponse est exécuté pendant ou après un incident.</t>
         </is>
       </c>
-      <c r="J293" t="inlineStr"/>
       <c r="L293" s="16" t="inlineStr">
         <is>
           <t>Het responsplan wordt uitgevoerd tijdens of na een incident.</t>
@@ -14097,7 +13995,6 @@
           <t>Les activités de réponse sont coordonnées avec les parties prenantes internes et externes (par exemple, le soutien externe des forces de l'ordre).</t>
         </is>
       </c>
-      <c r="J295" t="inlineStr"/>
       <c r="K295" s="11" t="inlineStr">
         <is>
           <t>Communicatie</t>
@@ -14128,7 +14025,6 @@
           <t>Le personnel connaît ses rôles et l'ordre des opérations lorsqu'une réponse est nécessaire.</t>
         </is>
       </c>
-      <c r="J296" t="inlineStr"/>
       <c r="L296" s="16" t="inlineStr">
         <is>
           <t>Het personeel kent zijn rol en volgorde van handelen wanneer een reactie nodig is.</t>
@@ -14204,7 +14100,6 @@
           <t>Les incidents sont signalés conformément aux critères établis.</t>
         </is>
       </c>
-      <c r="J298" t="inlineStr"/>
       <c r="L298" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden gemeld overeenkomstig de vastgestelde criteria.</t>
@@ -14330,7 +14225,6 @@
           <t>Les informations sont partagées conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J301" t="inlineStr"/>
       <c r="L301" s="16" t="inlineStr">
         <is>
           <t>Informatie wordt gedeeld in overeenstemming met de responsplannen.</t>
@@ -14456,7 +14350,6 @@
           <t>La coordination avec les parties prenantes se fait conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J304" t="inlineStr"/>
       <c r="L304" s="16" t="inlineStr">
         <is>
           <t>Coördinatie met belanghebbenden vindt plaats in overeenstemming met de responsplannen.</t>
@@ -14535,7 +14428,6 @@
           <t>Le partage volontaire d'informations se fait avec des parties prenantes externes afin d'obtenir une meilleure connaissance de la situation en matière de cybersécurité.</t>
         </is>
       </c>
-      <c r="J306" t="inlineStr"/>
       <c r="L306" s="16" t="inlineStr">
         <is>
           <t>Er vindt vrijwillige informatie-uitwisseling plaats met externe belanghebbenden om een breder situationeel bewustzijn over cyberbeveiliging te bereiken.</t>
@@ -14621,7 +14513,6 @@
           <t>Une analyse est effectuée pour garantir une réponse efficace et soutenir les activités de rétablissement.</t>
         </is>
       </c>
-      <c r="J308" t="inlineStr"/>
       <c r="K308" s="11" t="inlineStr">
         <is>
           <t>Analyse</t>
@@ -14652,7 +14543,6 @@
           <t>Les notifications des systèmes de détection sont examinées.</t>
         </is>
       </c>
-      <c r="J309" t="inlineStr"/>
       <c r="L309" s="16" t="inlineStr">
         <is>
           <t>RS.AN-1:  Meldingen van detectiesystemen worden onderzocht.</t>
@@ -14778,7 +14668,6 @@
           <t>L'impact de l'incident est compris.</t>
         </is>
       </c>
-      <c r="J312" t="inlineStr"/>
       <c r="L312" s="16" t="inlineStr">
         <is>
           <t>De gevolgen van het incident worden begrepen.</t>
@@ -14907,7 +14796,6 @@
           <t>L'analyse forensique est réalisée.</t>
         </is>
       </c>
-      <c r="J315" t="inlineStr"/>
       <c r="L315" s="16" t="inlineStr">
         <is>
           <t>Forensisch onderzoek wordt uitgevoerd.</t>
@@ -15033,7 +14921,6 @@
           <t>Les incidents sont classés par catégories conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J318" t="inlineStr"/>
       <c r="L318" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden in categorieën ingedeeld overeenkomstig de responsplannen.</t>
@@ -15114,7 +15001,6 @@
           <t>Des processus sont établis pour recevoir, analyser et répondre aux vulnérabilités divulguées à l'organisation par des sources internes et externes (par exemple, tests internes, bulletins de sécurité ou chercheurs en sécurité).</t>
         </is>
       </c>
-      <c r="J320" t="inlineStr"/>
       <c r="L320" s="16" t="inlineStr">
         <is>
           <t>Er zijn processen vastgesteld voor het ontvangen, analyseren en reageren op kwetsbaarheden die uit interne en externe bronnen (bv. interne tests, beveiligingsbulletins of beveiligingsonderzoekers) aan de organisatie bekend zijn gemaakt.</t>
@@ -15250,7 +15136,6 @@
           <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
         </is>
       </c>
-      <c r="J323" t="inlineStr"/>
       <c r="K323" s="11" t="inlineStr">
         <is>
           <t>Mitigatie</t>
@@ -15281,7 +15166,6 @@
           <t>Les incidents sont contenus.</t>
         </is>
       </c>
-      <c r="J324" t="inlineStr"/>
       <c r="L324" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden beheerst.</t>
@@ -15307,74 +15191,149 @@
           <t>IMPORTANT_RS.MI-1.1</t>
         </is>
       </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>The organization shall implement an incident handling capability for information/cybersecurity incidents on its business critical systems that includes preparation, detection and analysis, containment, eradication, recovery and documented risk acceptance.</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>A documented risk acceptance deals with risks that the organisation assesses as not dangerous to the organisation's business critical systems and where the risk owner formally accepts the risk (related with the risk appetite of the organization)</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre en œuvre une capacité de traitement des incidents de sécurité de l'information/cybersécurité sur ses systèmes essentiels à l'activité, qui comprend la préparation, la détection et l'analyse, le confinement, l'éradication, le rétablissement et l'acceptation documentée des risques.</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>Une acceptation des risques documentée concerne les risques que l'organisation évalue comme non dangereux pour les systèmes critiques de l'organisation et pour lesquels le propriétaire du risque accepte formellement le risque (en relation avec l'appétit de l'organisation pour le risque).</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>De organisatie moet een capaciteit voor het afhandelen van informatie- /cyberbeveiligingsincidenten op haar bedrijfskritische systemen implementeren die de voorbereiding, detectie, analyse, insluiting (“containment”), uitroeiing, herstel en gedocumenteerde risicoaanvaarding omvat.</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>Een gedocumenteerde risicoaanvaarding heeft betrekking op risico's die volgens de organisatie niet gevaarlijk zijn voor de bedrijfskritische systemen van de organisatie en waarbij de eigenaar van het risico het risico formeel aanvaardt (gerelateerd aan de risicobereidheid, ”risk appetite”, van de organisatie).</t>
+        </is>
+      </c>
     </row>
     <row r="326">
-      <c r="B326" s="13" t="n">
+      <c r="B326" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D326" s="8" t="inlineStr">
+        <is>
+          <t>RS.IM</t>
+        </is>
+      </c>
+      <c r="E326" s="8" t="inlineStr">
+        <is>
+          <t>Improvements</t>
+        </is>
+      </c>
+      <c r="F326" s="9" t="inlineStr">
+        <is>
+          <t>Organizational response activities are improved by incorporating lessons learned from current and previous detection/response activities.</t>
+        </is>
+      </c>
+      <c r="H326" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Améliorations </t>
+        </is>
+      </c>
+      <c r="I326" s="11" t="inlineStr">
+        <is>
+          <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
+        </is>
+      </c>
+      <c r="K326" s="11" t="inlineStr">
+        <is>
+          <t>Verbeteringen</t>
+        </is>
+      </c>
+      <c r="L326" s="12" t="inlineStr">
+        <is>
+          <t>De responsactiviteiten van de organisatie worden verbeterd door lessen te trekken uit huidige en eerdere opsporings- en responsactiviteiten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="B327" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D326" s="13" t="inlineStr">
-        <is>
-          <t>RS.MI-2</t>
-        </is>
-      </c>
-      <c r="F326" s="14" t="inlineStr">
-        <is>
-          <t>Incidents are mitigated</t>
-        </is>
-      </c>
-      <c r="I326" s="15" t="inlineStr">
-        <is>
-          <t>Les incidents sont atténués.</t>
-        </is>
-      </c>
-      <c r="L326" s="16" t="inlineStr">
-        <is>
-          <t>Incidenten worden gemitigeerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B327" t="n">
-        <v>4</v>
-      </c>
-      <c r="C327" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D327" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RS.MI-2.1</t>
+      <c r="D327" s="13" t="inlineStr">
+        <is>
+          <t>RS.IM-1</t>
+        </is>
+      </c>
+      <c r="F327" s="14" t="inlineStr">
+        <is>
+          <t>Response plans incorporate lessons learned</t>
+        </is>
+      </c>
+      <c r="I327" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de réponse intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L327" s="16" t="inlineStr">
+        <is>
+          <t>In de responsplannen zijn de geleerde lessen verwerkt.</t>
         </is>
       </c>
     </row>
     <row r="328" ht="43.2" customHeight="1">
-      <c r="B328" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D328" s="13" t="inlineStr">
-        <is>
-          <t>RS.MI-3</t>
-        </is>
-      </c>
-      <c r="F328" s="14" t="inlineStr">
-        <is>
-          <t>Newly identified vulnerabilities are mitigated or documented as accepted risks</t>
-        </is>
-      </c>
-      <c r="I328" s="15" t="inlineStr">
-        <is>
-          <t>Les vulnérabilités nouvellement identifiées sont atténuées ou documentées comme des risques acceptés.</t>
-        </is>
-      </c>
-      <c r="L328" s="16" t="inlineStr">
-        <is>
-          <t>Nieuw vastgestelde kwetsbaarheden worden gemitigeerd of gedocumenteerd als aanvaarde risico's.</t>
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>4</v>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>B,I,E</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>BASIC_RS.IM-1.1</t>
+        </is>
+      </c>
+      <c r="F328" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall conduct post-incident evaluations to analyse lessons learned from incident response and recovery, and consequently improve processes / procedures / technologies to enhance its cyber resilience.</t>
+        </is>
+      </c>
+      <c r="G328" s="17" t="inlineStr">
+        <is>
+          <t>Consider bringing involved people together after each incident and reflect together on ways to improve what happened, how it happened, how we reacted, how it could have gone better, what should be done to prevent it from happening again, etc.</t>
+        </is>
+      </c>
+      <c r="I328" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit effectuer des évaluations post-incident afin d'analyser les enseignements tirés de la réponse à l'incident et du rétablissement, et par conséquent améliorer les processus / procédures / technologies pour renforcer sa cyber-résilience.</t>
+        </is>
+      </c>
+      <c r="J328" s="18" t="inlineStr">
+        <is>
+          <t>Envisagez de réunir les personnes concernées après chaque incident et réfléchissez ensemble aux moyens d'améliorer ce qui s'est passé, comment cela s'est passé, comment nous avons réagi, comment cela aurait pu mieux se passer, ce qui devrait être fait pour éviter que cela ne se reproduise, etc.</t>
+        </is>
+      </c>
+      <c r="L328" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet evaluaties uitvoeren na een incident om lessen te trekken uit de reactie op en het herstel van incidenten, en verbetert vervolgens de processen / procedures / technologieën om haar cyberweerbaarheid te vergroten.</t>
+        </is>
+      </c>
+      <c r="M328" s="18" t="inlineStr">
+        <is>
+          <t>Overweeg na elk incident de betrokkenen samen te brengen en samen na te denken over manieren om te verbeteren wat er is gebeurd, hoe het is gebeurd, hoe er is gereageerd, hoe het beter had kunnen gaan, wat er moet gebeuren om herhaling te voorkomen, enz.</t>
         </is>
       </c>
     </row>
@@ -15394,204 +15353,177 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>IMPORTANT_RS.MI-3.1</t>
+          <t>IMPORTANT_RS.IM-1.2</t>
         </is>
       </c>
       <c r="F329" s="17" t="inlineStr">
         <is>
-          <t>The organization shall implement an incident handling capability for information/cybersecurity incidents on its business critical systems that includes preparation, detection and analysis, containment, eradication, recovery and documented risk acceptance.</t>
+          <t>Lessons learned from incident handling shall be translated into updated or new incident handling procedures that shall be tested, approved and trained.</t>
         </is>
       </c>
       <c r="G329" s="17" t="inlineStr">
         <is>
-          <t>A documented risk acceptance deals with risks that the organisation assesses as not dangerous to the organisation's business critical systems and where the risk owner formally accepts the risk (related with the risk appetite of the organization)</t>
+          <t>No additional guidance on this topic.</t>
         </is>
       </c>
       <c r="I329" s="18" t="inlineStr">
         <is>
-          <t>L'organisation doit mettre en œuvre une capacité de traitement des incidents de sécurité de l'information/cybersécurité sur ses systèmes essentiels à l'activité, qui comprend la préparation, la détection et l'analyse, le confinement, l'éradication, le rétablissement et l'acceptation documentée des risques.</t>
+          <t>Les enseignements tirés du traitement des incidents sont traduits en procédures de traitement des incidents actualisées ou nouvelles qui sont testées, approuvées et enseignées.</t>
         </is>
       </c>
       <c r="J329" s="18" t="inlineStr">
         <is>
-          <t>Une acceptation des risques documentée concerne les risques que l'organisation évalue comme non dangereux pour les systèmes critiques de l'organisation et pour lesquels le propriétaire du risque accepte formellement le risque (en relation avec l'appétit de l'organisation pour le risque).</t>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
         </is>
       </c>
       <c r="L329" s="18" t="inlineStr">
         <is>
-          <t>De organisatie moet een capaciteit voor het afhandelen van informatie- /cyberbeveiligingsincidenten op haar bedrijfskritische systemen implementeren die de voorbereiding, detectie, analyse, insluiting (“containment”), uitroeiing, herstel en gedocumenteerde risicoaanvaarding omvat.</t>
+          <t>De uit de afhandeling van incidenten geleerde lessen moeten worden vertaald in bijgewerkte of nieuwe procedures voor de afhandeling van incidenten, die op hun beurt moeten worden getest, goedgekeurd en getraind.</t>
         </is>
       </c>
       <c r="M329" s="18" t="inlineStr">
         <is>
-          <t>Een gedocumenteerde risicoaanvaarding heeft betrekking op risico's die volgens de organisatie niet gevaarlijk zijn voor de bedrijfskritische systemen van de organisatie en waarbij de eigenaar van het risico het risico formeel aanvaardt (gerelateerd aan de risicobereidheid, ”risk appetite”, van de organisatie).</t>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
         </is>
       </c>
     </row>
     <row r="330" ht="57.6" customHeight="1">
-      <c r="B330" s="8" t="n">
+      <c r="B330" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D330" s="13" t="inlineStr">
+        <is>
+          <t>RS.IM-2</t>
+        </is>
+      </c>
+      <c r="F330" s="14" t="inlineStr">
+        <is>
+          <t>Response and Recovery strategies are updated</t>
+        </is>
+      </c>
+      <c r="I330" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de réponse intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L330" s="16" t="inlineStr">
+        <is>
+          <t>Reactie- en herstelstrategieën worden bijgewerkt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>4</v>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RS.IM-2.1</t>
+        </is>
+      </c>
+      <c r="F331" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall update the response and recovery  plans to address changes in its context.</t>
+        </is>
+      </c>
+      <c r="G331" s="17" t="inlineStr">
+        <is>
+          <t>The organization’s context relates to the organizational structure, its critical systems, attack vectors, new threats, improved technology, environment of operation, problems encountered during plan implementation/execution/testing and lessons learned.</t>
+        </is>
+      </c>
+      <c r="I331" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre à jour les plans de réponse et de rétablissement pour tenir compte des changements survenus dans son contexte.</t>
+        </is>
+      </c>
+      <c r="J331" s="18" t="inlineStr">
+        <is>
+          <t>Le contexte de l'organisation concerne la structure organisationnelle, ses systèmes critiques, les vecteurs d'attaque, les nouvelles menaces, les améliorations technologiques, l'environnement d'exploitation, les problèmes rencontrés lors de la mise en œuvre/exécution/test du plan et les enseignements tirés.</t>
+        </is>
+      </c>
+      <c r="L331" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de reactie- en herstelplannen aanpassen aan veranderingen in haar context.</t>
+        </is>
+      </c>
+      <c r="M331" s="18" t="inlineStr">
+        <is>
+          <t>De context van de organisatie heeft betrekking op de organisatiestructuur, haar kritieke systemen, aanvalsvectoren, nieuwe bedreigingen, verbeterde technologie, de bedrijfsomgeving, problemen die zich hebben voorgedaan tijdens de implementatie/uitvoering/testen van het plan en de lessen die zijn geleerd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="86.40000000000001" customHeight="1">
+      <c r="B332" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D332" s="5" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="E332" s="5" t="inlineStr">
+        <is>
+          <t>RECOVER (RC)</t>
+        </is>
+      </c>
+      <c r="H332" s="5" t="inlineStr">
+        <is>
+          <t>RETABLIR (RC)</t>
+        </is>
+      </c>
+      <c r="K332" s="7" t="inlineStr">
+        <is>
+          <t>HERSTELLEN (RC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="57.6" customHeight="1">
+      <c r="B333" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D330" s="8" t="inlineStr">
-        <is>
-          <t>RS.IM</t>
-        </is>
-      </c>
-      <c r="E330" s="8" t="inlineStr">
-        <is>
-          <t>Improvements</t>
-        </is>
-      </c>
-      <c r="F330" s="9" t="inlineStr">
-        <is>
-          <t>Organizational response activities are improved by incorporating lessons learned from current and previous detection/response activities.</t>
-        </is>
-      </c>
-      <c r="H330" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Améliorations </t>
-        </is>
-      </c>
-      <c r="I330" s="11" t="inlineStr">
-        <is>
-          <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
-        </is>
-      </c>
-      <c r="J330" t="inlineStr"/>
-      <c r="K330" s="11" t="inlineStr">
-        <is>
-          <t>Verbeteringen</t>
-        </is>
-      </c>
-      <c r="L330" s="12" t="inlineStr">
-        <is>
-          <t>De responsactiviteiten van de organisatie worden verbeterd door lessen te trekken uit huidige en eerdere opsporings- en responsactiviteiten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="331">
-      <c r="B331" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D331" s="13" t="inlineStr">
-        <is>
-          <t>RS.IM-1</t>
-        </is>
-      </c>
-      <c r="F331" s="14" t="inlineStr">
-        <is>
-          <t>Response plans incorporate lessons learned</t>
-        </is>
-      </c>
-      <c r="I331" s="15" t="inlineStr">
-        <is>
-          <t>Les plans de réponse intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J331" t="inlineStr"/>
-      <c r="L331" s="16" t="inlineStr">
-        <is>
-          <t>In de responsplannen zijn de geleerde lessen verwerkt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="332" ht="86.40000000000001" customHeight="1">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B332" t="n">
-        <v>4</v>
-      </c>
-      <c r="C332" t="inlineStr">
-        <is>
-          <t>B,I,E</t>
-        </is>
-      </c>
-      <c r="D332" t="inlineStr">
-        <is>
-          <t>BASIC_RS.IM-1.1</t>
-        </is>
-      </c>
-      <c r="F332" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall conduct post-incident evaluations to analyse lessons learned from incident response and recovery, and consequently improve processes / procedures / technologies to enhance its cyber resilience.</t>
-        </is>
-      </c>
-      <c r="G332" s="17" t="inlineStr">
-        <is>
-          <t>Consider bringing involved people together after each incident and reflect together on ways to improve what happened, how it happened, how we reacted, how it could have gone better, what should be done to prevent it from happening again, etc.</t>
-        </is>
-      </c>
-      <c r="I332" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit effectuer des évaluations post-incident afin d'analyser les enseignements tirés de la réponse à l'incident et du rétablissement, et par conséquent améliorer les processus / procédures / technologies pour renforcer sa cyber-résilience.</t>
-        </is>
-      </c>
-      <c r="J332" s="18" t="inlineStr">
-        <is>
-          <t>Envisagez de réunir les personnes concernées après chaque incident et réfléchissez ensemble aux moyens d'améliorer ce qui s'est passé, comment cela s'est passé, comment nous avons réagi, comment cela aurait pu mieux se passer, ce qui devrait être fait pour éviter que cela ne se reproduise, etc.</t>
-        </is>
-      </c>
-      <c r="L332" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet evaluaties uitvoeren na een incident om lessen te trekken uit de reactie op en het herstel van incidenten, en verbetert vervolgens de processen / procedures / technologieën om haar cyberweerbaarheid te vergroten.</t>
-        </is>
-      </c>
-      <c r="M332" s="18" t="inlineStr">
-        <is>
-          <t>Overweeg na elk incident de betrokkenen samen te brengen en samen na te denken over manieren om te verbeteren wat er is gebeurd, hoe het is gebeurd, hoe er is gereageerd, hoe het beter had kunnen gaan, wat er moet gebeuren om herhaling te voorkomen, enz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="333" ht="57.6" customHeight="1">
-      <c r="A333" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B333" t="n">
-        <v>4</v>
-      </c>
-      <c r="C333" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D333" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RS.IM-1.2</t>
-        </is>
-      </c>
-      <c r="F333" s="17" t="inlineStr">
-        <is>
-          <t>Lessons learned from incident handling shall be translated into updated or new incident handling procedures that shall be tested, approved and trained.</t>
-        </is>
-      </c>
-      <c r="G333" s="17" t="inlineStr">
-        <is>
-          <t>No additional guidance on this topic.</t>
-        </is>
-      </c>
-      <c r="I333" s="18" t="inlineStr">
-        <is>
-          <t>Les enseignements tirés du traitement des incidents sont traduits en procédures de traitement des incidents actualisées ou nouvelles qui sont testées, approuvées et enseignées.</t>
-        </is>
-      </c>
-      <c r="J333" s="18" t="inlineStr">
-        <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
-        </is>
-      </c>
-      <c r="L333" s="18" t="inlineStr">
-        <is>
-          <t>De uit de afhandeling van incidenten geleerde lessen moeten worden vertaald in bijgewerkte of nieuwe procedures voor de afhandeling van incidenten, die op hun beurt moeten worden getest, goedgekeurd en getraind.</t>
-        </is>
-      </c>
-      <c r="M333" s="18" t="inlineStr">
-        <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+      <c r="D333" s="8" t="inlineStr">
+        <is>
+          <t>RC.RP</t>
+        </is>
+      </c>
+      <c r="E333" s="8" t="inlineStr">
+        <is>
+          <t>Recovery Planning</t>
+        </is>
+      </c>
+      <c r="F333" s="9" t="inlineStr">
+        <is>
+          <t>Recovery processes and procedures are executed and maintained to ensure restoration of systems or assets affected by cybersecurity incidents.</t>
+        </is>
+      </c>
+      <c r="H333" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planification du rétablissement </t>
+        </is>
+      </c>
+      <c r="I333" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K333" s="11" t="inlineStr">
+        <is>
+          <t>Herstelplanning</t>
+        </is>
+      </c>
+      <c r="L333" s="12" t="inlineStr">
+        <is>
+          <t>Herstelprocessen en -procedures worden uitgevoerd en gehandhaafd om te zorgen voor herstel van systemen of activa die zijn getroffen door cyberbeveiligingsincidenten.</t>
         </is>
       </c>
     </row>
@@ -15601,23 +15533,22 @@
       </c>
       <c r="D334" s="13" t="inlineStr">
         <is>
-          <t>RS.IM-2</t>
+          <t>RC.RP-1</t>
         </is>
       </c>
       <c r="F334" s="14" t="inlineStr">
         <is>
-          <t>Response and Recovery strategies are updated</t>
+          <t xml:space="preserve">Recovery plan is executed during or after a cybersecurity incident </t>
         </is>
       </c>
       <c r="I334" s="15" t="inlineStr">
         <is>
-          <t>Les plans de réponse intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J334" t="inlineStr"/>
+          <t xml:space="preserve"> Le plan de reprise est exécuté pendant ou après un incident de cybersécurité.</t>
+        </is>
+      </c>
       <c r="L334" s="16" t="inlineStr">
         <is>
-          <t>Reactie- en herstelstrategieën worden bijgewerkt.</t>
+          <t>Het herstelplan wordt uitgevoerd tijdens of na een cyberbeveiligingsincident.</t>
         </is>
       </c>
     </row>
@@ -15632,164 +15563,20 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>I,E</t>
+          <t>B,I,E</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>IMPORTANT_RS.IM-2.1</t>
+          <t>BASIC_RC.RP-1.1</t>
         </is>
       </c>
       <c r="F335" s="17" t="inlineStr">
         <is>
-          <t>The organization shall update the response and recovery  plans to address changes in its context.</t>
+          <t>A recovery process for disasters and information/cybersecurity incidents shall be developed and executed as appropriate.</t>
         </is>
       </c>
       <c r="G335" s="17" t="inlineStr">
-        <is>
-          <t>The organization’s context relates to the organizational structure, its critical systems, attack vectors, new threats, improved technology, environment of operation, problems encountered during plan implementation/execution/testing and lessons learned.</t>
-        </is>
-      </c>
-      <c r="I335" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit mettre à jour les plans de réponse et de rétablissement pour tenir compte des changements survenus dans son contexte.</t>
-        </is>
-      </c>
-      <c r="J335" s="18" t="inlineStr">
-        <is>
-          <t>Le contexte de l'organisation concerne la structure organisationnelle, ses systèmes critiques, les vecteurs d'attaque, les nouvelles menaces, les améliorations technologiques, l'environnement d'exploitation, les problèmes rencontrés lors de la mise en œuvre/exécution/test du plan et les enseignements tirés.</t>
-        </is>
-      </c>
-      <c r="L335" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de reactie- en herstelplannen aanpassen aan veranderingen in haar context.</t>
-        </is>
-      </c>
-      <c r="M335" s="18" t="inlineStr">
-        <is>
-          <t>De context van de organisatie heeft betrekking op de organisatiestructuur, haar kritieke systemen, aanvalsvectoren, nieuwe bedreigingen, verbeterde technologie, de bedrijfsomgeving, problemen die zich hebben voorgedaan tijdens de implementatie/uitvoering/testen van het plan en de lessen die zijn geleerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="B336" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D336" s="5" t="inlineStr">
-        <is>
-          <t>RC</t>
-        </is>
-      </c>
-      <c r="E336" s="5" t="inlineStr">
-        <is>
-          <t>RECOVER (RC)</t>
-        </is>
-      </c>
-      <c r="H336" s="5" t="inlineStr">
-        <is>
-          <t>RETABLIR (RC)</t>
-        </is>
-      </c>
-      <c r="I336" t="inlineStr"/>
-      <c r="J336" t="inlineStr"/>
-      <c r="K336" s="7" t="inlineStr">
-        <is>
-          <t>HERSTELLEN (RC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="337" ht="57.6" customHeight="1">
-      <c r="B337" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D337" s="8" t="inlineStr">
-        <is>
-          <t>RC.RP</t>
-        </is>
-      </c>
-      <c r="E337" s="8" t="inlineStr">
-        <is>
-          <t>Recovery Planning</t>
-        </is>
-      </c>
-      <c r="F337" s="9" t="inlineStr">
-        <is>
-          <t>Recovery processes and procedures are executed and maintained to ensure restoration of systems or assets affected by cybersecurity incidents.</t>
-        </is>
-      </c>
-      <c r="H337" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Planification du rétablissement </t>
-        </is>
-      </c>
-      <c r="I337" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J337" t="inlineStr"/>
-      <c r="K337" s="11" t="inlineStr">
-        <is>
-          <t>Herstelplanning</t>
-        </is>
-      </c>
-      <c r="L337" s="12" t="inlineStr">
-        <is>
-          <t>Herstelprocessen en -procedures worden uitgevoerd en gehandhaafd om te zorgen voor herstel van systemen of activa die zijn getroffen door cyberbeveiligingsincidenten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="338" ht="28.8" customHeight="1">
-      <c r="B338" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D338" s="13" t="inlineStr">
-        <is>
-          <t>RC.RP-1</t>
-        </is>
-      </c>
-      <c r="F338" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recovery plan is executed during or after a cybersecurity incident </t>
-        </is>
-      </c>
-      <c r="I338" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Le plan de reprise est exécuté pendant ou après un incident de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J338" t="inlineStr"/>
-      <c r="L338" s="16" t="inlineStr">
-        <is>
-          <t>Het herstelplan wordt uitgevoerd tijdens of na een cyberbeveiligingsincident.</t>
-        </is>
-      </c>
-    </row>
-    <row r="339" ht="244.8" customHeight="1">
-      <c r="A339" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B339" t="n">
-        <v>4</v>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>B,I,E</t>
-        </is>
-      </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>BASIC_RC.RP-1.1</t>
-        </is>
-      </c>
-      <c r="F339" s="17" t="inlineStr">
-        <is>
-          <t>A recovery process for disasters and information/cybersecurity incidents shall be developed and executed as appropriate.</t>
-        </is>
-      </c>
-      <c r="G339" s="17" t="inlineStr">
         <is>
           <t>A process should be developed for what immediate actions will be taken in case of a fire, medical emergency, burglary, natural disaster, or  an information/cyber security incident.
 This process should consider:
@@ -15798,12 +15585,12 @@
 •	Who to call in case of an incident.</t>
         </is>
       </c>
-      <c r="I339" s="18" t="inlineStr">
+      <c r="I335" s="18" t="inlineStr">
         <is>
           <t>Un processus de rétablissement en cas de catastrophes et d'incidents liés à l'information et à la cybersécurité est élaboré et exécuté selon les besoins.</t>
         </is>
       </c>
-      <c r="J339" s="18" t="inlineStr">
+      <c r="J335" s="18" t="inlineStr">
         <is>
           <t>• Il convient qu’un processus soit élaboré pour déterminer les mesures immédiates à prendre en cas d'incendie, d'urgence médicale, de cambriolage, de catastrophe naturelle ou d'incident de sécurité informatique.
 • Il convient que ce processus prenne en compte : 
@@ -15812,12 +15599,12 @@
 	o Qui appeler en cas d'incident.</t>
         </is>
       </c>
-      <c r="L339" s="18" t="inlineStr">
+      <c r="L335" s="18" t="inlineStr">
         <is>
           <t>Er moet een herstelproces voor rampen en informatie-/cyberbeveiligingsincidenten worden ontwikkeld en zo nodig uitgevoerd.+L339</t>
         </is>
       </c>
-      <c r="M339" s="18" t="inlineStr">
+      <c r="M335" s="18" t="inlineStr">
         <is>
           <t>• Er zou een proces moeten worden ontwikkeld voor de onmiddellijke acties in geval van brand, medisch noodgeval, inbraak, natuurramp of een incident op het gebied van informatie-/cyberbeveiliging. 
 • Dit proces zou rekening moeten houden met: 
@@ -15827,120 +15614,283 @@
         </is>
       </c>
     </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>4</v>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>RC.RP-1.2</t>
+        </is>
+      </c>
+      <c r="F336" s="17" t="inlineStr">
+        <is>
+          <t>The essential organization’s functions and services shall be continued with little or no loss of operational continuity and continuity shall be sustained until full system restoration.</t>
+        </is>
+      </c>
+      <c r="G336" s="17" t="inlineStr">
+        <is>
+          <t>No additional guidance on this topic.</t>
+        </is>
+      </c>
+      <c r="I336" s="18" t="inlineStr">
+        <is>
+          <t>Les fonctions et services de l'organisation essentielle doivent être poursuivis avec peu ou pas de perte de continuité opérationnelle et la continuité doit être maintenue jusqu'à la restauration complète du système.</t>
+        </is>
+      </c>
+      <c r="J336" s="18" t="inlineStr">
+        <is>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+        </is>
+      </c>
+      <c r="L336" s="18" t="inlineStr">
+        <is>
+          <t>De essentiële functies en diensten van de organisatie moeten worden voortgezet met weinig of geen verlies van operationele continuïteit en de continuïteit moet worden gehandhaafd totdat het systeem volledig is hersteld.</t>
+        </is>
+      </c>
+      <c r="M336" s="18" t="inlineStr">
+        <is>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="57.6" customHeight="1">
+      <c r="B337" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D337" s="8" t="inlineStr">
+        <is>
+          <t>RC.IM</t>
+        </is>
+      </c>
+      <c r="E337" s="8" t="inlineStr">
+        <is>
+          <t>Improvements</t>
+        </is>
+      </c>
+      <c r="F337" s="9" t="inlineStr">
+        <is>
+          <t>Recovery planning and processes are improved by incorporating lessons learned into future activities.</t>
+        </is>
+      </c>
+      <c r="H337" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Améliorations </t>
+        </is>
+      </c>
+      <c r="I337" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K337" s="11" t="inlineStr">
+        <is>
+          <t>Verbeteringen</t>
+        </is>
+      </c>
+      <c r="L337" s="12" t="inlineStr">
+        <is>
+          <t>De herstelplanning en -processen worden verbeterd door in toekomstige activiteiten rekening te houden met de opgedane ervaring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="28.8" customHeight="1">
+      <c r="B338" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D338" s="13" t="inlineStr">
+        <is>
+          <t>RC.IM-1</t>
+        </is>
+      </c>
+      <c r="F338" s="14" t="inlineStr">
+        <is>
+          <t>Recovery plans incorporate lessons learned</t>
+        </is>
+      </c>
+      <c r="I338" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de rétablissement intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L338" s="16" t="inlineStr">
+        <is>
+          <t>In de herstelplannen zijn de geleerde lessen verwerkt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="244.8" customHeight="1">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>4</v>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RC.IM-1.1</t>
+        </is>
+      </c>
+      <c r="F339" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall incorporate lessons learned from incident recovery activities into updated or new system recovery procedures and, after testing, frame this with appropriate training.</t>
+        </is>
+      </c>
+      <c r="G339" s="17" t="inlineStr">
+        <is>
+          <t>No additional guidance on this topic.</t>
+        </is>
+      </c>
+      <c r="I339" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit intégrer les enseignements tirés des activités de rétablissement des incidents dans les procédures de rétablissement du système, nouvelles ou mises à jour, et, après les avoir testées, les encadrer par une formation appropriée.</t>
+        </is>
+      </c>
+      <c r="J339" s="18" t="inlineStr">
+        <is>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+        </is>
+      </c>
+      <c r="L339" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de lessen die zijn getrokken uit herstelactiviteiten bij incidenten verwerken in bijgewerkte of nieuwe herstelprocedures voor systemen en dit, na het testen, borgen met een passende opleiding.</t>
+        </is>
+      </c>
+      <c r="M339" s="18" t="inlineStr">
+        <is>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
+        </is>
+      </c>
+    </row>
     <row r="340" ht="72" customHeight="1">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B340" t="n">
-        <v>4</v>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>RC.RP-1.2</t>
-        </is>
-      </c>
-      <c r="F340" s="17" t="inlineStr">
-        <is>
-          <t>The essential organization’s functions and services shall be continued with little or no loss of operational continuity and continuity shall be sustained until full system restoration.</t>
-        </is>
-      </c>
-      <c r="G340" s="17" t="inlineStr">
-        <is>
-          <t>No additional guidance on this topic.</t>
-        </is>
-      </c>
-      <c r="I340" s="18" t="inlineStr">
-        <is>
-          <t>Les fonctions et services de l'organisation essentielle doivent être poursuivis avec peu ou pas de perte de continuité opérationnelle et la continuité doit être maintenue jusqu'à la restauration complète du système.</t>
-        </is>
-      </c>
-      <c r="J340" s="18" t="inlineStr">
-        <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
-        </is>
-      </c>
-      <c r="L340" s="18" t="inlineStr">
-        <is>
-          <t>De essentiële functies en diensten van de organisatie moeten worden voortgezet met weinig of geen verlies van operationele continuïteit en de continuïteit moet worden gehandhaafd totdat het systeem volledig is hersteld.</t>
-        </is>
-      </c>
-      <c r="M340" s="18" t="inlineStr">
-        <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+      <c r="B340" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D340" s="8" t="inlineStr">
+        <is>
+          <t>RC.CO</t>
+        </is>
+      </c>
+      <c r="E340" s="8" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="F340" s="9" t="inlineStr">
+        <is>
+          <t>Restoration activities are coordinated with internal and external parties (e.g.  coordinating centers, Internet Service Providers, owners of attacking systems, victims, other CSIRTs, and vendors).</t>
+        </is>
+      </c>
+      <c r="H340" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Communications </t>
+        </is>
+      </c>
+      <c r="I340" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K340" s="11" t="inlineStr">
+        <is>
+          <t>Communicatie</t>
+        </is>
+      </c>
+      <c r="L340" s="12" t="inlineStr">
+        <is>
+          <t>Herstelactiviteiten worden gecoördineerd met interne en externe partijen (bv. coördinatiecentra, internetproviders, eigenaars van aanvallende systemen, slachtoffers, andere CSIRT's en verkopers).</t>
         </is>
       </c>
     </row>
     <row r="341" ht="57.6" customHeight="1">
-      <c r="B341" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D341" s="8" t="inlineStr">
-        <is>
-          <t>RC.IM</t>
-        </is>
-      </c>
-      <c r="E341" s="8" t="inlineStr">
-        <is>
-          <t>Improvements</t>
-        </is>
-      </c>
-      <c r="F341" s="9" t="inlineStr">
-        <is>
-          <t>Recovery planning and processes are improved by incorporating lessons learned into future activities.</t>
-        </is>
-      </c>
-      <c r="H341" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Améliorations </t>
-        </is>
-      </c>
-      <c r="I341" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J341" t="inlineStr"/>
-      <c r="K341" s="11" t="inlineStr">
-        <is>
-          <t>Verbeteringen</t>
-        </is>
-      </c>
-      <c r="L341" s="12" t="inlineStr">
-        <is>
-          <t>De herstelplanning en -processen worden verbeterd door in toekomstige activiteiten rekening te houden met de opgedane ervaring.</t>
+      <c r="B341" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D341" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-1</t>
+        </is>
+      </c>
+      <c r="F341" s="14" t="inlineStr">
+        <is>
+          <t>Public relations are managed</t>
+        </is>
+      </c>
+      <c r="I341" s="15" t="inlineStr">
+        <is>
+          <t>Les relations publiques sont gérées.</t>
+        </is>
+      </c>
+      <c r="L341" s="16" t="inlineStr">
+        <is>
+          <t>De public relations worden beheerd.</t>
         </is>
       </c>
     </row>
     <row r="342" ht="28.8" customHeight="1">
-      <c r="B342" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D342" s="13" t="inlineStr">
-        <is>
-          <t>RC.IM-1</t>
-        </is>
-      </c>
-      <c r="F342" s="14" t="inlineStr">
-        <is>
-          <t>Recovery plans incorporate lessons learned</t>
-        </is>
-      </c>
-      <c r="I342" s="15" t="inlineStr">
-        <is>
-          <t>Les plans de rétablissement intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J342" t="inlineStr"/>
-      <c r="L342" s="16" t="inlineStr">
-        <is>
-          <t>In de herstelplannen zijn de geleerde lessen verwerkt.</t>
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B342" t="n">
+        <v>4</v>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RC.CO-1.1</t>
+        </is>
+      </c>
+      <c r="F342" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall centralize and coordinate how information is disseminated and manage how the organization is presented to the public.</t>
+        </is>
+      </c>
+      <c r="G342" s="17" t="inlineStr">
+        <is>
+          <t>Public relations management may include, for example, managing media interactions, coordinating and logging all requests for interviews, handling and ‘triaging’ phone calls and e-mail requests, matching media requests with appropriate and available internal experts who are ready to be interviewed, screening all of information provided to the media, ensuring personnel are familiar with public relations and privacy policies.</t>
+        </is>
+      </c>
+      <c r="I342" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit centraliser et coordonner la manière dont les informations sont diffusées et gérer la manière dont l'organisation est présentée au public.</t>
+        </is>
+      </c>
+      <c r="J342" s="18" t="inlineStr">
+        <is>
+          <t>La gestion des relations publiques peut comprendre, par exemple, la gestion des interactions avec les médias, la coordination et l'enregistrement de toutes les demandes d'interviews, le traitement et le triage des appels téléphoniques et des demandes par e-mail, la mise en relation des demandes des médias avec les experts internes appropriés et disponibles qui sont prêts à être interviewés, le filtrage de toutes les informations fournies aux médias, l'assurance que le personnel connaît bien les politiques en matière de relations publiques et de confidentialité.</t>
+        </is>
+      </c>
+      <c r="L342" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
+        </is>
+      </c>
+      <c r="M342" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
         </is>
       </c>
     </row>
@@ -15955,159 +15905,143 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>I,E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>IMPORTANT_RC.IM-1.1</t>
+          <t>RC.CO-1.2</t>
         </is>
       </c>
       <c r="F343" s="17" t="inlineStr">
         <is>
-          <t>The organization shall incorporate lessons learned from incident recovery activities into updated or new system recovery procedures and, after testing, frame this with appropriate training.</t>
+          <t>A Public Relations Officer shall be assigned.</t>
         </is>
       </c>
       <c r="G343" s="17" t="inlineStr">
         <is>
-          <t>No additional guidance on this topic.</t>
+          <t>The Public Relations Officer should consider the use of pre-define external contacts 
+(e.g. press, regulators, interest groups).</t>
         </is>
       </c>
       <c r="I343" s="18" t="inlineStr">
         <is>
-          <t>L'organisation doit intégrer les enseignements tirés des activités de rétablissement des incidents dans les procédures de rétablissement du système, nouvelles ou mises à jour, et, après les avoir testées, les encadrer par une formation appropriée.</t>
+          <t>Un responsable des relations publiques est désigné.</t>
         </is>
       </c>
       <c r="J343" s="18" t="inlineStr">
         <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+          <t>Il convient que le responsable des relations publiques envisage l'utilisation de contacts externes prédéfinis (par exemple, la presse, les régulateurs, les groupes d'intérêt).</t>
         </is>
       </c>
       <c r="L343" s="18" t="inlineStr">
         <is>
-          <t>De organisatie moet de lessen die zijn getrokken uit herstelactiviteiten bij incidenten verwerken in bijgewerkte of nieuwe herstelprocedures voor systemen en dit, na het testen, borgen met een passende opleiding.</t>
+          <t>Er moet een Public Relations Officer worden aangesteld.</t>
         </is>
       </c>
       <c r="M343" s="18" t="inlineStr">
         <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+          <t>De Public Relations Officer zou moeten overwegen gebruik te maken van vooraf bepaalde externe contacten (bijv. pers, regelgevers, belangengroepen).</t>
         </is>
       </c>
     </row>
     <row r="344" ht="57.6" customHeight="1">
-      <c r="B344" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D344" s="8" t="inlineStr">
-        <is>
-          <t>RC.CO</t>
-        </is>
-      </c>
-      <c r="E344" s="8" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="F344" s="9" t="inlineStr">
-        <is>
-          <t>Restoration activities are coordinated with internal and external parties (e.g.  coordinating centers, Internet Service Providers, owners of attacking systems, victims, other CSIRTs, and vendors).</t>
-        </is>
-      </c>
-      <c r="H344" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Communications </t>
-        </is>
-      </c>
-      <c r="I344" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J344" t="inlineStr"/>
-      <c r="K344" s="11" t="inlineStr">
-        <is>
-          <t>Communicatie</t>
-        </is>
-      </c>
-      <c r="L344" s="12" t="inlineStr">
-        <is>
-          <t>Herstelactiviteiten worden gecoördineerd met interne en externe partijen (bv. coördinatiecentra, internetproviders, eigenaars van aanvallende systemen, slachtoffers, andere CSIRT's en verkopers).</t>
+      <c r="B344" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D344" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-2</t>
+        </is>
+      </c>
+      <c r="F344" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reputation is repaired after an incident </t>
+        </is>
+      </c>
+      <c r="I344" s="15" t="inlineStr">
+        <is>
+          <t>La réputation est réparée après un incident.</t>
+        </is>
+      </c>
+      <c r="L344" s="16" t="inlineStr">
+        <is>
+          <t>Reputatie wordt hersteld na een incident.</t>
         </is>
       </c>
     </row>
     <row r="345">
-      <c r="B345" s="13" t="n">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>4</v>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>RC.CO-2.1</t>
+        </is>
+      </c>
+      <c r="F345" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall implement a crisis response strategy to protect the organization from the negative consequences of a crisis and help restore its reputation.</t>
+        </is>
+      </c>
+      <c r="G345" s="17" t="inlineStr">
+        <is>
+          <t>Crisis response strategies include, for example, actions to shape attributions of the crisis, change perceptions of the organization in crisis, and reduce the negative effect generated by the crisis.</t>
+        </is>
+      </c>
+      <c r="I345" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre en œuvre une stratégie de réponse aux crises afin de protéger l'organisation des conséquences négatives d'une crise et de contribuer à restaurer sa réputation.</t>
+        </is>
+      </c>
+      <c r="J345" s="18" t="inlineStr">
+        <is>
+          <t>Les stratégies de réponse aux crises comprennent, par exemple, des actions visant à déterminer les attributions de la crise, à modifier les perceptions de l'organisation en crise et à réduire l'effet négatif généré par la crise.</t>
+        </is>
+      </c>
+      <c r="L345" s="18" t="inlineStr">
+        <is>
+          <t>Er moet een crisisbestrijdingsstrategie worden toegepast om de organisatie te beschermen tegen de negatieve gevolgen van een crisis en te helpen haar reputatie te herstellen.</t>
+        </is>
+      </c>
+      <c r="M345" s="18" t="inlineStr">
+        <is>
+          <t>Crisisbestrijdingsstrategieën omvatten bijvoorbeeld maatregelen om de beeldvorming over de crisis vorm te geven, de perceptie van de organisatie in crisis te veranderen, en het negatieve effect dat de crisis teweegbrengt te verminderen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="158.4" customHeight="1">
+      <c r="B346" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D345" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-1</t>
-        </is>
-      </c>
-      <c r="F345" s="14" t="inlineStr">
-        <is>
-          <t>Public relations are managed</t>
-        </is>
-      </c>
-      <c r="I345" s="15" t="inlineStr">
-        <is>
-          <t>Les relations publiques sont gérées.</t>
-        </is>
-      </c>
-      <c r="J345" t="inlineStr"/>
-      <c r="L345" s="16" t="inlineStr">
-        <is>
-          <t>De public relations worden beheerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="346" ht="158.4" customHeight="1">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B346" t="n">
-        <v>4</v>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RC.CO-1.1</t>
-        </is>
-      </c>
-      <c r="F346" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall centralize and coordinate how information is disseminated and manage how the organization is presented to the public.</t>
-        </is>
-      </c>
-      <c r="G346" s="17" t="inlineStr">
-        <is>
-          <t>Public relations management may include, for example, managing media interactions, coordinating and logging all requests for interviews, handling and ‘triaging’ phone calls and e-mail requests, matching media requests with appropriate and available internal experts who are ready to be interviewed, screening all of information provided to the media, ensuring personnel are familiar with public relations and privacy policies.</t>
-        </is>
-      </c>
-      <c r="I346" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit centraliser et coordonner la manière dont les informations sont diffusées et gérer la manière dont l'organisation est présentée au public.</t>
-        </is>
-      </c>
-      <c r="J346" s="18" t="inlineStr">
-        <is>
-          <t>La gestion des relations publiques peut comprendre, par exemple, la gestion des interactions avec les médias, la coordination et l'enregistrement de toutes les demandes d'interviews, le traitement et le triage des appels téléphoniques et des demandes par e-mail, la mise en relation des demandes des médias avec les experts internes appropriés et disponibles qui sont prêts à être interviewés, le filtrage de toutes les informations fournies aux médias, l'assurance que le personnel connaît bien les politiques en matière de relations publiques et de confidentialité.</t>
-        </is>
-      </c>
-      <c r="L346" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
-        </is>
-      </c>
-      <c r="M346" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
+      <c r="D346" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-3</t>
+        </is>
+      </c>
+      <c r="F346" s="14" t="inlineStr">
+        <is>
+          <t>Recovery activities are communicated to internal and external stakeholders as well as executive and management teams</t>
+        </is>
+      </c>
+      <c r="I346" s="15" t="inlineStr">
+        <is>
+          <t>Les activités de rétablissement sont communiquées aux parties prenantes internes et externes, ainsi qu'aux équipes de direction et de gestion.</t>
+        </is>
+      </c>
+      <c r="L346" s="16" t="inlineStr">
+        <is>
+          <t>De herstelactiviteiten worden gecommuniceerd aan interne en externe belanghebbenden en aan directie- en managementteams.</t>
         </is>
       </c>
     </row>
@@ -16122,198 +16056,48 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>I,E</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>RC.CO-1.2</t>
+          <t>IMPORTANT_RC.CO-3.1</t>
         </is>
       </c>
       <c r="F347" s="17" t="inlineStr">
         <is>
-          <t>A Public Relations Officer shall be assigned.</t>
+          <t>The organization shall communicate recovery activities to predefined stakeholders, executive and management teams.</t>
         </is>
       </c>
       <c r="G347" s="17" t="inlineStr">
         <is>
-          <t>The Public Relations Officer should consider the use of pre-define external contacts 
-(e.g. press, regulators, interest groups).</t>
+          <t>Communication of recovery activities to all relevant stakeholders applies only to entities subject to the NIS legislation.</t>
         </is>
       </c>
       <c r="I347" s="18" t="inlineStr">
         <is>
-          <t>Un responsable des relations publiques est désigné.</t>
+          <t>L'organisation doit communiquer les activités de rétablissement aux parties prenantes prédéfinies, aux équipes de direction et de gestion.</t>
         </is>
       </c>
       <c r="J347" s="18" t="inlineStr">
         <is>
-          <t>Il convient que le responsable des relations publiques envisage l'utilisation de contacts externes prédéfinis (par exemple, la presse, les régulateurs, les groupes d'intérêt).</t>
+          <t>La communication des activités de rétablissement à toutes les parties prenantes concernées ne s'applique qu'aux entités soumises à la législation NIS.</t>
         </is>
       </c>
       <c r="L347" s="18" t="inlineStr">
         <is>
-          <t>Er moet een Public Relations Officer worden aangesteld.</t>
+          <t>De organisatie moet de herstelactiviteiten meedelen aan vooraf bepaalde belanghebbenden, directie- en managementteams.</t>
         </is>
       </c>
       <c r="M347" s="18" t="inlineStr">
         <is>
-          <t>De Public Relations Officer zou moeten overwegen gebruik te maken van vooraf bepaalde externe contacten (bijv. pers, regelgevers, belangengroepen).</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="B348" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D348" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-2</t>
-        </is>
-      </c>
-      <c r="F348" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reputation is repaired after an incident </t>
-        </is>
-      </c>
-      <c r="I348" s="15" t="inlineStr">
-        <is>
-          <t>La réputation est réparée après un incident.</t>
-        </is>
-      </c>
-      <c r="J348" t="inlineStr"/>
-      <c r="L348" s="16" t="inlineStr">
-        <is>
-          <t>Reputatie wordt hersteld na een incident.</t>
-        </is>
-      </c>
-    </row>
-    <row r="349" ht="72" customHeight="1">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B349" t="n">
-        <v>4</v>
-      </c>
-      <c r="C349" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D349" t="inlineStr">
-        <is>
-          <t>RC.CO-2.1</t>
-        </is>
-      </c>
-      <c r="F349" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall implement a crisis response strategy to protect the organization from the negative consequences of a crisis and help restore its reputation.</t>
-        </is>
-      </c>
-      <c r="G349" s="17" t="inlineStr">
-        <is>
-          <t>Crisis response strategies include, for example, actions to shape attributions of the crisis, change perceptions of the organization in crisis, and reduce the negative effect generated by the crisis.</t>
-        </is>
-      </c>
-      <c r="I349" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit mettre en œuvre une stratégie de réponse aux crises afin de protéger l'organisation des conséquences négatives d'une crise et de contribuer à restaurer sa réputation.</t>
-        </is>
-      </c>
-      <c r="J349" s="18" t="inlineStr">
-        <is>
-          <t>Les stratégies de réponse aux crises comprennent, par exemple, des actions visant à déterminer les attributions de la crise, à modifier les perceptions de l'organisation en crise et à réduire l'effet négatif généré par la crise.</t>
-        </is>
-      </c>
-      <c r="L349" s="18" t="inlineStr">
-        <is>
-          <t>Er moet een crisisbestrijdingsstrategie worden toegepast om de organisatie te beschermen tegen de negatieve gevolgen van een crisis en te helpen haar reputatie te herstellen.</t>
-        </is>
-      </c>
-      <c r="M349" s="18" t="inlineStr">
-        <is>
-          <t>Crisisbestrijdingsstrategieën omvatten bijvoorbeeld maatregelen om de beeldvorming over de crisis vorm te geven, de perceptie van de organisatie in crisis te veranderen, en het negatieve effect dat de crisis teweegbrengt te verminderen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="350" ht="43.2" customHeight="1">
-      <c r="B350" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D350" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-3</t>
-        </is>
-      </c>
-      <c r="F350" s="14" t="inlineStr">
-        <is>
-          <t>Recovery activities are communicated to internal and external stakeholders as well as executive and management teams</t>
-        </is>
-      </c>
-      <c r="I350" s="15" t="inlineStr">
-        <is>
-          <t>Les activités de rétablissement sont communiquées aux parties prenantes internes et externes, ainsi qu'aux équipes de direction et de gestion.</t>
-        </is>
-      </c>
-      <c r="J350" t="inlineStr"/>
-      <c r="L350" s="16" t="inlineStr">
-        <is>
-          <t>De herstelactiviteiten worden gecommuniceerd aan interne en externe belanghebbenden en aan directie- en managementteams.</t>
-        </is>
-      </c>
-    </row>
-    <row r="351" ht="57.6" customHeight="1">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B351" t="n">
-        <v>4</v>
-      </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D351" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RC.CO-3.1</t>
-        </is>
-      </c>
-      <c r="F351" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall communicate recovery activities to predefined stakeholders, executive and management teams.</t>
-        </is>
-      </c>
-      <c r="G351" s="17" t="inlineStr">
-        <is>
-          <t>Communication of recovery activities to all relevant stakeholders applies only to entities subject to the NIS legislation.</t>
-        </is>
-      </c>
-      <c r="I351" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit communiquer les activités de rétablissement aux parties prenantes prédéfinies, aux équipes de direction et de gestion.</t>
-        </is>
-      </c>
-      <c r="J351" s="18" t="inlineStr">
-        <is>
-          <t>La communication des activités de rétablissement à toutes les parties prenantes concernées ne s'applique qu'aux entités soumises à la législation NIS.</t>
-        </is>
-      </c>
-      <c r="L351" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de herstelactiviteiten meedelen aan vooraf bepaalde belanghebbenden, directie- en managementteams.</t>
-        </is>
-      </c>
-      <c r="M351" s="18" t="inlineStr">
-        <is>
           <t>Communicatie van herstelactiviteiten aan belanghebbenden geldt alleen voor entiteiten die onder de NIS- wetgeving vallen.</t>
         </is>
       </c>
     </row>
+    <row r="349" ht="72" customHeight="1"/>
+    <row r="350" ht="43.2" customHeight="1"/>
+    <row r="351" ht="57.6" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(lib)!: RS.MI-1.1 correction on cyfun 2023 (#4678)
* fix(lib): RS.MI-1.1 correction on cyfun 2023

Release note: due to a fix in the standard, some assessment data in RS.MI can be lost when upgrading to the new version of the library.
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
+++ b/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="cff_meta" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="cff_content" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="implementation_groups_meta" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="implementation_groups_content" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cff_meta" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cff_content" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="implementation_groups_meta" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="implementation_groups_content" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -124,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -201,6 +203,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,7 +604,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -611,10 +614,8 @@
           <t>publication_date</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2025-06-18 00:00:00</t>
-        </is>
+      <c r="B4" s="30" t="n">
+        <v>46255</v>
       </c>
     </row>
     <row r="5">
@@ -948,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M351"/>
+  <dimension ref="A1:M347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1052,8 +1053,6 @@
           <t>IDENTIFIER (ID)</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" s="7" t="inlineStr">
         <is>
           <t>IDENTIFICEREN (ID)</t>
@@ -1089,7 +1088,6 @@
           <t>Les données, le personnel, les dispositifs, les systèmes et les installations qui permettent à l'organisation d'atteindre ses objectifs opérationnels sont identifiés et gérés en fonction de leur importance relative par rapport aux objectifs de l'organisation et à sa stratégie en matière de risques.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" s="11" t="inlineStr">
         <is>
           <t>Vermogensbeheer</t>
@@ -1120,7 +1118,6 @@
           <t>Les dispositifs et systèmes physiques utilisés dans l'organisation sont inventoriés.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="L4" s="16" t="inlineStr">
         <is>
           <t>Inventarisatie van de binnen de organisatie gebruikte fysieke apparaten en systemen.</t>
@@ -1364,7 +1361,6 @@
           <t>Les plateformes et applications logicielles utilisées au sein de l'organisation sont inventoriées.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="L9" s="16" t="inlineStr">
         <is>
           <t>Inventarisatie van de binnen de organisatie gebruikte softwareplatforms en - toepassingen.</t>
@@ -1658,7 +1654,6 @@
           <t>La communication organisationnelle et les flux de données sont schématisés.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="L15" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve"> De organisatorische communicatie- en gegevensstromen worden in kaart gebracht.</t>
@@ -1858,7 +1853,6 @@
           <t xml:space="preserve"> Les systèmes d'information externes sont catalogués.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="L19" s="16" t="inlineStr">
         <is>
           <t>Externe informatiesystemen worden gecatalogiseerd.</t>
@@ -1990,7 +1984,6 @@
           <t>Les ressources sont organisées par ordre de priorité en fonction de leur classification, de leur criticité et de leur valeur opérationnelle.</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="L22" s="16" t="inlineStr">
         <is>
           <t>Middelen worden geprioriteerd op basis van hun classificatie, kriticiteit en bedrijfswaarde.</t>
@@ -2099,7 +2092,6 @@
           <t>Les rôles, responsabilités et pouvoirs en matière de cybersécurité pour l'ensemble du personnel et les parties prenantes tierces (par exemple, les fournisseurs, les clients, les partenaires) sont établis.</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
       <c r="L24" s="16" t="inlineStr">
         <is>
           <t>Rollen, verantwoordelijkheden en bevoegdheden op het gebied van informatie- en cyberbeveiliging worden vastgesteld voor het gehele personeel en belanghebbenden van derden.</t>
@@ -2244,7 +2236,6 @@
           <t>La mission, les objectifs, les parties prenantes et les activités de l'organisation sont compris et classés par ordre de priorité ; ces informations sont utilisées pour définir les rôles, les responsabilités et les décisions en matière de gestion des risques liés à la cybersécurité.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" s="11" t="inlineStr">
         <is>
           <t>Bedrijfsomgeving</t>
@@ -2275,7 +2266,6 @@
           <t>Le rôle de l'organisation dans la chaîne d'approvisionnement est identifié et communiqué.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="L28" s="16" t="inlineStr">
         <is>
           <t>De rol van de organisatie in de toeleveringsketen wordt vastgesteld en gecommuniceerd.</t>
@@ -2403,7 +2393,6 @@
           <t>La place de l'organisation dans les infrastructures critiques et son secteur d'activité est identifiée et communiquée.</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="L31" s="16" t="inlineStr">
         <is>
           <t>De plaats van de organisatie in de kritieke infrastructuur en haar bedrijfstak wordt vastgesteld en gecommuniceerd.</t>
@@ -2554,7 +2543,6 @@
           <t>Les dépendances et les fonctions critiques pour la prestation des services critiques sont établies.</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="L35" s="16" t="inlineStr">
         <is>
           <t>Afhankelijkheden en kritieke functies voor de levering van kritieke diensten zijn vastgesteld.</t>
@@ -2630,7 +2618,6 @@
           <t>Les exigences en matière de résilience pour soutenir la prestation de services essentiels sont établies pour tous les états de fonctionnement (par exemple, en cas de contrainte/attaque, pendant le rétablissement, les opérations normales).</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="L37" s="16" t="inlineStr">
         <is>
           <t>Voor alle operationele staten (bv. onder dwang/aanval, tijdens herstel, normale operaties) worden vereisten vastgesteld met betrekking tot weerbaarheid ter ondersteuning van de levering van kritieke diensten.</t>
@@ -2824,7 +2811,6 @@
           <t>Les politiques, procédures et processus de gestion et de suivi des exigences réglementaires, juridiques, environnementales et opérationnelles de l'organisation sont compris et contribuent à la gestion du risque de cybersécurité.</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" s="11" t="inlineStr">
         <is>
           <t>Bestuur</t>
@@ -2855,7 +2841,6 @@
           <t>La politique de cybersécurité de l'organisation est établie et communiquée .</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
       <c r="L42" s="16" t="inlineStr">
         <is>
           <t>Het cyberbeveiligingsbeleid van de organisatie wordt vastgesteld en gecommuniceerd.</t>
@@ -2995,7 +2980,6 @@
           <t>Les exigences légales et réglementaires concernant la cybersécurité, y compris les obligations en matière de vie privée et de libertés civiles, sont comprises et gérées .</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
       <c r="L45" s="16" t="inlineStr">
         <is>
           <t>Wettelijke en regelgevende voorschriften inzake cyberbeveiliging, met inbegrip van verplichtingen inzake privacy en burgerlijke vrijheden, worden begrepen en beheerd.</t>
@@ -3124,7 +3108,6 @@
           <t>Les processus de gouvernance et de gestion des risques traitent les risques de cybersécurité .</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
       <c r="L48" s="16" t="inlineStr">
         <is>
           <t>Governance- en risicobeheerprocessen adresseren risico's met betrekking tot cyberbeveiliging.</t>
@@ -3260,7 +3243,6 @@
           <t>L'organisation comprend le risque de cybersécurité pour les opérations de l'organisation (y compris la mission, les fonctions, l'image ou la réputation), ses actifs et les individus.</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" s="11" t="inlineStr">
         <is>
           <t>Risicobeoordeling</t>
@@ -3291,7 +3273,6 @@
           <t xml:space="preserve"> Les vulnérabilités des actifs sont identifiées et documentées.</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
       <c r="L52" s="16" t="inlineStr">
         <is>
           <t>Kwetsbaarheden van activa worden vastgesteld en gedocumenteerd.</t>
@@ -3475,7 +3456,6 @@
           <t>Les renseignements sur les cybermenaces sont reçus de forums de partage d'informations et de sources.</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
       <c r="L56" s="16" t="inlineStr">
         <is>
           <t>Informatie over cyberdreigingen wordt ontvangen van fora en bronnen voor informatie-uitwisseling.</t>
@@ -3601,7 +3581,6 @@
           <t>Les menaces, les vulnérabilités, les probabilités et les impacts sont utilisés pour déterminer les risques.</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
       <c r="L59" s="16" t="inlineStr">
         <is>
           <t>Bedreigingen, kwetsbaarheden, waarschijnlijkheden en gevolgen worden gebruikt om het risico te bepalen.</t>
@@ -3784,7 +3763,6 @@
           <t>Les réponses aux risques sont identifiées et classées par ordre de priorité.</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
       <c r="L63" s="16" t="inlineStr">
         <is>
           <t>Respons op risico’s worden vastgesteld en geprioriteerd.</t>
@@ -3879,7 +3857,6 @@
           <t>Les priorités, contraintes, tolérances au risque et hypothèses de l'organisation sont établies et utilisées pour soutenir les décisions relatives au risque opérationnel.</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
       <c r="K65" s="11" t="inlineStr">
         <is>
           <t>Risicobeheer</t>
@@ -3910,7 +3887,6 @@
           <t>Les processus de gestion des risques sont établis, gérés et acceptés par les parties prenantes de l’organisation.</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
       <c r="L66" s="16" t="inlineStr">
         <is>
           <t>Risicobeheerprocessen worden vastgesteld, beheerd en goedgekeurd door belanghebbenden in de organisatie.</t>
@@ -3986,7 +3962,6 @@
           <t>La tolérance de l'organisation au risque est déterminée et clairement exprimée.</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
       <c r="L68" s="16" t="inlineStr">
         <is>
           <t>De risicotolerantie van de organisatie wordt bepaald en duidelijk uitgedrukt.</t>
@@ -4062,7 +4037,6 @@
           <t>La détermination de la tolérance au risque de l'organisation est éclairée par son rôle dans l'infrastructure critique et l'analyse des risques spécifiques au secteur.</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
       <c r="L70" s="16" t="inlineStr">
         <is>
           <t>De organisatie bepaalt haar risicotolerantie op basis van haar rol in de analyse van kritieke infrastructuur en sectorspecifieke risico's.</t>
@@ -4148,7 +4122,6 @@
           <t>Les priorités, les contraintes, les tolérances au risque et les hypothèses de l'organisation sont établies et utilisées pour soutenir les décisions liées à la gestion des risques de la chaîne d'approvisionnement. L'organisation a établi et mis en œuvre les processus pour identifier, évaluer et gérer les risques liés à la chaîne d'approvisionnement.</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
       <c r="K72" s="11" t="inlineStr">
         <is>
           <t>Risicobeheer van de toeleveringsketen</t>
@@ -4179,7 +4152,6 @@
           <t>Les processus de gestion des risques liés à la chaîne d'approvisionnement sont identifiés, établis, évalués, gérés et acceptés par les parties prenantes de l'organisation.</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
       <c r="L73" s="16" t="inlineStr">
         <is>
           <t>De processen voor het beheer van cyberrisico's in de toeleveringsketen worden geïdentificeerd, vastgesteld, beoordeeld, beheerd en goedgekeurd door de belanghebbenden van de organisatie.</t>
@@ -4255,7 +4227,6 @@
           <t>Les fournisseurs et les partenaires tiers de systèmes d'information, de composants et de services sont identifiés, classés par ordre de priorité et évalués à l'aide d'un processus d'évaluation des risques de la cyberchaîne d’approvisionnement.</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
       <c r="L75" s="16" t="inlineStr">
         <is>
           <t>Leveranciers en externe partners van informatiesystemen, componenten en diensten worden geïdentificeerd, geprioriteerd en beoordeeld met behulp van een risicobeoordelingsproces voor de cybertoeleveringsketen.</t>
@@ -4381,7 +4352,6 @@
           <t>Les contrats avec les fournisseurs et les partenaires tiers sont utilisés pour mettre en œuvre des mesures appropriées conçues pour atteindre les objectifs du programme de cybersécurité et du plan de gestion des risques de la chaîne d'approvisionnement de l'organisation.</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
       <c r="L78" s="16" t="inlineStr">
         <is>
           <t>Contracten met leveranciers en externe partners worden gebruikt om passende maatregelen te implementeren, die dermate zijn ontworpen opdat wordt beantwoord aan de doelstellingen van het cyberbeveiligingsprogramma van de organisatie en haar cyber risicobeheersplan voor de toeleveringsketen.</t>
@@ -4563,7 +4533,6 @@
           <t>Les fournisseurs et les partenaires tiers sont régulièrement évalués à l'aide d'audits, de résultats de tests ou d'autres formes d'évaluation pour confirmer qu'ils respectent leurs obligations contractuelles.</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
       <c r="L82" s="16" t="inlineStr">
         <is>
           <t>Leveranciers en externe partners worden routinematig beoordeeld aan de hand van audits, testresultaten of andere vormen van evaluaties om te bevestigen dat zij aan hun contractuele verplichtingen voldoen.</t>
@@ -4689,7 +4658,6 @@
           <t>La planification et les tests de réponse et de rétablissement sont effectués avec les fournisseurs et les prestataires tiers.</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
       <c r="L85" s="16" t="inlineStr">
         <is>
           <t>Respons- en herstelplanning en tests worden uitgevoerd met leveranciers en derde partijen.</t>
@@ -4815,7 +4783,6 @@
           <t>PROTEGER (PR)</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
       <c r="K88" s="7" t="inlineStr">
         <is>
           <t>BESCHERMEN (PR)</t>
@@ -4851,7 +4818,6 @@
           <t>L'accès aux actifs physiques et logiques et aux installations associées est limité aux utilisateurs, processus et dispositifs autorisés, et est géré en fonction du risque évalué d'accès non autorisé aux activités et transactions autorisées.</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" s="11" t="inlineStr">
         <is>
           <t>Identiteitsbeheer, authenticatie en toegangscontrole</t>
@@ -4882,7 +4848,6 @@
           <t>Les identités et les identifiants sont émis, gérés, vérifiés, révoqués et audités pour les dispositifs, utilisateurs et processus autorisés.</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
       <c r="L90" s="16" t="inlineStr">
         <is>
           <t>Identiteiten en referenties (“credentials”) worden afgegeven, beheerd, geverifieerd, ingetrokken en gecontroleerd voor geautoriseerde apparaten, gebruikers en processen.</t>
@@ -5194,7 +5159,6 @@
           <t>L'accès physique aux actifs est géré et protégé.</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
       <c r="L96" s="16" t="inlineStr">
         <is>
           <t>De fysieke toegang tot activa wordt beheerd en beschermd.</t>
@@ -5449,7 +5413,6 @@
           <t>L'accès à distance est géré.</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
       <c r="L101" s="16" t="inlineStr">
         <is>
           <t>De toegang op afstand wordt beheerd.</t>
@@ -5755,7 +5718,6 @@
           <t>Les permissions et autorisations d'accès sont gérées en intégrant les principes du moindre privilège et de la séparation des tâches.</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
       <c r="L107" s="16" t="inlineStr">
         <is>
           <t>De toegangsrechten en machtigingen worden beheerd, met inachtneming van de beginselen van "least privilege" en scheiding van taken.</t>
@@ -6283,7 +6245,6 @@
           <t>L'intégrité du réseau (séparation du réseau, segmentation du réseau...) est protégée.</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
       <c r="L117" s="16" t="inlineStr">
         <is>
           <t>Netwerkintegriteit (netwerksegregatie, netwerksegmentatie...) wordt beschermd.</t>
@@ -6654,7 +6615,6 @@
           <t>Les identités sont prouvées et liées aux identifiants et présentées dans les interactions.</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
       <c r="L124" s="16" t="inlineStr">
         <is>
           <t>Identiteiten worden aangetoond en verbonden aan referenties (“credentials”) en bevestigd in interacties.</t>
@@ -6780,7 +6740,6 @@
           <t>Les utilisateurs, les appareils et les autres actifs sont authentifiés (par exemple, à un seul facteur, à plusieurs facteurs) en fonction du risque de la transaction (par exemple, les risques pour la sécurité et la confidentialité des individus et d’autres risques organisationnels)</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr"/>
       <c r="L127" s="16" t="inlineStr">
         <is>
           <t>Identiteiten worden aangetoond en verbonden aan referenties (“credentials”) en bevestigd in interacties.</t>
@@ -6866,7 +6825,6 @@
           <t>Le personnel et les partenaires de l'organisation reçoivent une formation de sensibilisation à la cybersécurité et sont formés à l'exécution de leurs tâches et responsabilités liées à la cybersécurité, conformément aux politiques, procédures et accords connexes.</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr"/>
       <c r="K129" s="11" t="inlineStr">
         <is>
           <t>Bewustmaking en opleiding</t>
@@ -6897,7 +6855,6 @@
           <t>Tous les utilisateurs sont informés et entrainés.</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr"/>
       <c r="L130" s="16" t="inlineStr">
         <is>
           <t>Alle gebruikers worden geïnformeerd en opgeleid.</t>
@@ -7091,7 +7048,6 @@
           <t xml:space="preserve"> Les utilisateurs privilégiés comprennent leurs rôles et leurs responsabilités.</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr"/>
       <c r="L134" s="16" t="inlineStr">
         <is>
           <t>Geprivilegieerde gebruikers begrijpen hun rollen en verantwoordelijkheden.</t>
@@ -7167,7 +7123,6 @@
           <t>Les parties prenantes tierces (par exemple, les fournisseurs, les clients, les partenaires) comprennent leurs rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
       <c r="L136" s="16" t="inlineStr">
         <is>
           <t>Belanghebbenden van derden (bijv. leveranciers, klanten, partners) begrijpen hun rol en verantwoordelijkheden.</t>
@@ -7393,7 +7348,6 @@
           <t>Les cadres supérieurs comprennent leurs rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
       <c r="L141" s="16" t="inlineStr">
         <is>
           <t>Hogere leidinggevenden begrijpen hun taken en verantwoordelijkheden.</t>
@@ -7469,7 +7423,6 @@
           <t>Le personnel de la sécurité physique et de la cybersécurité comprend ses rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr"/>
       <c r="L143" s="16" t="inlineStr">
         <is>
           <t>Fysiek en cyberbeveiligingspersoneel begrijpt hun rollen en verantwoordelijkheden.</t>
@@ -7555,7 +7508,6 @@
           <t>Les informations et les enregistrements (données) sont gérés conformément à la stratégie de l'organisation en matière de risques afin de protéger la confidentialité, l'intégrité et la disponibilité des informations.</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
       <c r="K145" s="12" t="inlineStr">
         <is>
           <t>Gegevensbeveiliging</t>
@@ -7586,7 +7538,6 @@
           <t>Les données au repos sont protégées.</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
       <c r="L146" s="15" t="inlineStr">
         <is>
           <t>Data in rust is beschermd.</t>
@@ -7674,7 +7625,6 @@
           <t>Les données en transit sont protégées.</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
       <c r="L148" s="16" t="inlineStr">
         <is>
           <t>Data-in-transitie is beschermd.</t>
@@ -7751,7 +7701,6 @@
           <t>Les actifs sont gérés de manière formelle tout au long de leur retrait, de leur transfert et de leur mise à disposition.</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
       <c r="L150" s="16" t="inlineStr">
         <is>
           <t>Activa worden formeel beheerd gedurende de verhuizing, overdracht en verwijdering.</t>
@@ -7986,7 +7935,6 @@
           <t>Une capacité adéquate pour assurer la disponibilité est maintenue.</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
       <c r="L155" s="16" t="inlineStr">
         <is>
           <t>Voldoende capaciteit om de beschikbaarheid te waarborgen.</t>
@@ -8162,7 +8110,6 @@
           <t>Les protections contre les fuites de données sont mises en œuvre.</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
       <c r="L159" s="16" t="inlineStr">
         <is>
           <t>Beveiligingen tegen datalekken worden geïmplementeerd.</t>
@@ -8241,7 +8188,6 @@
           <t>Des mécanismes de vérification de l'intégrité sont utilisés pour vérifier l'intégrité des logiciels, des microprogrammes et des informations.</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr"/>
       <c r="L161" s="16" t="inlineStr">
         <is>
           <t>Integriteitscontrolemechanismen worden gebruikt om de integriteit van software, firmware en informatie te controleren.</t>
@@ -8417,7 +8363,6 @@
           <t>L'environnement ou les environnements de développement et de test sont séparés de l'environnement de production.</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr"/>
       <c r="L165" s="16" t="inlineStr">
         <is>
           <t>De ontwikkelings- en testomgeving(en) zijn gescheiden van de productieomgeving.</t>
@@ -8497,7 +8442,6 @@
           <t>Les mécanismes de contrôle d'intégrité sont utilisés pour vérifier l'intégrité du matériel.</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr"/>
       <c r="L167" s="16" t="inlineStr">
         <is>
           <t>Integriteitscontrolemechanismen worden gebruikt om de integriteit van de hardware te verifiëren.</t>
@@ -8633,7 +8577,6 @@
           <t>Les politiques de sécurité (qui traitent de l'objectif, de la portée, des rôles, des responsabilités, de l'engagement de la direction et de la coordination entre les entités organisationnelles), les processus et les procédures sont maintenus et utilisés pour gérer la protection des systèmes d'information et des actifs.</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr"/>
       <c r="K170" s="11" t="inlineStr">
         <is>
           <t>Informatiebeschermingsprocessen en - procedures</t>
@@ -8664,7 +8607,6 @@
           <t>Une configuration de base des systèmes de contrôle des technologies de l'information/de l'industrie est créée et maintenue en intégrant les principes de sécurité.</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr"/>
       <c r="L171" s="16" t="inlineStr">
         <is>
           <t>Er wordt een basisconfiguratie van informatietechnologie/industriële controlesystemen gecreëerd en onderhouden, waarin de beveiligingsbeginselen zijn verwerkt .</t>
@@ -8798,7 +8740,6 @@
           <t>Un cycle de vie du développement des systèmes pour gérer les systèmes est mis en œuvre .</t>
         </is>
       </c>
-      <c r="J174" t="inlineStr"/>
       <c r="L174" s="16" t="inlineStr">
         <is>
           <t>Een levenscyclus voor systeemontwikkeling om systemen te beheren wordt geïmplementeerd.</t>
@@ -8942,7 +8883,6 @@
           <t>Des processus de contrôle des changements de configuration sont en place.</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr"/>
       <c r="L177" s="16" t="inlineStr">
         <is>
           <t>Er zijn processen voor het beheer van configuratiewijzigingen aanwezig.</t>
@@ -9068,7 +9008,6 @@
           <t>Des sauvegardes des informations sont effectuées, maintenues et testées .</t>
         </is>
       </c>
-      <c r="J180" t="inlineStr"/>
       <c r="L180" s="16" t="inlineStr">
         <is>
           <t>Er worden back-ups van informatie gemaakt, onderhouden en getest.</t>
@@ -9356,7 +9295,6 @@
           <t>La politique et les règlements concernant l'environnement physique d'exploitation des actifs de l'organisation sont respectés.</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr"/>
       <c r="L186" s="16" t="inlineStr">
         <is>
           <t>Beleid en voorschriften met betrekking tot de fysieke bedrijfsomgeving voor bedrijfsmiddelen van de organisatie worden nageleefd .</t>
@@ -9488,7 +9426,6 @@
           <t>Les données sont détruites conformément à la politique.</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr"/>
       <c r="L189" s="16" t="inlineStr">
         <is>
           <t>Gegevens worden vernietigd overeenkomstig beleid.</t>
@@ -9629,7 +9566,6 @@
           <t>Les processus de protection sont améliorés</t>
         </is>
       </c>
-      <c r="J192" t="inlineStr"/>
       <c r="L192" s="16" t="inlineStr">
         <is>
           <t>De beschermingsprocessen worden verbeterd.</t>
@@ -9808,7 +9744,6 @@
           <t>L'efficacité des technologies de protection est partagée.</t>
         </is>
       </c>
-      <c r="J196" t="inlineStr"/>
       <c r="L196" s="16" t="inlineStr">
         <is>
           <t>De doeltreffendheid van beschermingstechnologieën wordt gedeeld.</t>
@@ -9984,7 +9919,6 @@
           <t>Des plans de réponse (réponse aux incidents et continuité des activités) et des plans de rétablissement (reprise après incident et reprise après sinistre) sont en place et gérés.</t>
         </is>
       </c>
-      <c r="J200" t="inlineStr"/>
       <c r="L200" s="16" t="inlineStr">
         <is>
           <t>Responsplannen (Incident Response en Business Continuity) en herstelplannen (Incident Recovery en Disaster Recovery) zijn aanwezig en worden beheerd.</t>
@@ -10119,7 +10053,6 @@
           <t>La cybersécurité est incluse dans les pratiques de ressources humaines (déprovisionnement, sélection du personnel...).</t>
         </is>
       </c>
-      <c r="J203" t="inlineStr"/>
       <c r="L203" s="16" t="inlineStr">
         <is>
           <t>Cyberbeveiliging is opgenomen in de personeelsbeheer (afbouwen, personeelsscreening...).</t>
@@ -10248,7 +10181,6 @@
           <t>Un plan de gestion des vulnérabilités est élaboré et mis en œuvre.</t>
         </is>
       </c>
-      <c r="J206" t="inlineStr"/>
       <c r="L206" s="16" t="inlineStr">
         <is>
           <t>Een plan voor het beheer van kwetsbaarheden wordt ontwikkeld en uitgevoerd.</t>
@@ -10337,7 +10269,6 @@
           <t>La maintenance et la réparation des composants des systèmes de contrôle et d'information industriels sont effectuées conformément aux politiques et procédures.</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr"/>
       <c r="K208" s="11" t="inlineStr">
         <is>
           <t>Onderhoud</t>
@@ -10368,7 +10299,6 @@
           <t>L'entretien et la réparation des actifs de l'organisation sont effectués et consignés, avec des outils approuvés et contrôlés.</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr"/>
       <c r="L209" s="16" t="inlineStr">
         <is>
           <t>Onderhoud en reparatie van bedrijfsmiddelen van de organisatie worden uitgevoerd en geregistreerd, met goedgekeurde en gecontroleerde gereedschappen.</t>
@@ -10754,7 +10684,6 @@
           <t>La maintenance à distance des actifs de l'organisation est approuvée, consignée et effectuée de manière à empêcher tout accès non autorisé.</t>
         </is>
       </c>
-      <c r="J217" t="inlineStr"/>
       <c r="L217" s="16" t="inlineStr">
         <is>
           <t>Onderhoud op afstand van bedrijfsmiddelen van de organisatie moet worden goedgekeurd, geregistreerd en uitgevoerd op een wijze die ongeoorloofde toegang voorkomt.</t>
@@ -10940,7 +10869,6 @@
           <t>Les solutions de sécurité technique sont gérées de manière à garantir la sécurité et la résilience des systèmes et des actifs, conformément aux politiques, procédures et accords connexes.</t>
         </is>
       </c>
-      <c r="J221" t="inlineStr"/>
       <c r="K221" s="11" t="inlineStr">
         <is>
           <t>Beschermingstechnologie</t>
@@ -10971,7 +10899,6 @@
           <t>Les enregistrements d'audit/logs sont déterminés, documentés, mis en œuvre et révisés conformément à la politique.</t>
         </is>
       </c>
-      <c r="J222" t="inlineStr"/>
       <c r="L222" s="16" t="inlineStr">
         <is>
           <t>Registraties van audits/logs worden vastgesteld, gedocumenteerd, uitgevoerd en herzien overeenkomstig beleid.</t>
@@ -11203,7 +11130,6 @@
           <t>Les supports amovibles sont protégés et leur utilisation est limitée conformément à la politique.</t>
         </is>
       </c>
-      <c r="J227" t="inlineStr"/>
       <c r="L227" s="16" t="inlineStr">
         <is>
           <t>Verwisselbare media worden beschermd en het gebruik ervan wordt beperkt overeenkomstig het beleid.</t>
@@ -11379,7 +11305,6 @@
           <t>Le principe de la moindre fonctionnalité est incorporé en configurant les systèmes de manière à ne fournir que les capacités essentielles.</t>
         </is>
       </c>
-      <c r="J231" t="inlineStr"/>
       <c r="L231" s="16" t="inlineStr">
         <is>
           <t>Het beginsel van minimale functionaliteit wordt toegepast door systemen zo te configureren dat ze alleen essentiële mogelijkheden bieden.</t>
@@ -11555,7 +11480,6 @@
           <t>Les réseaux de communication et de contrôle sont protégés.</t>
         </is>
       </c>
-      <c r="J235" t="inlineStr"/>
       <c r="L235" s="16" t="inlineStr">
         <is>
           <t>Communicatie- en besturingsnetwerken zijn beveiligd.</t>
@@ -11743,7 +11667,6 @@
           <t>DETECTER (DE)</t>
         </is>
       </c>
-      <c r="J239" t="inlineStr"/>
       <c r="K239" s="7" t="inlineStr">
         <is>
           <t>DETECTEREN (DE)</t>
@@ -11774,8 +11697,6 @@
           <t>Anomalies et événements</t>
         </is>
       </c>
-      <c r="I240" t="inlineStr"/>
-      <c r="J240" t="inlineStr"/>
       <c r="K240" s="11" t="inlineStr">
         <is>
           <t>Anomalieën en gebeurtenissen</t>
@@ -11806,7 +11727,6 @@
           <t>Une base de référence des opérations du réseau et des flux de données attendus pour les utilisateurs et les systèmes est établie et gérée.</t>
         </is>
       </c>
-      <c r="J241" t="inlineStr"/>
       <c r="L241" s="16" t="inlineStr">
         <is>
           <t>Een baseline van netwerkoperaties en verwachte gegevensstromen voor gebruikers en systemen wordt vastgesteld en beheerd.</t>
@@ -11891,7 +11811,6 @@
           <t>Les événements détectés sont analysés pour comprendre les cibles et les méthodes d’attaque.</t>
         </is>
       </c>
-      <c r="J243" t="inlineStr"/>
       <c r="L243" s="16" t="inlineStr">
         <is>
           <t>Gedetecteerde events worden geanalyseerd om inzicht te krijgen in aanvalsdoelen en -methoden.</t>
@@ -12017,7 +11936,6 @@
           <t>Les données d'événements sont collectées et corrélées à partir de sources et de capteurs multiples.</t>
         </is>
       </c>
-      <c r="J246" t="inlineStr"/>
       <c r="L246" s="16" t="inlineStr">
         <is>
           <t>Gegevens m.b.t. events worden verzameld en gecorreleerd uit meerdere bronnen en sensoren.</t>
@@ -12197,7 +12115,6 @@
           <t>L'impact des événements est déterminé.</t>
         </is>
       </c>
-      <c r="J250" t="inlineStr"/>
       <c r="L250" s="16" t="inlineStr">
         <is>
           <t>De impact van events wordt bepaald.</t>
@@ -12273,7 +12190,6 @@
           <t>Les seuils d'alerte des incidents sont établis.</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr"/>
       <c r="L252" s="16" t="inlineStr">
         <is>
           <t>Er worden alarmdrempels voor incidenten vastgesteld.</t>
@@ -12409,7 +12325,6 @@
           <t>Le système d'information et les actifs sont surveillés pour identifier les événements de cybersécurité et vérifier l'efficacité des mesures de protection.</t>
         </is>
       </c>
-      <c r="J255" t="inlineStr"/>
       <c r="K255" s="11" t="inlineStr">
         <is>
           <t>Voortdurende bewaking van de beveiliging</t>
@@ -12440,7 +12355,6 @@
           <t>Le réseau est surveillé pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
       <c r="L256" s="16" t="inlineStr">
         <is>
           <t>Het netwerk wordt gemonitord om potentiële cyberbeveiligingsevents op te sporen.</t>
@@ -12637,7 +12551,6 @@
           <t>L'environnement physique est surveillé pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J260" t="inlineStr"/>
       <c r="L260" s="16" t="inlineStr">
         <is>
           <t>De fysieke omgeving wordt bewaakt om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -12763,7 +12676,6 @@
           <t>L'activité du personnel est surveillée pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J263" t="inlineStr"/>
       <c r="L263" s="16" t="inlineStr">
         <is>
           <t>Personeelsactiviteiten worden gemonitord om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -12941,7 +12853,6 @@
           <t>Le code malveillant est détecté.</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr"/>
       <c r="L267" s="16" t="inlineStr">
         <is>
           <t>Kwaadaardige code wordt gedetecteerd.</t>
@@ -13073,7 +12984,6 @@
           <t>Un code mobile non autorisé est détecté.</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr"/>
       <c r="L270" s="16" t="inlineStr">
         <is>
           <t>Ongeoorloofde mobiele code is gedetecteerd.</t>
@@ -13152,7 +13062,6 @@
           <t>L'activité des prestataires de services externes est surveillée pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr"/>
       <c r="L272" s="16" t="inlineStr">
         <is>
           <t>De activiteit van externe dienstverleners wordt gemonitord om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -13278,7 +13187,6 @@
           <t>La surveillance du personnel, des connexions, des dispositifs et des logiciels non autorisés est effectuée.</t>
         </is>
       </c>
-      <c r="J275" t="inlineStr"/>
       <c r="L275" s="16" t="inlineStr">
         <is>
           <t>Monitoring op onbevoegd personeel, verbindingen, apparatuur en software wordt uitgevoerd.</t>
@@ -13410,7 +13318,6 @@
           <t>Les analyses de vulnérabilité sont effectuées.</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr"/>
       <c r="L278" s="16" t="inlineStr">
         <is>
           <t>Kwetsbaarheidsscans worden uitgevoerd.</t>
@@ -13546,7 +13453,6 @@
           <t>Les processus et procédures de détection sont maintenus et testés pour garantir la prise de conscience des événements anormaux.</t>
         </is>
       </c>
-      <c r="J281" t="inlineStr"/>
       <c r="K281" s="11" t="inlineStr">
         <is>
           <t>Opsporingsprocessen</t>
@@ -13577,7 +13483,6 @@
           <t>Les activités de détection sont conformes à toutes les exigences applicables.</t>
         </is>
       </c>
-      <c r="J282" t="inlineStr"/>
       <c r="L282" s="16" t="inlineStr">
         <is>
           <t>Detectie moet gebeuren conform alle toepasselijke eisen.</t>
@@ -13653,7 +13558,6 @@
           <t>Les processus de détection sont testés.</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr"/>
       <c r="L284" s="16" t="inlineStr">
         <is>
           <t>Detectieprocessen worden getest.</t>
@@ -13732,7 +13636,6 @@
           <t>Les informations relatives à la détection des événements sont communiquées.</t>
         </is>
       </c>
-      <c r="J286" t="inlineStr"/>
       <c r="L286" s="16" t="inlineStr">
         <is>
           <t>Informatie over gedetecteerde events wordt gecommuniceerd.</t>
@@ -13808,7 +13711,6 @@
           <t>Les processus de détection sont améliorés en permanence.</t>
         </is>
       </c>
-      <c r="J288" t="inlineStr"/>
       <c r="L288" s="16" t="inlineStr">
         <is>
           <t>De processen voor het detecteren van abnormale events worden voortdurend verbeterd.</t>
@@ -13937,8 +13839,6 @@
           <t>REPONDRE (RS)</t>
         </is>
       </c>
-      <c r="I291" t="inlineStr"/>
-      <c r="J291" t="inlineStr"/>
       <c r="K291" s="7" t="inlineStr">
         <is>
           <t>REAGEREN (RS)</t>
@@ -13974,7 +13874,6 @@
           <t>Les processus et procédures de réponse sont exécutés et maintenus, afin de garantir une réponse aux incidents de cybersécurité détectés.</t>
         </is>
       </c>
-      <c r="J292" t="inlineStr"/>
       <c r="K292" s="11" t="inlineStr">
         <is>
           <t>Responsplanning</t>
@@ -14005,7 +13904,6 @@
           <t xml:space="preserve"> Le plan de réponse est exécuté pendant ou après un incident.</t>
         </is>
       </c>
-      <c r="J293" t="inlineStr"/>
       <c r="L293" s="16" t="inlineStr">
         <is>
           <t>Het responsplan wordt uitgevoerd tijdens of na een incident.</t>
@@ -14097,7 +13995,6 @@
           <t>Les activités de réponse sont coordonnées avec les parties prenantes internes et externes (par exemple, le soutien externe des forces de l'ordre).</t>
         </is>
       </c>
-      <c r="J295" t="inlineStr"/>
       <c r="K295" s="11" t="inlineStr">
         <is>
           <t>Communicatie</t>
@@ -14128,7 +14025,6 @@
           <t>Le personnel connaît ses rôles et l'ordre des opérations lorsqu'une réponse est nécessaire.</t>
         </is>
       </c>
-      <c r="J296" t="inlineStr"/>
       <c r="L296" s="16" t="inlineStr">
         <is>
           <t>Het personeel kent zijn rol en volgorde van handelen wanneer een reactie nodig is.</t>
@@ -14204,7 +14100,6 @@
           <t>Les incidents sont signalés conformément aux critères établis.</t>
         </is>
       </c>
-      <c r="J298" t="inlineStr"/>
       <c r="L298" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden gemeld overeenkomstig de vastgestelde criteria.</t>
@@ -14330,7 +14225,6 @@
           <t>Les informations sont partagées conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J301" t="inlineStr"/>
       <c r="L301" s="16" t="inlineStr">
         <is>
           <t>Informatie wordt gedeeld in overeenstemming met de responsplannen.</t>
@@ -14456,7 +14350,6 @@
           <t>La coordination avec les parties prenantes se fait conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J304" t="inlineStr"/>
       <c r="L304" s="16" t="inlineStr">
         <is>
           <t>Coördinatie met belanghebbenden vindt plaats in overeenstemming met de responsplannen.</t>
@@ -14535,7 +14428,6 @@
           <t>Le partage volontaire d'informations se fait avec des parties prenantes externes afin d'obtenir une meilleure connaissance de la situation en matière de cybersécurité.</t>
         </is>
       </c>
-      <c r="J306" t="inlineStr"/>
       <c r="L306" s="16" t="inlineStr">
         <is>
           <t>Er vindt vrijwillige informatie-uitwisseling plaats met externe belanghebbenden om een breder situationeel bewustzijn over cyberbeveiliging te bereiken.</t>
@@ -14621,7 +14513,6 @@
           <t>Une analyse est effectuée pour garantir une réponse efficace et soutenir les activités de rétablissement.</t>
         </is>
       </c>
-      <c r="J308" t="inlineStr"/>
       <c r="K308" s="11" t="inlineStr">
         <is>
           <t>Analyse</t>
@@ -14652,7 +14543,6 @@
           <t>Les notifications des systèmes de détection sont examinées.</t>
         </is>
       </c>
-      <c r="J309" t="inlineStr"/>
       <c r="L309" s="16" t="inlineStr">
         <is>
           <t>RS.AN-1:  Meldingen van detectiesystemen worden onderzocht.</t>
@@ -14778,7 +14668,6 @@
           <t>L'impact de l'incident est compris.</t>
         </is>
       </c>
-      <c r="J312" t="inlineStr"/>
       <c r="L312" s="16" t="inlineStr">
         <is>
           <t>De gevolgen van het incident worden begrepen.</t>
@@ -14907,7 +14796,6 @@
           <t>L'analyse forensique est réalisée.</t>
         </is>
       </c>
-      <c r="J315" t="inlineStr"/>
       <c r="L315" s="16" t="inlineStr">
         <is>
           <t>Forensisch onderzoek wordt uitgevoerd.</t>
@@ -15033,7 +14921,6 @@
           <t>Les incidents sont classés par catégories conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J318" t="inlineStr"/>
       <c r="L318" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden in categorieën ingedeeld overeenkomstig de responsplannen.</t>
@@ -15114,7 +15001,6 @@
           <t>Des processus sont établis pour recevoir, analyser et répondre aux vulnérabilités divulguées à l'organisation par des sources internes et externes (par exemple, tests internes, bulletins de sécurité ou chercheurs en sécurité).</t>
         </is>
       </c>
-      <c r="J320" t="inlineStr"/>
       <c r="L320" s="16" t="inlineStr">
         <is>
           <t>Er zijn processen vastgesteld voor het ontvangen, analyseren en reageren op kwetsbaarheden die uit interne en externe bronnen (bv. interne tests, beveiligingsbulletins of beveiligingsonderzoekers) aan de organisatie bekend zijn gemaakt.</t>
@@ -15247,10 +15133,9 @@
       </c>
       <c r="I323" s="11" t="inlineStr">
         <is>
-          <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
-        </is>
-      </c>
-      <c r="J323" t="inlineStr"/>
+          <t>Des activités sont menées afin d'empêcher l'extension d'un événement, d'en atténuer les effets et de résoudre l'incident.</t>
+        </is>
+      </c>
       <c r="K323" s="11" t="inlineStr">
         <is>
           <t>Mitigatie</t>
@@ -15281,7 +15166,6 @@
           <t>Les incidents sont contenus.</t>
         </is>
       </c>
-      <c r="J324" t="inlineStr"/>
       <c r="L324" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden beheerst.</t>
@@ -15307,74 +15191,149 @@
           <t>IMPORTANT_RS.MI-1.1</t>
         </is>
       </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>The organization shall implement an incident handling capability for information/cybersecurity incidents on its business critical systems that includes preparation, detection and analysis, containment, eradication, recovery and documented risk acceptance.</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>A documented risk acceptance deals with risks that the organisation assesses as not dangerous to the organisation's business critical systems and where the risk owner formally accepts the risk (related with the risk appetite of the organization)</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre en œuvre une capacité de traitement des incidents de sécurité de l'information/cybersécurité sur ses systèmes essentiels à l'activité, qui comprend la préparation, la détection et l'analyse, le confinement, l'éradication, le rétablissement et l'acceptation documentée des risques.</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>Une acceptation des risques documentée concerne les risques que l'organisation évalue comme non dangereux pour les systèmes critiques de l'organisation et pour lesquels le propriétaire du risque accepte formellement le risque (en relation avec l'appétit de l'organisation pour le risque).</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>De organisatie moet een capaciteit voor het afhandelen van informatie- /cyberbeveiligingsincidenten op haar bedrijfskritische systemen implementeren die de voorbereiding, detectie, analyse, insluiting (“containment”), uitroeiing, herstel en gedocumenteerde risicoaanvaarding omvat.</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>Een gedocumenteerde risicoaanvaarding heeft betrekking op risico's die volgens de organisatie niet gevaarlijk zijn voor de bedrijfskritische systemen van de organisatie en waarbij de eigenaar van het risico het risico formeel aanvaardt (gerelateerd aan de risicobereidheid, ”risk appetite”, van de organisatie).</t>
+        </is>
+      </c>
     </row>
     <row r="326">
-      <c r="B326" s="13" t="n">
+      <c r="B326" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D326" s="8" t="inlineStr">
+        <is>
+          <t>RS.IM</t>
+        </is>
+      </c>
+      <c r="E326" s="8" t="inlineStr">
+        <is>
+          <t>Improvements</t>
+        </is>
+      </c>
+      <c r="F326" s="9" t="inlineStr">
+        <is>
+          <t>Organizational response activities are improved by incorporating lessons learned from current and previous detection/response activities.</t>
+        </is>
+      </c>
+      <c r="H326" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Améliorations </t>
+        </is>
+      </c>
+      <c r="I326" s="11" t="inlineStr">
+        <is>
+          <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
+        </is>
+      </c>
+      <c r="K326" s="11" t="inlineStr">
+        <is>
+          <t>Verbeteringen</t>
+        </is>
+      </c>
+      <c r="L326" s="12" t="inlineStr">
+        <is>
+          <t>De responsactiviteiten van de organisatie worden verbeterd door lessen te trekken uit huidige en eerdere opsporings- en responsactiviteiten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="B327" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D326" s="13" t="inlineStr">
-        <is>
-          <t>RS.MI-2</t>
-        </is>
-      </c>
-      <c r="F326" s="14" t="inlineStr">
-        <is>
-          <t>Incidents are mitigated</t>
-        </is>
-      </c>
-      <c r="I326" s="15" t="inlineStr">
-        <is>
-          <t>Les incidents sont atténués.</t>
-        </is>
-      </c>
-      <c r="L326" s="16" t="inlineStr">
-        <is>
-          <t>Incidenten worden gemitigeerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B327" t="n">
-        <v>4</v>
-      </c>
-      <c r="C327" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D327" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RS.MI-2.1</t>
+      <c r="D327" s="13" t="inlineStr">
+        <is>
+          <t>RS.IM-1</t>
+        </is>
+      </c>
+      <c r="F327" s="14" t="inlineStr">
+        <is>
+          <t>Response plans incorporate lessons learned</t>
+        </is>
+      </c>
+      <c r="I327" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de réponse intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L327" s="16" t="inlineStr">
+        <is>
+          <t>In de responsplannen zijn de geleerde lessen verwerkt.</t>
         </is>
       </c>
     </row>
     <row r="328" ht="43.2" customHeight="1">
-      <c r="B328" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D328" s="13" t="inlineStr">
-        <is>
-          <t>RS.MI-3</t>
-        </is>
-      </c>
-      <c r="F328" s="14" t="inlineStr">
-        <is>
-          <t>Newly identified vulnerabilities are mitigated or documented as accepted risks</t>
-        </is>
-      </c>
-      <c r="I328" s="15" t="inlineStr">
-        <is>
-          <t>Les vulnérabilités nouvellement identifiées sont atténuées ou documentées comme des risques acceptés.</t>
-        </is>
-      </c>
-      <c r="L328" s="16" t="inlineStr">
-        <is>
-          <t>Nieuw vastgestelde kwetsbaarheden worden gemitigeerd of gedocumenteerd als aanvaarde risico's.</t>
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>4</v>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>B,I,E</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>BASIC_RS.IM-1.1</t>
+        </is>
+      </c>
+      <c r="F328" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall conduct post-incident evaluations to analyse lessons learned from incident response and recovery, and consequently improve processes / procedures / technologies to enhance its cyber resilience.</t>
+        </is>
+      </c>
+      <c r="G328" s="17" t="inlineStr">
+        <is>
+          <t>Consider bringing involved people together after each incident and reflect together on ways to improve what happened, how it happened, how we reacted, how it could have gone better, what should be done to prevent it from happening again, etc.</t>
+        </is>
+      </c>
+      <c r="I328" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit effectuer des évaluations post-incident afin d'analyser les enseignements tirés de la réponse à l'incident et du rétablissement, et par conséquent améliorer les processus / procédures / technologies pour renforcer sa cyber-résilience.</t>
+        </is>
+      </c>
+      <c r="J328" s="18" t="inlineStr">
+        <is>
+          <t>Envisagez de réunir les personnes concernées après chaque incident et réfléchissez ensemble aux moyens d'améliorer ce qui s'est passé, comment cela s'est passé, comment nous avons réagi, comment cela aurait pu mieux se passer, ce qui devrait être fait pour éviter que cela ne se reproduise, etc.</t>
+        </is>
+      </c>
+      <c r="L328" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet evaluaties uitvoeren na een incident om lessen te trekken uit de reactie op en het herstel van incidenten, en verbetert vervolgens de processen / procedures / technologieën om haar cyberweerbaarheid te vergroten.</t>
+        </is>
+      </c>
+      <c r="M328" s="18" t="inlineStr">
+        <is>
+          <t>Overweeg na elk incident de betrokkenen samen te brengen en samen na te denken over manieren om te verbeteren wat er is gebeurd, hoe het is gebeurd, hoe er is gereageerd, hoe het beter had kunnen gaan, wat er moet gebeuren om herhaling te voorkomen, enz.</t>
         </is>
       </c>
     </row>
@@ -15394,204 +15353,177 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>IMPORTANT_RS.MI-3.1</t>
+          <t>IMPORTANT_RS.IM-1.2</t>
         </is>
       </c>
       <c r="F329" s="17" t="inlineStr">
         <is>
-          <t>The organization shall implement an incident handling capability for information/cybersecurity incidents on its business critical systems that includes preparation, detection and analysis, containment, eradication, recovery and documented risk acceptance.</t>
+          <t>Lessons learned from incident handling shall be translated into updated or new incident handling procedures that shall be tested, approved and trained.</t>
         </is>
       </c>
       <c r="G329" s="17" t="inlineStr">
         <is>
-          <t>A documented risk acceptance deals with risks that the organisation assesses as not dangerous to the organisation's business critical systems and where the risk owner formally accepts the risk (related with the risk appetite of the organization)</t>
+          <t>No additional guidance on this topic.</t>
         </is>
       </c>
       <c r="I329" s="18" t="inlineStr">
         <is>
-          <t>L'organisation doit mettre en œuvre une capacité de traitement des incidents de sécurité de l'information/cybersécurité sur ses systèmes essentiels à l'activité, qui comprend la préparation, la détection et l'analyse, le confinement, l'éradication, le rétablissement et l'acceptation documentée des risques.</t>
+          <t>Les enseignements tirés du traitement des incidents sont traduits en procédures de traitement des incidents actualisées ou nouvelles qui sont testées, approuvées et enseignées.</t>
         </is>
       </c>
       <c r="J329" s="18" t="inlineStr">
         <is>
-          <t>Une acceptation des risques documentée concerne les risques que l'organisation évalue comme non dangereux pour les systèmes critiques de l'organisation et pour lesquels le propriétaire du risque accepte formellement le risque (en relation avec l'appétit de l'organisation pour le risque).</t>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
         </is>
       </c>
       <c r="L329" s="18" t="inlineStr">
         <is>
-          <t>De organisatie moet een capaciteit voor het afhandelen van informatie- /cyberbeveiligingsincidenten op haar bedrijfskritische systemen implementeren die de voorbereiding, detectie, analyse, insluiting (“containment”), uitroeiing, herstel en gedocumenteerde risicoaanvaarding omvat.</t>
+          <t>De uit de afhandeling van incidenten geleerde lessen moeten worden vertaald in bijgewerkte of nieuwe procedures voor de afhandeling van incidenten, die op hun beurt moeten worden getest, goedgekeurd en getraind.</t>
         </is>
       </c>
       <c r="M329" s="18" t="inlineStr">
         <is>
-          <t>Een gedocumenteerde risicoaanvaarding heeft betrekking op risico's die volgens de organisatie niet gevaarlijk zijn voor de bedrijfskritische systemen van de organisatie en waarbij de eigenaar van het risico het risico formeel aanvaardt (gerelateerd aan de risicobereidheid, ”risk appetite”, van de organisatie).</t>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
         </is>
       </c>
     </row>
     <row r="330" ht="57.6" customHeight="1">
-      <c r="B330" s="8" t="n">
+      <c r="B330" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D330" s="13" t="inlineStr">
+        <is>
+          <t>RS.IM-2</t>
+        </is>
+      </c>
+      <c r="F330" s="14" t="inlineStr">
+        <is>
+          <t>Response and Recovery strategies are updated</t>
+        </is>
+      </c>
+      <c r="I330" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de réponse intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L330" s="16" t="inlineStr">
+        <is>
+          <t>Reactie- en herstelstrategieën worden bijgewerkt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>4</v>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RS.IM-2.1</t>
+        </is>
+      </c>
+      <c r="F331" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall update the response and recovery  plans to address changes in its context.</t>
+        </is>
+      </c>
+      <c r="G331" s="17" t="inlineStr">
+        <is>
+          <t>The organization’s context relates to the organizational structure, its critical systems, attack vectors, new threats, improved technology, environment of operation, problems encountered during plan implementation/execution/testing and lessons learned.</t>
+        </is>
+      </c>
+      <c r="I331" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre à jour les plans de réponse et de rétablissement pour tenir compte des changements survenus dans son contexte.</t>
+        </is>
+      </c>
+      <c r="J331" s="18" t="inlineStr">
+        <is>
+          <t>Le contexte de l'organisation concerne la structure organisationnelle, ses systèmes critiques, les vecteurs d'attaque, les nouvelles menaces, les améliorations technologiques, l'environnement d'exploitation, les problèmes rencontrés lors de la mise en œuvre/exécution/test du plan et les enseignements tirés.</t>
+        </is>
+      </c>
+      <c r="L331" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de reactie- en herstelplannen aanpassen aan veranderingen in haar context.</t>
+        </is>
+      </c>
+      <c r="M331" s="18" t="inlineStr">
+        <is>
+          <t>De context van de organisatie heeft betrekking op de organisatiestructuur, haar kritieke systemen, aanvalsvectoren, nieuwe bedreigingen, verbeterde technologie, de bedrijfsomgeving, problemen die zich hebben voorgedaan tijdens de implementatie/uitvoering/testen van het plan en de lessen die zijn geleerd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="86.40000000000001" customHeight="1">
+      <c r="B332" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D332" s="5" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="E332" s="5" t="inlineStr">
+        <is>
+          <t>RECOVER (RC)</t>
+        </is>
+      </c>
+      <c r="H332" s="5" t="inlineStr">
+        <is>
+          <t>RETABLIR (RC)</t>
+        </is>
+      </c>
+      <c r="K332" s="7" t="inlineStr">
+        <is>
+          <t>HERSTELLEN (RC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="57.6" customHeight="1">
+      <c r="B333" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D330" s="8" t="inlineStr">
-        <is>
-          <t>RS.IM</t>
-        </is>
-      </c>
-      <c r="E330" s="8" t="inlineStr">
-        <is>
-          <t>Improvements</t>
-        </is>
-      </c>
-      <c r="F330" s="9" t="inlineStr">
-        <is>
-          <t>Organizational response activities are improved by incorporating lessons learned from current and previous detection/response activities.</t>
-        </is>
-      </c>
-      <c r="H330" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Améliorations </t>
-        </is>
-      </c>
-      <c r="I330" s="11" t="inlineStr">
-        <is>
-          <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
-        </is>
-      </c>
-      <c r="J330" t="inlineStr"/>
-      <c r="K330" s="11" t="inlineStr">
-        <is>
-          <t>Verbeteringen</t>
-        </is>
-      </c>
-      <c r="L330" s="12" t="inlineStr">
-        <is>
-          <t>De responsactiviteiten van de organisatie worden verbeterd door lessen te trekken uit huidige en eerdere opsporings- en responsactiviteiten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="331">
-      <c r="B331" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D331" s="13" t="inlineStr">
-        <is>
-          <t>RS.IM-1</t>
-        </is>
-      </c>
-      <c r="F331" s="14" t="inlineStr">
-        <is>
-          <t>Response plans incorporate lessons learned</t>
-        </is>
-      </c>
-      <c r="I331" s="15" t="inlineStr">
-        <is>
-          <t>Les plans de réponse intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J331" t="inlineStr"/>
-      <c r="L331" s="16" t="inlineStr">
-        <is>
-          <t>In de responsplannen zijn de geleerde lessen verwerkt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="332" ht="86.40000000000001" customHeight="1">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B332" t="n">
-        <v>4</v>
-      </c>
-      <c r="C332" t="inlineStr">
-        <is>
-          <t>B,I,E</t>
-        </is>
-      </c>
-      <c r="D332" t="inlineStr">
-        <is>
-          <t>BASIC_RS.IM-1.1</t>
-        </is>
-      </c>
-      <c r="F332" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall conduct post-incident evaluations to analyse lessons learned from incident response and recovery, and consequently improve processes / procedures / technologies to enhance its cyber resilience.</t>
-        </is>
-      </c>
-      <c r="G332" s="17" t="inlineStr">
-        <is>
-          <t>Consider bringing involved people together after each incident and reflect together on ways to improve what happened, how it happened, how we reacted, how it could have gone better, what should be done to prevent it from happening again, etc.</t>
-        </is>
-      </c>
-      <c r="I332" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit effectuer des évaluations post-incident afin d'analyser les enseignements tirés de la réponse à l'incident et du rétablissement, et par conséquent améliorer les processus / procédures / technologies pour renforcer sa cyber-résilience.</t>
-        </is>
-      </c>
-      <c r="J332" s="18" t="inlineStr">
-        <is>
-          <t>Envisagez de réunir les personnes concernées après chaque incident et réfléchissez ensemble aux moyens d'améliorer ce qui s'est passé, comment cela s'est passé, comment nous avons réagi, comment cela aurait pu mieux se passer, ce qui devrait être fait pour éviter que cela ne se reproduise, etc.</t>
-        </is>
-      </c>
-      <c r="L332" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet evaluaties uitvoeren na een incident om lessen te trekken uit de reactie op en het herstel van incidenten, en verbetert vervolgens de processen / procedures / technologieën om haar cyberweerbaarheid te vergroten.</t>
-        </is>
-      </c>
-      <c r="M332" s="18" t="inlineStr">
-        <is>
-          <t>Overweeg na elk incident de betrokkenen samen te brengen en samen na te denken over manieren om te verbeteren wat er is gebeurd, hoe het is gebeurd, hoe er is gereageerd, hoe het beter had kunnen gaan, wat er moet gebeuren om herhaling te voorkomen, enz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="333" ht="57.6" customHeight="1">
-      <c r="A333" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B333" t="n">
-        <v>4</v>
-      </c>
-      <c r="C333" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D333" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RS.IM-1.2</t>
-        </is>
-      </c>
-      <c r="F333" s="17" t="inlineStr">
-        <is>
-          <t>Lessons learned from incident handling shall be translated into updated or new incident handling procedures that shall be tested, approved and trained.</t>
-        </is>
-      </c>
-      <c r="G333" s="17" t="inlineStr">
-        <is>
-          <t>No additional guidance on this topic.</t>
-        </is>
-      </c>
-      <c r="I333" s="18" t="inlineStr">
-        <is>
-          <t>Les enseignements tirés du traitement des incidents sont traduits en procédures de traitement des incidents actualisées ou nouvelles qui sont testées, approuvées et enseignées.</t>
-        </is>
-      </c>
-      <c r="J333" s="18" t="inlineStr">
-        <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
-        </is>
-      </c>
-      <c r="L333" s="18" t="inlineStr">
-        <is>
-          <t>De uit de afhandeling van incidenten geleerde lessen moeten worden vertaald in bijgewerkte of nieuwe procedures voor de afhandeling van incidenten, die op hun beurt moeten worden getest, goedgekeurd en getraind.</t>
-        </is>
-      </c>
-      <c r="M333" s="18" t="inlineStr">
-        <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+      <c r="D333" s="8" t="inlineStr">
+        <is>
+          <t>RC.RP</t>
+        </is>
+      </c>
+      <c r="E333" s="8" t="inlineStr">
+        <is>
+          <t>Recovery Planning</t>
+        </is>
+      </c>
+      <c r="F333" s="9" t="inlineStr">
+        <is>
+          <t>Recovery processes and procedures are executed and maintained to ensure restoration of systems or assets affected by cybersecurity incidents.</t>
+        </is>
+      </c>
+      <c r="H333" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planification du rétablissement </t>
+        </is>
+      </c>
+      <c r="I333" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K333" s="11" t="inlineStr">
+        <is>
+          <t>Herstelplanning</t>
+        </is>
+      </c>
+      <c r="L333" s="12" t="inlineStr">
+        <is>
+          <t>Herstelprocessen en -procedures worden uitgevoerd en gehandhaafd om te zorgen voor herstel van systemen of activa die zijn getroffen door cyberbeveiligingsincidenten.</t>
         </is>
       </c>
     </row>
@@ -15601,23 +15533,22 @@
       </c>
       <c r="D334" s="13" t="inlineStr">
         <is>
-          <t>RS.IM-2</t>
+          <t>RC.RP-1</t>
         </is>
       </c>
       <c r="F334" s="14" t="inlineStr">
         <is>
-          <t>Response and Recovery strategies are updated</t>
+          <t xml:space="preserve">Recovery plan is executed during or after a cybersecurity incident </t>
         </is>
       </c>
       <c r="I334" s="15" t="inlineStr">
         <is>
-          <t>Les plans de réponse intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J334" t="inlineStr"/>
+          <t xml:space="preserve"> Le plan de reprise est exécuté pendant ou après un incident de cybersécurité.</t>
+        </is>
+      </c>
       <c r="L334" s="16" t="inlineStr">
         <is>
-          <t>Reactie- en herstelstrategieën worden bijgewerkt.</t>
+          <t>Het herstelplan wordt uitgevoerd tijdens of na een cyberbeveiligingsincident.</t>
         </is>
       </c>
     </row>
@@ -15632,164 +15563,20 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>I,E</t>
+          <t>B,I,E</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>IMPORTANT_RS.IM-2.1</t>
+          <t>BASIC_RC.RP-1.1</t>
         </is>
       </c>
       <c r="F335" s="17" t="inlineStr">
         <is>
-          <t>The organization shall update the response and recovery  plans to address changes in its context.</t>
+          <t>A recovery process for disasters and information/cybersecurity incidents shall be developed and executed as appropriate.</t>
         </is>
       </c>
       <c r="G335" s="17" t="inlineStr">
-        <is>
-          <t>The organization’s context relates to the organizational structure, its critical systems, attack vectors, new threats, improved technology, environment of operation, problems encountered during plan implementation/execution/testing and lessons learned.</t>
-        </is>
-      </c>
-      <c r="I335" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit mettre à jour les plans de réponse et de rétablissement pour tenir compte des changements survenus dans son contexte.</t>
-        </is>
-      </c>
-      <c r="J335" s="18" t="inlineStr">
-        <is>
-          <t>Le contexte de l'organisation concerne la structure organisationnelle, ses systèmes critiques, les vecteurs d'attaque, les nouvelles menaces, les améliorations technologiques, l'environnement d'exploitation, les problèmes rencontrés lors de la mise en œuvre/exécution/test du plan et les enseignements tirés.</t>
-        </is>
-      </c>
-      <c r="L335" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de reactie- en herstelplannen aanpassen aan veranderingen in haar context.</t>
-        </is>
-      </c>
-      <c r="M335" s="18" t="inlineStr">
-        <is>
-          <t>De context van de organisatie heeft betrekking op de organisatiestructuur, haar kritieke systemen, aanvalsvectoren, nieuwe bedreigingen, verbeterde technologie, de bedrijfsomgeving, problemen die zich hebben voorgedaan tijdens de implementatie/uitvoering/testen van het plan en de lessen die zijn geleerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="B336" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D336" s="5" t="inlineStr">
-        <is>
-          <t>RC</t>
-        </is>
-      </c>
-      <c r="E336" s="5" t="inlineStr">
-        <is>
-          <t>RECOVER (RC)</t>
-        </is>
-      </c>
-      <c r="H336" s="5" t="inlineStr">
-        <is>
-          <t>RETABLIR (RC)</t>
-        </is>
-      </c>
-      <c r="I336" t="inlineStr"/>
-      <c r="J336" t="inlineStr"/>
-      <c r="K336" s="7" t="inlineStr">
-        <is>
-          <t>HERSTELLEN (RC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="337" ht="57.6" customHeight="1">
-      <c r="B337" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D337" s="8" t="inlineStr">
-        <is>
-          <t>RC.RP</t>
-        </is>
-      </c>
-      <c r="E337" s="8" t="inlineStr">
-        <is>
-          <t>Recovery Planning</t>
-        </is>
-      </c>
-      <c r="F337" s="9" t="inlineStr">
-        <is>
-          <t>Recovery processes and procedures are executed and maintained to ensure restoration of systems or assets affected by cybersecurity incidents.</t>
-        </is>
-      </c>
-      <c r="H337" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Planification du rétablissement </t>
-        </is>
-      </c>
-      <c r="I337" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J337" t="inlineStr"/>
-      <c r="K337" s="11" t="inlineStr">
-        <is>
-          <t>Herstelplanning</t>
-        </is>
-      </c>
-      <c r="L337" s="12" t="inlineStr">
-        <is>
-          <t>Herstelprocessen en -procedures worden uitgevoerd en gehandhaafd om te zorgen voor herstel van systemen of activa die zijn getroffen door cyberbeveiligingsincidenten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="338" ht="28.8" customHeight="1">
-      <c r="B338" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D338" s="13" t="inlineStr">
-        <is>
-          <t>RC.RP-1</t>
-        </is>
-      </c>
-      <c r="F338" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recovery plan is executed during or after a cybersecurity incident </t>
-        </is>
-      </c>
-      <c r="I338" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Le plan de reprise est exécuté pendant ou après un incident de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J338" t="inlineStr"/>
-      <c r="L338" s="16" t="inlineStr">
-        <is>
-          <t>Het herstelplan wordt uitgevoerd tijdens of na een cyberbeveiligingsincident.</t>
-        </is>
-      </c>
-    </row>
-    <row r="339" ht="244.8" customHeight="1">
-      <c r="A339" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B339" t="n">
-        <v>4</v>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>B,I,E</t>
-        </is>
-      </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>BASIC_RC.RP-1.1</t>
-        </is>
-      </c>
-      <c r="F339" s="17" t="inlineStr">
-        <is>
-          <t>A recovery process for disasters and information/cybersecurity incidents shall be developed and executed as appropriate.</t>
-        </is>
-      </c>
-      <c r="G339" s="17" t="inlineStr">
         <is>
           <t>A process should be developed for what immediate actions will be taken in case of a fire, medical emergency, burglary, natural disaster, or  an information/cyber security incident.
 This process should consider:
@@ -15798,12 +15585,12 @@
 •	Who to call in case of an incident.</t>
         </is>
       </c>
-      <c r="I339" s="18" t="inlineStr">
+      <c r="I335" s="18" t="inlineStr">
         <is>
           <t>Un processus de rétablissement en cas de catastrophes et d'incidents liés à l'information et à la cybersécurité est élaboré et exécuté selon les besoins.</t>
         </is>
       </c>
-      <c r="J339" s="18" t="inlineStr">
+      <c r="J335" s="18" t="inlineStr">
         <is>
           <t>• Il convient qu’un processus soit élaboré pour déterminer les mesures immédiates à prendre en cas d'incendie, d'urgence médicale, de cambriolage, de catastrophe naturelle ou d'incident de sécurité informatique.
 • Il convient que ce processus prenne en compte : 
@@ -15812,12 +15599,12 @@
 	o Qui appeler en cas d'incident.</t>
         </is>
       </c>
-      <c r="L339" s="18" t="inlineStr">
+      <c r="L335" s="18" t="inlineStr">
         <is>
           <t>Er moet een herstelproces voor rampen en informatie-/cyberbeveiligingsincidenten worden ontwikkeld en zo nodig uitgevoerd.+L339</t>
         </is>
       </c>
-      <c r="M339" s="18" t="inlineStr">
+      <c r="M335" s="18" t="inlineStr">
         <is>
           <t>• Er zou een proces moeten worden ontwikkeld voor de onmiddellijke acties in geval van brand, medisch noodgeval, inbraak, natuurramp of een incident op het gebied van informatie-/cyberbeveiliging. 
 • Dit proces zou rekening moeten houden met: 
@@ -15827,120 +15614,283 @@
         </is>
       </c>
     </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>4</v>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>RC.RP-1.2</t>
+        </is>
+      </c>
+      <c r="F336" s="17" t="inlineStr">
+        <is>
+          <t>The essential organization’s functions and services shall be continued with little or no loss of operational continuity and continuity shall be sustained until full system restoration.</t>
+        </is>
+      </c>
+      <c r="G336" s="17" t="inlineStr">
+        <is>
+          <t>No additional guidance on this topic.</t>
+        </is>
+      </c>
+      <c r="I336" s="18" t="inlineStr">
+        <is>
+          <t>Les fonctions et services de l'organisation essentielle doivent être poursuivis avec peu ou pas de perte de continuité opérationnelle et la continuité doit être maintenue jusqu'à la restauration complète du système.</t>
+        </is>
+      </c>
+      <c r="J336" s="18" t="inlineStr">
+        <is>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+        </is>
+      </c>
+      <c r="L336" s="18" t="inlineStr">
+        <is>
+          <t>De essentiële functies en diensten van de organisatie moeten worden voortgezet met weinig of geen verlies van operationele continuïteit en de continuïteit moet worden gehandhaafd totdat het systeem volledig is hersteld.</t>
+        </is>
+      </c>
+      <c r="M336" s="18" t="inlineStr">
+        <is>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="57.6" customHeight="1">
+      <c r="B337" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D337" s="8" t="inlineStr">
+        <is>
+          <t>RC.IM</t>
+        </is>
+      </c>
+      <c r="E337" s="8" t="inlineStr">
+        <is>
+          <t>Improvements</t>
+        </is>
+      </c>
+      <c r="F337" s="9" t="inlineStr">
+        <is>
+          <t>Recovery planning and processes are improved by incorporating lessons learned into future activities.</t>
+        </is>
+      </c>
+      <c r="H337" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Améliorations </t>
+        </is>
+      </c>
+      <c r="I337" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K337" s="11" t="inlineStr">
+        <is>
+          <t>Verbeteringen</t>
+        </is>
+      </c>
+      <c r="L337" s="12" t="inlineStr">
+        <is>
+          <t>De herstelplanning en -processen worden verbeterd door in toekomstige activiteiten rekening te houden met de opgedane ervaring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="28.8" customHeight="1">
+      <c r="B338" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D338" s="13" t="inlineStr">
+        <is>
+          <t>RC.IM-1</t>
+        </is>
+      </c>
+      <c r="F338" s="14" t="inlineStr">
+        <is>
+          <t>Recovery plans incorporate lessons learned</t>
+        </is>
+      </c>
+      <c r="I338" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de rétablissement intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L338" s="16" t="inlineStr">
+        <is>
+          <t>In de herstelplannen zijn de geleerde lessen verwerkt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="244.8" customHeight="1">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>4</v>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RC.IM-1.1</t>
+        </is>
+      </c>
+      <c r="F339" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall incorporate lessons learned from incident recovery activities into updated or new system recovery procedures and, after testing, frame this with appropriate training.</t>
+        </is>
+      </c>
+      <c r="G339" s="17" t="inlineStr">
+        <is>
+          <t>No additional guidance on this topic.</t>
+        </is>
+      </c>
+      <c r="I339" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit intégrer les enseignements tirés des activités de rétablissement des incidents dans les procédures de rétablissement du système, nouvelles ou mises à jour, et, après les avoir testées, les encadrer par une formation appropriée.</t>
+        </is>
+      </c>
+      <c r="J339" s="18" t="inlineStr">
+        <is>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+        </is>
+      </c>
+      <c r="L339" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de lessen die zijn getrokken uit herstelactiviteiten bij incidenten verwerken in bijgewerkte of nieuwe herstelprocedures voor systemen en dit, na het testen, borgen met een passende opleiding.</t>
+        </is>
+      </c>
+      <c r="M339" s="18" t="inlineStr">
+        <is>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
+        </is>
+      </c>
+    </row>
     <row r="340" ht="72" customHeight="1">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B340" t="n">
-        <v>4</v>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>RC.RP-1.2</t>
-        </is>
-      </c>
-      <c r="F340" s="17" t="inlineStr">
-        <is>
-          <t>The essential organization’s functions and services shall be continued with little or no loss of operational continuity and continuity shall be sustained until full system restoration.</t>
-        </is>
-      </c>
-      <c r="G340" s="17" t="inlineStr">
-        <is>
-          <t>No additional guidance on this topic.</t>
-        </is>
-      </c>
-      <c r="I340" s="18" t="inlineStr">
-        <is>
-          <t>Les fonctions et services de l'organisation essentielle doivent être poursuivis avec peu ou pas de perte de continuité opérationnelle et la continuité doit être maintenue jusqu'à la restauration complète du système.</t>
-        </is>
-      </c>
-      <c r="J340" s="18" t="inlineStr">
-        <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
-        </is>
-      </c>
-      <c r="L340" s="18" t="inlineStr">
-        <is>
-          <t>De essentiële functies en diensten van de organisatie moeten worden voortgezet met weinig of geen verlies van operationele continuïteit en de continuïteit moet worden gehandhaafd totdat het systeem volledig is hersteld.</t>
-        </is>
-      </c>
-      <c r="M340" s="18" t="inlineStr">
-        <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+      <c r="B340" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D340" s="8" t="inlineStr">
+        <is>
+          <t>RC.CO</t>
+        </is>
+      </c>
+      <c r="E340" s="8" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="F340" s="9" t="inlineStr">
+        <is>
+          <t>Restoration activities are coordinated with internal and external parties (e.g.  coordinating centers, Internet Service Providers, owners of attacking systems, victims, other CSIRTs, and vendors).</t>
+        </is>
+      </c>
+      <c r="H340" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Communications </t>
+        </is>
+      </c>
+      <c r="I340" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K340" s="11" t="inlineStr">
+        <is>
+          <t>Communicatie</t>
+        </is>
+      </c>
+      <c r="L340" s="12" t="inlineStr">
+        <is>
+          <t>Herstelactiviteiten worden gecoördineerd met interne en externe partijen (bv. coördinatiecentra, internetproviders, eigenaars van aanvallende systemen, slachtoffers, andere CSIRT's en verkopers).</t>
         </is>
       </c>
     </row>
     <row r="341" ht="57.6" customHeight="1">
-      <c r="B341" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D341" s="8" t="inlineStr">
-        <is>
-          <t>RC.IM</t>
-        </is>
-      </c>
-      <c r="E341" s="8" t="inlineStr">
-        <is>
-          <t>Improvements</t>
-        </is>
-      </c>
-      <c r="F341" s="9" t="inlineStr">
-        <is>
-          <t>Recovery planning and processes are improved by incorporating lessons learned into future activities.</t>
-        </is>
-      </c>
-      <c r="H341" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Améliorations </t>
-        </is>
-      </c>
-      <c r="I341" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J341" t="inlineStr"/>
-      <c r="K341" s="11" t="inlineStr">
-        <is>
-          <t>Verbeteringen</t>
-        </is>
-      </c>
-      <c r="L341" s="12" t="inlineStr">
-        <is>
-          <t>De herstelplanning en -processen worden verbeterd door in toekomstige activiteiten rekening te houden met de opgedane ervaring.</t>
+      <c r="B341" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D341" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-1</t>
+        </is>
+      </c>
+      <c r="F341" s="14" t="inlineStr">
+        <is>
+          <t>Public relations are managed</t>
+        </is>
+      </c>
+      <c r="I341" s="15" t="inlineStr">
+        <is>
+          <t>Les relations publiques sont gérées.</t>
+        </is>
+      </c>
+      <c r="L341" s="16" t="inlineStr">
+        <is>
+          <t>De public relations worden beheerd.</t>
         </is>
       </c>
     </row>
     <row r="342" ht="28.8" customHeight="1">
-      <c r="B342" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D342" s="13" t="inlineStr">
-        <is>
-          <t>RC.IM-1</t>
-        </is>
-      </c>
-      <c r="F342" s="14" t="inlineStr">
-        <is>
-          <t>Recovery plans incorporate lessons learned</t>
-        </is>
-      </c>
-      <c r="I342" s="15" t="inlineStr">
-        <is>
-          <t>Les plans de rétablissement intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J342" t="inlineStr"/>
-      <c r="L342" s="16" t="inlineStr">
-        <is>
-          <t>In de herstelplannen zijn de geleerde lessen verwerkt.</t>
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B342" t="n">
+        <v>4</v>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RC.CO-1.1</t>
+        </is>
+      </c>
+      <c r="F342" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall centralize and coordinate how information is disseminated and manage how the organization is presented to the public.</t>
+        </is>
+      </c>
+      <c r="G342" s="17" t="inlineStr">
+        <is>
+          <t>Public relations management may include, for example, managing media interactions, coordinating and logging all requests for interviews, handling and ‘triaging’ phone calls and e-mail requests, matching media requests with appropriate and available internal experts who are ready to be interviewed, screening all of information provided to the media, ensuring personnel are familiar with public relations and privacy policies.</t>
+        </is>
+      </c>
+      <c r="I342" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit centraliser et coordonner la manière dont les informations sont diffusées et gérer la manière dont l'organisation est présentée au public.</t>
+        </is>
+      </c>
+      <c r="J342" s="18" t="inlineStr">
+        <is>
+          <t>La gestion des relations publiques peut comprendre, par exemple, la gestion des interactions avec les médias, la coordination et l'enregistrement de toutes les demandes d'interviews, le traitement et le triage des appels téléphoniques et des demandes par e-mail, la mise en relation des demandes des médias avec les experts internes appropriés et disponibles qui sont prêts à être interviewés, le filtrage de toutes les informations fournies aux médias, l'assurance que le personnel connaît bien les politiques en matière de relations publiques et de confidentialité.</t>
+        </is>
+      </c>
+      <c r="L342" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
+        </is>
+      </c>
+      <c r="M342" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
         </is>
       </c>
     </row>
@@ -15955,159 +15905,143 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>I,E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>IMPORTANT_RC.IM-1.1</t>
+          <t>RC.CO-1.2</t>
         </is>
       </c>
       <c r="F343" s="17" t="inlineStr">
         <is>
-          <t>The organization shall incorporate lessons learned from incident recovery activities into updated or new system recovery procedures and, after testing, frame this with appropriate training.</t>
+          <t>A Public Relations Officer shall be assigned.</t>
         </is>
       </c>
       <c r="G343" s="17" t="inlineStr">
         <is>
-          <t>No additional guidance on this topic.</t>
+          <t>The Public Relations Officer should consider the use of pre-define external contacts 
+(e.g. press, regulators, interest groups).</t>
         </is>
       </c>
       <c r="I343" s="18" t="inlineStr">
         <is>
-          <t>L'organisation doit intégrer les enseignements tirés des activités de rétablissement des incidents dans les procédures de rétablissement du système, nouvelles ou mises à jour, et, après les avoir testées, les encadrer par une formation appropriée.</t>
+          <t>Un responsable des relations publiques est désigné.</t>
         </is>
       </c>
       <c r="J343" s="18" t="inlineStr">
         <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+          <t>Il convient que le responsable des relations publiques envisage l'utilisation de contacts externes prédéfinis (par exemple, la presse, les régulateurs, les groupes d'intérêt).</t>
         </is>
       </c>
       <c r="L343" s="18" t="inlineStr">
         <is>
-          <t>De organisatie moet de lessen die zijn getrokken uit herstelactiviteiten bij incidenten verwerken in bijgewerkte of nieuwe herstelprocedures voor systemen en dit, na het testen, borgen met een passende opleiding.</t>
+          <t>Er moet een Public Relations Officer worden aangesteld.</t>
         </is>
       </c>
       <c r="M343" s="18" t="inlineStr">
         <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+          <t>De Public Relations Officer zou moeten overwegen gebruik te maken van vooraf bepaalde externe contacten (bijv. pers, regelgevers, belangengroepen).</t>
         </is>
       </c>
     </row>
     <row r="344" ht="57.6" customHeight="1">
-      <c r="B344" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D344" s="8" t="inlineStr">
-        <is>
-          <t>RC.CO</t>
-        </is>
-      </c>
-      <c r="E344" s="8" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="F344" s="9" t="inlineStr">
-        <is>
-          <t>Restoration activities are coordinated with internal and external parties (e.g.  coordinating centers, Internet Service Providers, owners of attacking systems, victims, other CSIRTs, and vendors).</t>
-        </is>
-      </c>
-      <c r="H344" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Communications </t>
-        </is>
-      </c>
-      <c r="I344" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J344" t="inlineStr"/>
-      <c r="K344" s="11" t="inlineStr">
-        <is>
-          <t>Communicatie</t>
-        </is>
-      </c>
-      <c r="L344" s="12" t="inlineStr">
-        <is>
-          <t>Herstelactiviteiten worden gecoördineerd met interne en externe partijen (bv. coördinatiecentra, internetproviders, eigenaars van aanvallende systemen, slachtoffers, andere CSIRT's en verkopers).</t>
+      <c r="B344" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D344" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-2</t>
+        </is>
+      </c>
+      <c r="F344" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reputation is repaired after an incident </t>
+        </is>
+      </c>
+      <c r="I344" s="15" t="inlineStr">
+        <is>
+          <t>La réputation est réparée après un incident.</t>
+        </is>
+      </c>
+      <c r="L344" s="16" t="inlineStr">
+        <is>
+          <t>Reputatie wordt hersteld na een incident.</t>
         </is>
       </c>
     </row>
     <row r="345">
-      <c r="B345" s="13" t="n">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>4</v>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>RC.CO-2.1</t>
+        </is>
+      </c>
+      <c r="F345" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall implement a crisis response strategy to protect the organization from the negative consequences of a crisis and help restore its reputation.</t>
+        </is>
+      </c>
+      <c r="G345" s="17" t="inlineStr">
+        <is>
+          <t>Crisis response strategies include, for example, actions to shape attributions of the crisis, change perceptions of the organization in crisis, and reduce the negative effect generated by the crisis.</t>
+        </is>
+      </c>
+      <c r="I345" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre en œuvre une stratégie de réponse aux crises afin de protéger l'organisation des conséquences négatives d'une crise et de contribuer à restaurer sa réputation.</t>
+        </is>
+      </c>
+      <c r="J345" s="18" t="inlineStr">
+        <is>
+          <t>Les stratégies de réponse aux crises comprennent, par exemple, des actions visant à déterminer les attributions de la crise, à modifier les perceptions de l'organisation en crise et à réduire l'effet négatif généré par la crise.</t>
+        </is>
+      </c>
+      <c r="L345" s="18" t="inlineStr">
+        <is>
+          <t>Er moet een crisisbestrijdingsstrategie worden toegepast om de organisatie te beschermen tegen de negatieve gevolgen van een crisis en te helpen haar reputatie te herstellen.</t>
+        </is>
+      </c>
+      <c r="M345" s="18" t="inlineStr">
+        <is>
+          <t>Crisisbestrijdingsstrategieën omvatten bijvoorbeeld maatregelen om de beeldvorming over de crisis vorm te geven, de perceptie van de organisatie in crisis te veranderen, en het negatieve effect dat de crisis teweegbrengt te verminderen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="158.4" customHeight="1">
+      <c r="B346" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D345" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-1</t>
-        </is>
-      </c>
-      <c r="F345" s="14" t="inlineStr">
-        <is>
-          <t>Public relations are managed</t>
-        </is>
-      </c>
-      <c r="I345" s="15" t="inlineStr">
-        <is>
-          <t>Les relations publiques sont gérées.</t>
-        </is>
-      </c>
-      <c r="J345" t="inlineStr"/>
-      <c r="L345" s="16" t="inlineStr">
-        <is>
-          <t>De public relations worden beheerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="346" ht="158.4" customHeight="1">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B346" t="n">
-        <v>4</v>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RC.CO-1.1</t>
-        </is>
-      </c>
-      <c r="F346" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall centralize and coordinate how information is disseminated and manage how the organization is presented to the public.</t>
-        </is>
-      </c>
-      <c r="G346" s="17" t="inlineStr">
-        <is>
-          <t>Public relations management may include, for example, managing media interactions, coordinating and logging all requests for interviews, handling and ‘triaging’ phone calls and e-mail requests, matching media requests with appropriate and available internal experts who are ready to be interviewed, screening all of information provided to the media, ensuring personnel are familiar with public relations and privacy policies.</t>
-        </is>
-      </c>
-      <c r="I346" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit centraliser et coordonner la manière dont les informations sont diffusées et gérer la manière dont l'organisation est présentée au public.</t>
-        </is>
-      </c>
-      <c r="J346" s="18" t="inlineStr">
-        <is>
-          <t>La gestion des relations publiques peut comprendre, par exemple, la gestion des interactions avec les médias, la coordination et l'enregistrement de toutes les demandes d'interviews, le traitement et le triage des appels téléphoniques et des demandes par e-mail, la mise en relation des demandes des médias avec les experts internes appropriés et disponibles qui sont prêts à être interviewés, le filtrage de toutes les informations fournies aux médias, l'assurance que le personnel connaît bien les politiques en matière de relations publiques et de confidentialité.</t>
-        </is>
-      </c>
-      <c r="L346" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
-        </is>
-      </c>
-      <c r="M346" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
+      <c r="D346" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-3</t>
+        </is>
+      </c>
+      <c r="F346" s="14" t="inlineStr">
+        <is>
+          <t>Recovery activities are communicated to internal and external stakeholders as well as executive and management teams</t>
+        </is>
+      </c>
+      <c r="I346" s="15" t="inlineStr">
+        <is>
+          <t>Les activités de rétablissement sont communiquées aux parties prenantes internes et externes, ainsi qu'aux équipes de direction et de gestion.</t>
+        </is>
+      </c>
+      <c r="L346" s="16" t="inlineStr">
+        <is>
+          <t>De herstelactiviteiten worden gecommuniceerd aan interne en externe belanghebbenden en aan directie- en managementteams.</t>
         </is>
       </c>
     </row>
@@ -16122,198 +16056,48 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>I,E</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>RC.CO-1.2</t>
+          <t>IMPORTANT_RC.CO-3.1</t>
         </is>
       </c>
       <c r="F347" s="17" t="inlineStr">
         <is>
-          <t>A Public Relations Officer shall be assigned.</t>
+          <t>The organization shall communicate recovery activities to predefined stakeholders, executive and management teams.</t>
         </is>
       </c>
       <c r="G347" s="17" t="inlineStr">
         <is>
-          <t>The Public Relations Officer should consider the use of pre-define external contacts 
-(e.g. press, regulators, interest groups).</t>
+          <t>Communication of recovery activities to all relevant stakeholders applies only to entities subject to the NIS legislation.</t>
         </is>
       </c>
       <c r="I347" s="18" t="inlineStr">
         <is>
-          <t>Un responsable des relations publiques est désigné.</t>
+          <t>L'organisation doit communiquer les activités de rétablissement aux parties prenantes prédéfinies, aux équipes de direction et de gestion.</t>
         </is>
       </c>
       <c r="J347" s="18" t="inlineStr">
         <is>
-          <t>Il convient que le responsable des relations publiques envisage l'utilisation de contacts externes prédéfinis (par exemple, la presse, les régulateurs, les groupes d'intérêt).</t>
+          <t>La communication des activités de rétablissement à toutes les parties prenantes concernées ne s'applique qu'aux entités soumises à la législation NIS.</t>
         </is>
       </c>
       <c r="L347" s="18" t="inlineStr">
         <is>
-          <t>Er moet een Public Relations Officer worden aangesteld.</t>
+          <t>De organisatie moet de herstelactiviteiten meedelen aan vooraf bepaalde belanghebbenden, directie- en managementteams.</t>
         </is>
       </c>
       <c r="M347" s="18" t="inlineStr">
         <is>
-          <t>De Public Relations Officer zou moeten overwegen gebruik te maken van vooraf bepaalde externe contacten (bijv. pers, regelgevers, belangengroepen).</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="B348" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D348" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-2</t>
-        </is>
-      </c>
-      <c r="F348" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reputation is repaired after an incident </t>
-        </is>
-      </c>
-      <c r="I348" s="15" t="inlineStr">
-        <is>
-          <t>La réputation est réparée après un incident.</t>
-        </is>
-      </c>
-      <c r="J348" t="inlineStr"/>
-      <c r="L348" s="16" t="inlineStr">
-        <is>
-          <t>Reputatie wordt hersteld na een incident.</t>
-        </is>
-      </c>
-    </row>
-    <row r="349" ht="72" customHeight="1">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B349" t="n">
-        <v>4</v>
-      </c>
-      <c r="C349" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D349" t="inlineStr">
-        <is>
-          <t>RC.CO-2.1</t>
-        </is>
-      </c>
-      <c r="F349" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall implement a crisis response strategy to protect the organization from the negative consequences of a crisis and help restore its reputation.</t>
-        </is>
-      </c>
-      <c r="G349" s="17" t="inlineStr">
-        <is>
-          <t>Crisis response strategies include, for example, actions to shape attributions of the crisis, change perceptions of the organization in crisis, and reduce the negative effect generated by the crisis.</t>
-        </is>
-      </c>
-      <c r="I349" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit mettre en œuvre une stratégie de réponse aux crises afin de protéger l'organisation des conséquences négatives d'une crise et de contribuer à restaurer sa réputation.</t>
-        </is>
-      </c>
-      <c r="J349" s="18" t="inlineStr">
-        <is>
-          <t>Les stratégies de réponse aux crises comprennent, par exemple, des actions visant à déterminer les attributions de la crise, à modifier les perceptions de l'organisation en crise et à réduire l'effet négatif généré par la crise.</t>
-        </is>
-      </c>
-      <c r="L349" s="18" t="inlineStr">
-        <is>
-          <t>Er moet een crisisbestrijdingsstrategie worden toegepast om de organisatie te beschermen tegen de negatieve gevolgen van een crisis en te helpen haar reputatie te herstellen.</t>
-        </is>
-      </c>
-      <c r="M349" s="18" t="inlineStr">
-        <is>
-          <t>Crisisbestrijdingsstrategieën omvatten bijvoorbeeld maatregelen om de beeldvorming over de crisis vorm te geven, de perceptie van de organisatie in crisis te veranderen, en het negatieve effect dat de crisis teweegbrengt te verminderen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="350" ht="43.2" customHeight="1">
-      <c r="B350" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D350" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-3</t>
-        </is>
-      </c>
-      <c r="F350" s="14" t="inlineStr">
-        <is>
-          <t>Recovery activities are communicated to internal and external stakeholders as well as executive and management teams</t>
-        </is>
-      </c>
-      <c r="I350" s="15" t="inlineStr">
-        <is>
-          <t>Les activités de rétablissement sont communiquées aux parties prenantes internes et externes, ainsi qu'aux équipes de direction et de gestion.</t>
-        </is>
-      </c>
-      <c r="J350" t="inlineStr"/>
-      <c r="L350" s="16" t="inlineStr">
-        <is>
-          <t>De herstelactiviteiten worden gecommuniceerd aan interne en externe belanghebbenden en aan directie- en managementteams.</t>
-        </is>
-      </c>
-    </row>
-    <row r="351" ht="57.6" customHeight="1">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B351" t="n">
-        <v>4</v>
-      </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D351" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RC.CO-3.1</t>
-        </is>
-      </c>
-      <c r="F351" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall communicate recovery activities to predefined stakeholders, executive and management teams.</t>
-        </is>
-      </c>
-      <c r="G351" s="17" t="inlineStr">
-        <is>
-          <t>Communication of recovery activities to all relevant stakeholders applies only to entities subject to the NIS legislation.</t>
-        </is>
-      </c>
-      <c r="I351" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit communiquer les activités de rétablissement aux parties prenantes prédéfinies, aux équipes de direction et de gestion.</t>
-        </is>
-      </c>
-      <c r="J351" s="18" t="inlineStr">
-        <is>
-          <t>La communication des activités de rétablissement à toutes les parties prenantes concernées ne s'applique qu'aux entités soumises à la législation NIS.</t>
-        </is>
-      </c>
-      <c r="L351" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de herstelactiviteiten meedelen aan vooraf bepaalde belanghebbenden, directie- en managementteams.</t>
-        </is>
-      </c>
-      <c r="M351" s="18" t="inlineStr">
-        <is>
           <t>Communicatie van herstelactiviteiten aan belanghebbenden geldt alleen voor entiteiten die onder de NIS- wetgeving vallen.</t>
         </is>
       </c>
     </row>
+    <row r="349" ht="72" customHeight="1"/>
+    <row r="350" ht="43.2" customHeight="1"/>
+    <row r="351" ht="57.6" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
replace Folder.viewable_from_descendants with Folder.default_role
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
+++ b/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="cff_meta" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="cff_content" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="implementation_groups_meta" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="implementation_groups_content" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="library_meta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cff_meta" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cff_content" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_meta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scores_content" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="implementation_groups_meta" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="implementation_groups_content" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -124,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -201,6 +203,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,7 +604,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -611,10 +614,8 @@
           <t>publication_date</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2025-06-18 00:00:00</t>
-        </is>
+      <c r="B4" s="30" t="n">
+        <v>46255</v>
       </c>
     </row>
     <row r="5">
@@ -948,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M351"/>
+  <dimension ref="A1:M347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1052,8 +1053,6 @@
           <t>IDENTIFIER (ID)</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" s="7" t="inlineStr">
         <is>
           <t>IDENTIFICEREN (ID)</t>
@@ -1089,7 +1088,6 @@
           <t>Les données, le personnel, les dispositifs, les systèmes et les installations qui permettent à l'organisation d'atteindre ses objectifs opérationnels sont identifiés et gérés en fonction de leur importance relative par rapport aux objectifs de l'organisation et à sa stratégie en matière de risques.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" s="11" t="inlineStr">
         <is>
           <t>Vermogensbeheer</t>
@@ -1120,7 +1118,6 @@
           <t>Les dispositifs et systèmes physiques utilisés dans l'organisation sont inventoriés.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="L4" s="16" t="inlineStr">
         <is>
           <t>Inventarisatie van de binnen de organisatie gebruikte fysieke apparaten en systemen.</t>
@@ -1364,7 +1361,6 @@
           <t>Les plateformes et applications logicielles utilisées au sein de l'organisation sont inventoriées.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="L9" s="16" t="inlineStr">
         <is>
           <t>Inventarisatie van de binnen de organisatie gebruikte softwareplatforms en - toepassingen.</t>
@@ -1658,7 +1654,6 @@
           <t>La communication organisationnelle et les flux de données sont schématisés.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="L15" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve"> De organisatorische communicatie- en gegevensstromen worden in kaart gebracht.</t>
@@ -1858,7 +1853,6 @@
           <t xml:space="preserve"> Les systèmes d'information externes sont catalogués.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="L19" s="16" t="inlineStr">
         <is>
           <t>Externe informatiesystemen worden gecatalogiseerd.</t>
@@ -1990,7 +1984,6 @@
           <t>Les ressources sont organisées par ordre de priorité en fonction de leur classification, de leur criticité et de leur valeur opérationnelle.</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="L22" s="16" t="inlineStr">
         <is>
           <t>Middelen worden geprioriteerd op basis van hun classificatie, kriticiteit en bedrijfswaarde.</t>
@@ -2099,7 +2092,6 @@
           <t>Les rôles, responsabilités et pouvoirs en matière de cybersécurité pour l'ensemble du personnel et les parties prenantes tierces (par exemple, les fournisseurs, les clients, les partenaires) sont établis.</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
       <c r="L24" s="16" t="inlineStr">
         <is>
           <t>Rollen, verantwoordelijkheden en bevoegdheden op het gebied van informatie- en cyberbeveiliging worden vastgesteld voor het gehele personeel en belanghebbenden van derden.</t>
@@ -2244,7 +2236,6 @@
           <t>La mission, les objectifs, les parties prenantes et les activités de l'organisation sont compris et classés par ordre de priorité ; ces informations sont utilisées pour définir les rôles, les responsabilités et les décisions en matière de gestion des risques liés à la cybersécurité.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" s="11" t="inlineStr">
         <is>
           <t>Bedrijfsomgeving</t>
@@ -2275,7 +2266,6 @@
           <t>Le rôle de l'organisation dans la chaîne d'approvisionnement est identifié et communiqué.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="L28" s="16" t="inlineStr">
         <is>
           <t>De rol van de organisatie in de toeleveringsketen wordt vastgesteld en gecommuniceerd.</t>
@@ -2403,7 +2393,6 @@
           <t>La place de l'organisation dans les infrastructures critiques et son secteur d'activité est identifiée et communiquée.</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="L31" s="16" t="inlineStr">
         <is>
           <t>De plaats van de organisatie in de kritieke infrastructuur en haar bedrijfstak wordt vastgesteld en gecommuniceerd.</t>
@@ -2554,7 +2543,6 @@
           <t>Les dépendances et les fonctions critiques pour la prestation des services critiques sont établies.</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="L35" s="16" t="inlineStr">
         <is>
           <t>Afhankelijkheden en kritieke functies voor de levering van kritieke diensten zijn vastgesteld.</t>
@@ -2630,7 +2618,6 @@
           <t>Les exigences en matière de résilience pour soutenir la prestation de services essentiels sont établies pour tous les états de fonctionnement (par exemple, en cas de contrainte/attaque, pendant le rétablissement, les opérations normales).</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="L37" s="16" t="inlineStr">
         <is>
           <t>Voor alle operationele staten (bv. onder dwang/aanval, tijdens herstel, normale operaties) worden vereisten vastgesteld met betrekking tot weerbaarheid ter ondersteuning van de levering van kritieke diensten.</t>
@@ -2824,7 +2811,6 @@
           <t>Les politiques, procédures et processus de gestion et de suivi des exigences réglementaires, juridiques, environnementales et opérationnelles de l'organisation sont compris et contribuent à la gestion du risque de cybersécurité.</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" s="11" t="inlineStr">
         <is>
           <t>Bestuur</t>
@@ -2855,7 +2841,6 @@
           <t>La politique de cybersécurité de l'organisation est établie et communiquée .</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
       <c r="L42" s="16" t="inlineStr">
         <is>
           <t>Het cyberbeveiligingsbeleid van de organisatie wordt vastgesteld en gecommuniceerd.</t>
@@ -2995,7 +2980,6 @@
           <t>Les exigences légales et réglementaires concernant la cybersécurité, y compris les obligations en matière de vie privée et de libertés civiles, sont comprises et gérées .</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
       <c r="L45" s="16" t="inlineStr">
         <is>
           <t>Wettelijke en regelgevende voorschriften inzake cyberbeveiliging, met inbegrip van verplichtingen inzake privacy en burgerlijke vrijheden, worden begrepen en beheerd.</t>
@@ -3124,7 +3108,6 @@
           <t>Les processus de gouvernance et de gestion des risques traitent les risques de cybersécurité .</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
       <c r="L48" s="16" t="inlineStr">
         <is>
           <t>Governance- en risicobeheerprocessen adresseren risico's met betrekking tot cyberbeveiliging.</t>
@@ -3260,7 +3243,6 @@
           <t>L'organisation comprend le risque de cybersécurité pour les opérations de l'organisation (y compris la mission, les fonctions, l'image ou la réputation), ses actifs et les individus.</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" s="11" t="inlineStr">
         <is>
           <t>Risicobeoordeling</t>
@@ -3291,7 +3273,6 @@
           <t xml:space="preserve"> Les vulnérabilités des actifs sont identifiées et documentées.</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
       <c r="L52" s="16" t="inlineStr">
         <is>
           <t>Kwetsbaarheden van activa worden vastgesteld en gedocumenteerd.</t>
@@ -3475,7 +3456,6 @@
           <t>Les renseignements sur les cybermenaces sont reçus de forums de partage d'informations et de sources.</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
       <c r="L56" s="16" t="inlineStr">
         <is>
           <t>Informatie over cyberdreigingen wordt ontvangen van fora en bronnen voor informatie-uitwisseling.</t>
@@ -3601,7 +3581,6 @@
           <t>Les menaces, les vulnérabilités, les probabilités et les impacts sont utilisés pour déterminer les risques.</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
       <c r="L59" s="16" t="inlineStr">
         <is>
           <t>Bedreigingen, kwetsbaarheden, waarschijnlijkheden en gevolgen worden gebruikt om het risico te bepalen.</t>
@@ -3784,7 +3763,6 @@
           <t>Les réponses aux risques sont identifiées et classées par ordre de priorité.</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
       <c r="L63" s="16" t="inlineStr">
         <is>
           <t>Respons op risico’s worden vastgesteld en geprioriteerd.</t>
@@ -3879,7 +3857,6 @@
           <t>Les priorités, contraintes, tolérances au risque et hypothèses de l'organisation sont établies et utilisées pour soutenir les décisions relatives au risque opérationnel.</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
       <c r="K65" s="11" t="inlineStr">
         <is>
           <t>Risicobeheer</t>
@@ -3910,7 +3887,6 @@
           <t>Les processus de gestion des risques sont établis, gérés et acceptés par les parties prenantes de l’organisation.</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
       <c r="L66" s="16" t="inlineStr">
         <is>
           <t>Risicobeheerprocessen worden vastgesteld, beheerd en goedgekeurd door belanghebbenden in de organisatie.</t>
@@ -3986,7 +3962,6 @@
           <t>La tolérance de l'organisation au risque est déterminée et clairement exprimée.</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
       <c r="L68" s="16" t="inlineStr">
         <is>
           <t>De risicotolerantie van de organisatie wordt bepaald en duidelijk uitgedrukt.</t>
@@ -4062,7 +4037,6 @@
           <t>La détermination de la tolérance au risque de l'organisation est éclairée par son rôle dans l'infrastructure critique et l'analyse des risques spécifiques au secteur.</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
       <c r="L70" s="16" t="inlineStr">
         <is>
           <t>De organisatie bepaalt haar risicotolerantie op basis van haar rol in de analyse van kritieke infrastructuur en sectorspecifieke risico's.</t>
@@ -4148,7 +4122,6 @@
           <t>Les priorités, les contraintes, les tolérances au risque et les hypothèses de l'organisation sont établies et utilisées pour soutenir les décisions liées à la gestion des risques de la chaîne d'approvisionnement. L'organisation a établi et mis en œuvre les processus pour identifier, évaluer et gérer les risques liés à la chaîne d'approvisionnement.</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
       <c r="K72" s="11" t="inlineStr">
         <is>
           <t>Risicobeheer van de toeleveringsketen</t>
@@ -4179,7 +4152,6 @@
           <t>Les processus de gestion des risques liés à la chaîne d'approvisionnement sont identifiés, établis, évalués, gérés et acceptés par les parties prenantes de l'organisation.</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
       <c r="L73" s="16" t="inlineStr">
         <is>
           <t>De processen voor het beheer van cyberrisico's in de toeleveringsketen worden geïdentificeerd, vastgesteld, beoordeeld, beheerd en goedgekeurd door de belanghebbenden van de organisatie.</t>
@@ -4255,7 +4227,6 @@
           <t>Les fournisseurs et les partenaires tiers de systèmes d'information, de composants et de services sont identifiés, classés par ordre de priorité et évalués à l'aide d'un processus d'évaluation des risques de la cyberchaîne d’approvisionnement.</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
       <c r="L75" s="16" t="inlineStr">
         <is>
           <t>Leveranciers en externe partners van informatiesystemen, componenten en diensten worden geïdentificeerd, geprioriteerd en beoordeeld met behulp van een risicobeoordelingsproces voor de cybertoeleveringsketen.</t>
@@ -4381,7 +4352,6 @@
           <t>Les contrats avec les fournisseurs et les partenaires tiers sont utilisés pour mettre en œuvre des mesures appropriées conçues pour atteindre les objectifs du programme de cybersécurité et du plan de gestion des risques de la chaîne d'approvisionnement de l'organisation.</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
       <c r="L78" s="16" t="inlineStr">
         <is>
           <t>Contracten met leveranciers en externe partners worden gebruikt om passende maatregelen te implementeren, die dermate zijn ontworpen opdat wordt beantwoord aan de doelstellingen van het cyberbeveiligingsprogramma van de organisatie en haar cyber risicobeheersplan voor de toeleveringsketen.</t>
@@ -4563,7 +4533,6 @@
           <t>Les fournisseurs et les partenaires tiers sont régulièrement évalués à l'aide d'audits, de résultats de tests ou d'autres formes d'évaluation pour confirmer qu'ils respectent leurs obligations contractuelles.</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
       <c r="L82" s="16" t="inlineStr">
         <is>
           <t>Leveranciers en externe partners worden routinematig beoordeeld aan de hand van audits, testresultaten of andere vormen van evaluaties om te bevestigen dat zij aan hun contractuele verplichtingen voldoen.</t>
@@ -4689,7 +4658,6 @@
           <t>La planification et les tests de réponse et de rétablissement sont effectués avec les fournisseurs et les prestataires tiers.</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
       <c r="L85" s="16" t="inlineStr">
         <is>
           <t>Respons- en herstelplanning en tests worden uitgevoerd met leveranciers en derde partijen.</t>
@@ -4815,7 +4783,6 @@
           <t>PROTEGER (PR)</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
       <c r="K88" s="7" t="inlineStr">
         <is>
           <t>BESCHERMEN (PR)</t>
@@ -4851,7 +4818,6 @@
           <t>L'accès aux actifs physiques et logiques et aux installations associées est limité aux utilisateurs, processus et dispositifs autorisés, et est géré en fonction du risque évalué d'accès non autorisé aux activités et transactions autorisées.</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" s="11" t="inlineStr">
         <is>
           <t>Identiteitsbeheer, authenticatie en toegangscontrole</t>
@@ -4882,7 +4848,6 @@
           <t>Les identités et les identifiants sont émis, gérés, vérifiés, révoqués et audités pour les dispositifs, utilisateurs et processus autorisés.</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
       <c r="L90" s="16" t="inlineStr">
         <is>
           <t>Identiteiten en referenties (“credentials”) worden afgegeven, beheerd, geverifieerd, ingetrokken en gecontroleerd voor geautoriseerde apparaten, gebruikers en processen.</t>
@@ -5194,7 +5159,6 @@
           <t>L'accès physique aux actifs est géré et protégé.</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
       <c r="L96" s="16" t="inlineStr">
         <is>
           <t>De fysieke toegang tot activa wordt beheerd en beschermd.</t>
@@ -5449,7 +5413,6 @@
           <t>L'accès à distance est géré.</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
       <c r="L101" s="16" t="inlineStr">
         <is>
           <t>De toegang op afstand wordt beheerd.</t>
@@ -5755,7 +5718,6 @@
           <t>Les permissions et autorisations d'accès sont gérées en intégrant les principes du moindre privilège et de la séparation des tâches.</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
       <c r="L107" s="16" t="inlineStr">
         <is>
           <t>De toegangsrechten en machtigingen worden beheerd, met inachtneming van de beginselen van "least privilege" en scheiding van taken.</t>
@@ -6283,7 +6245,6 @@
           <t>L'intégrité du réseau (séparation du réseau, segmentation du réseau...) est protégée.</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
       <c r="L117" s="16" t="inlineStr">
         <is>
           <t>Netwerkintegriteit (netwerksegregatie, netwerksegmentatie...) wordt beschermd.</t>
@@ -6654,7 +6615,6 @@
           <t>Les identités sont prouvées et liées aux identifiants et présentées dans les interactions.</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
       <c r="L124" s="16" t="inlineStr">
         <is>
           <t>Identiteiten worden aangetoond en verbonden aan referenties (“credentials”) en bevestigd in interacties.</t>
@@ -6780,7 +6740,6 @@
           <t>Les utilisateurs, les appareils et les autres actifs sont authentifiés (par exemple, à un seul facteur, à plusieurs facteurs) en fonction du risque de la transaction (par exemple, les risques pour la sécurité et la confidentialité des individus et d’autres risques organisationnels)</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr"/>
       <c r="L127" s="16" t="inlineStr">
         <is>
           <t>Identiteiten worden aangetoond en verbonden aan referenties (“credentials”) en bevestigd in interacties.</t>
@@ -6866,7 +6825,6 @@
           <t>Le personnel et les partenaires de l'organisation reçoivent une formation de sensibilisation à la cybersécurité et sont formés à l'exécution de leurs tâches et responsabilités liées à la cybersécurité, conformément aux politiques, procédures et accords connexes.</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr"/>
       <c r="K129" s="11" t="inlineStr">
         <is>
           <t>Bewustmaking en opleiding</t>
@@ -6897,7 +6855,6 @@
           <t>Tous les utilisateurs sont informés et entrainés.</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr"/>
       <c r="L130" s="16" t="inlineStr">
         <is>
           <t>Alle gebruikers worden geïnformeerd en opgeleid.</t>
@@ -7091,7 +7048,6 @@
           <t xml:space="preserve"> Les utilisateurs privilégiés comprennent leurs rôles et leurs responsabilités.</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr"/>
       <c r="L134" s="16" t="inlineStr">
         <is>
           <t>Geprivilegieerde gebruikers begrijpen hun rollen en verantwoordelijkheden.</t>
@@ -7167,7 +7123,6 @@
           <t>Les parties prenantes tierces (par exemple, les fournisseurs, les clients, les partenaires) comprennent leurs rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
       <c r="L136" s="16" t="inlineStr">
         <is>
           <t>Belanghebbenden van derden (bijv. leveranciers, klanten, partners) begrijpen hun rol en verantwoordelijkheden.</t>
@@ -7393,7 +7348,6 @@
           <t>Les cadres supérieurs comprennent leurs rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
       <c r="L141" s="16" t="inlineStr">
         <is>
           <t>Hogere leidinggevenden begrijpen hun taken en verantwoordelijkheden.</t>
@@ -7469,7 +7423,6 @@
           <t>Le personnel de la sécurité physique et de la cybersécurité comprend ses rôles et responsabilités.</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr"/>
       <c r="L143" s="16" t="inlineStr">
         <is>
           <t>Fysiek en cyberbeveiligingspersoneel begrijpt hun rollen en verantwoordelijkheden.</t>
@@ -7555,7 +7508,6 @@
           <t>Les informations et les enregistrements (données) sont gérés conformément à la stratégie de l'organisation en matière de risques afin de protéger la confidentialité, l'intégrité et la disponibilité des informations.</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
       <c r="K145" s="12" t="inlineStr">
         <is>
           <t>Gegevensbeveiliging</t>
@@ -7586,7 +7538,6 @@
           <t>Les données au repos sont protégées.</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
       <c r="L146" s="15" t="inlineStr">
         <is>
           <t>Data in rust is beschermd.</t>
@@ -7674,7 +7625,6 @@
           <t>Les données en transit sont protégées.</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
       <c r="L148" s="16" t="inlineStr">
         <is>
           <t>Data-in-transitie is beschermd.</t>
@@ -7751,7 +7701,6 @@
           <t>Les actifs sont gérés de manière formelle tout au long de leur retrait, de leur transfert et de leur mise à disposition.</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
       <c r="L150" s="16" t="inlineStr">
         <is>
           <t>Activa worden formeel beheerd gedurende de verhuizing, overdracht en verwijdering.</t>
@@ -7986,7 +7935,6 @@
           <t>Une capacité adéquate pour assurer la disponibilité est maintenue.</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
       <c r="L155" s="16" t="inlineStr">
         <is>
           <t>Voldoende capaciteit om de beschikbaarheid te waarborgen.</t>
@@ -8162,7 +8110,6 @@
           <t>Les protections contre les fuites de données sont mises en œuvre.</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
       <c r="L159" s="16" t="inlineStr">
         <is>
           <t>Beveiligingen tegen datalekken worden geïmplementeerd.</t>
@@ -8241,7 +8188,6 @@
           <t>Des mécanismes de vérification de l'intégrité sont utilisés pour vérifier l'intégrité des logiciels, des microprogrammes et des informations.</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr"/>
       <c r="L161" s="16" t="inlineStr">
         <is>
           <t>Integriteitscontrolemechanismen worden gebruikt om de integriteit van software, firmware en informatie te controleren.</t>
@@ -8417,7 +8363,6 @@
           <t>L'environnement ou les environnements de développement et de test sont séparés de l'environnement de production.</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr"/>
       <c r="L165" s="16" t="inlineStr">
         <is>
           <t>De ontwikkelings- en testomgeving(en) zijn gescheiden van de productieomgeving.</t>
@@ -8497,7 +8442,6 @@
           <t>Les mécanismes de contrôle d'intégrité sont utilisés pour vérifier l'intégrité du matériel.</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr"/>
       <c r="L167" s="16" t="inlineStr">
         <is>
           <t>Integriteitscontrolemechanismen worden gebruikt om de integriteit van de hardware te verifiëren.</t>
@@ -8633,7 +8577,6 @@
           <t>Les politiques de sécurité (qui traitent de l'objectif, de la portée, des rôles, des responsabilités, de l'engagement de la direction et de la coordination entre les entités organisationnelles), les processus et les procédures sont maintenus et utilisés pour gérer la protection des systèmes d'information et des actifs.</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr"/>
       <c r="K170" s="11" t="inlineStr">
         <is>
           <t>Informatiebeschermingsprocessen en - procedures</t>
@@ -8664,7 +8607,6 @@
           <t>Une configuration de base des systèmes de contrôle des technologies de l'information/de l'industrie est créée et maintenue en intégrant les principes de sécurité.</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr"/>
       <c r="L171" s="16" t="inlineStr">
         <is>
           <t>Er wordt een basisconfiguratie van informatietechnologie/industriële controlesystemen gecreëerd en onderhouden, waarin de beveiligingsbeginselen zijn verwerkt .</t>
@@ -8798,7 +8740,6 @@
           <t>Un cycle de vie du développement des systèmes pour gérer les systèmes est mis en œuvre .</t>
         </is>
       </c>
-      <c r="J174" t="inlineStr"/>
       <c r="L174" s="16" t="inlineStr">
         <is>
           <t>Een levenscyclus voor systeemontwikkeling om systemen te beheren wordt geïmplementeerd.</t>
@@ -8942,7 +8883,6 @@
           <t>Des processus de contrôle des changements de configuration sont en place.</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr"/>
       <c r="L177" s="16" t="inlineStr">
         <is>
           <t>Er zijn processen voor het beheer van configuratiewijzigingen aanwezig.</t>
@@ -9068,7 +9008,6 @@
           <t>Des sauvegardes des informations sont effectuées, maintenues et testées .</t>
         </is>
       </c>
-      <c r="J180" t="inlineStr"/>
       <c r="L180" s="16" t="inlineStr">
         <is>
           <t>Er worden back-ups van informatie gemaakt, onderhouden en getest.</t>
@@ -9356,7 +9295,6 @@
           <t>La politique et les règlements concernant l'environnement physique d'exploitation des actifs de l'organisation sont respectés.</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr"/>
       <c r="L186" s="16" t="inlineStr">
         <is>
           <t>Beleid en voorschriften met betrekking tot de fysieke bedrijfsomgeving voor bedrijfsmiddelen van de organisatie worden nageleefd .</t>
@@ -9488,7 +9426,6 @@
           <t>Les données sont détruites conformément à la politique.</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr"/>
       <c r="L189" s="16" t="inlineStr">
         <is>
           <t>Gegevens worden vernietigd overeenkomstig beleid.</t>
@@ -9629,7 +9566,6 @@
           <t>Les processus de protection sont améliorés</t>
         </is>
       </c>
-      <c r="J192" t="inlineStr"/>
       <c r="L192" s="16" t="inlineStr">
         <is>
           <t>De beschermingsprocessen worden verbeterd.</t>
@@ -9808,7 +9744,6 @@
           <t>L'efficacité des technologies de protection est partagée.</t>
         </is>
       </c>
-      <c r="J196" t="inlineStr"/>
       <c r="L196" s="16" t="inlineStr">
         <is>
           <t>De doeltreffendheid van beschermingstechnologieën wordt gedeeld.</t>
@@ -9984,7 +9919,6 @@
           <t>Des plans de réponse (réponse aux incidents et continuité des activités) et des plans de rétablissement (reprise après incident et reprise après sinistre) sont en place et gérés.</t>
         </is>
       </c>
-      <c r="J200" t="inlineStr"/>
       <c r="L200" s="16" t="inlineStr">
         <is>
           <t>Responsplannen (Incident Response en Business Continuity) en herstelplannen (Incident Recovery en Disaster Recovery) zijn aanwezig en worden beheerd.</t>
@@ -10119,7 +10053,6 @@
           <t>La cybersécurité est incluse dans les pratiques de ressources humaines (déprovisionnement, sélection du personnel...).</t>
         </is>
       </c>
-      <c r="J203" t="inlineStr"/>
       <c r="L203" s="16" t="inlineStr">
         <is>
           <t>Cyberbeveiliging is opgenomen in de personeelsbeheer (afbouwen, personeelsscreening...).</t>
@@ -10248,7 +10181,6 @@
           <t>Un plan de gestion des vulnérabilités est élaboré et mis en œuvre.</t>
         </is>
       </c>
-      <c r="J206" t="inlineStr"/>
       <c r="L206" s="16" t="inlineStr">
         <is>
           <t>Een plan voor het beheer van kwetsbaarheden wordt ontwikkeld en uitgevoerd.</t>
@@ -10337,7 +10269,6 @@
           <t>La maintenance et la réparation des composants des systèmes de contrôle et d'information industriels sont effectuées conformément aux politiques et procédures.</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr"/>
       <c r="K208" s="11" t="inlineStr">
         <is>
           <t>Onderhoud</t>
@@ -10368,7 +10299,6 @@
           <t>L'entretien et la réparation des actifs de l'organisation sont effectués et consignés, avec des outils approuvés et contrôlés.</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr"/>
       <c r="L209" s="16" t="inlineStr">
         <is>
           <t>Onderhoud en reparatie van bedrijfsmiddelen van de organisatie worden uitgevoerd en geregistreerd, met goedgekeurde en gecontroleerde gereedschappen.</t>
@@ -10754,7 +10684,6 @@
           <t>La maintenance à distance des actifs de l'organisation est approuvée, consignée et effectuée de manière à empêcher tout accès non autorisé.</t>
         </is>
       </c>
-      <c r="J217" t="inlineStr"/>
       <c r="L217" s="16" t="inlineStr">
         <is>
           <t>Onderhoud op afstand van bedrijfsmiddelen van de organisatie moet worden goedgekeurd, geregistreerd en uitgevoerd op een wijze die ongeoorloofde toegang voorkomt.</t>
@@ -10940,7 +10869,6 @@
           <t>Les solutions de sécurité technique sont gérées de manière à garantir la sécurité et la résilience des systèmes et des actifs, conformément aux politiques, procédures et accords connexes.</t>
         </is>
       </c>
-      <c r="J221" t="inlineStr"/>
       <c r="K221" s="11" t="inlineStr">
         <is>
           <t>Beschermingstechnologie</t>
@@ -10971,7 +10899,6 @@
           <t>Les enregistrements d'audit/logs sont déterminés, documentés, mis en œuvre et révisés conformément à la politique.</t>
         </is>
       </c>
-      <c r="J222" t="inlineStr"/>
       <c r="L222" s="16" t="inlineStr">
         <is>
           <t>Registraties van audits/logs worden vastgesteld, gedocumenteerd, uitgevoerd en herzien overeenkomstig beleid.</t>
@@ -11203,7 +11130,6 @@
           <t>Les supports amovibles sont protégés et leur utilisation est limitée conformément à la politique.</t>
         </is>
       </c>
-      <c r="J227" t="inlineStr"/>
       <c r="L227" s="16" t="inlineStr">
         <is>
           <t>Verwisselbare media worden beschermd en het gebruik ervan wordt beperkt overeenkomstig het beleid.</t>
@@ -11379,7 +11305,6 @@
           <t>Le principe de la moindre fonctionnalité est incorporé en configurant les systèmes de manière à ne fournir que les capacités essentielles.</t>
         </is>
       </c>
-      <c r="J231" t="inlineStr"/>
       <c r="L231" s="16" t="inlineStr">
         <is>
           <t>Het beginsel van minimale functionaliteit wordt toegepast door systemen zo te configureren dat ze alleen essentiële mogelijkheden bieden.</t>
@@ -11555,7 +11480,6 @@
           <t>Les réseaux de communication et de contrôle sont protégés.</t>
         </is>
       </c>
-      <c r="J235" t="inlineStr"/>
       <c r="L235" s="16" t="inlineStr">
         <is>
           <t>Communicatie- en besturingsnetwerken zijn beveiligd.</t>
@@ -11743,7 +11667,6 @@
           <t>DETECTER (DE)</t>
         </is>
       </c>
-      <c r="J239" t="inlineStr"/>
       <c r="K239" s="7" t="inlineStr">
         <is>
           <t>DETECTEREN (DE)</t>
@@ -11774,8 +11697,6 @@
           <t>Anomalies et événements</t>
         </is>
       </c>
-      <c r="I240" t="inlineStr"/>
-      <c r="J240" t="inlineStr"/>
       <c r="K240" s="11" t="inlineStr">
         <is>
           <t>Anomalieën en gebeurtenissen</t>
@@ -11806,7 +11727,6 @@
           <t>Une base de référence des opérations du réseau et des flux de données attendus pour les utilisateurs et les systèmes est établie et gérée.</t>
         </is>
       </c>
-      <c r="J241" t="inlineStr"/>
       <c r="L241" s="16" t="inlineStr">
         <is>
           <t>Een baseline van netwerkoperaties en verwachte gegevensstromen voor gebruikers en systemen wordt vastgesteld en beheerd.</t>
@@ -11891,7 +11811,6 @@
           <t>Les événements détectés sont analysés pour comprendre les cibles et les méthodes d’attaque.</t>
         </is>
       </c>
-      <c r="J243" t="inlineStr"/>
       <c r="L243" s="16" t="inlineStr">
         <is>
           <t>Gedetecteerde events worden geanalyseerd om inzicht te krijgen in aanvalsdoelen en -methoden.</t>
@@ -12017,7 +11936,6 @@
           <t>Les données d'événements sont collectées et corrélées à partir de sources et de capteurs multiples.</t>
         </is>
       </c>
-      <c r="J246" t="inlineStr"/>
       <c r="L246" s="16" t="inlineStr">
         <is>
           <t>Gegevens m.b.t. events worden verzameld en gecorreleerd uit meerdere bronnen en sensoren.</t>
@@ -12197,7 +12115,6 @@
           <t>L'impact des événements est déterminé.</t>
         </is>
       </c>
-      <c r="J250" t="inlineStr"/>
       <c r="L250" s="16" t="inlineStr">
         <is>
           <t>De impact van events wordt bepaald.</t>
@@ -12273,7 +12190,6 @@
           <t>Les seuils d'alerte des incidents sont établis.</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr"/>
       <c r="L252" s="16" t="inlineStr">
         <is>
           <t>Er worden alarmdrempels voor incidenten vastgesteld.</t>
@@ -12409,7 +12325,6 @@
           <t>Le système d'information et les actifs sont surveillés pour identifier les événements de cybersécurité et vérifier l'efficacité des mesures de protection.</t>
         </is>
       </c>
-      <c r="J255" t="inlineStr"/>
       <c r="K255" s="11" t="inlineStr">
         <is>
           <t>Voortdurende bewaking van de beveiliging</t>
@@ -12440,7 +12355,6 @@
           <t>Le réseau est surveillé pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
       <c r="L256" s="16" t="inlineStr">
         <is>
           <t>Het netwerk wordt gemonitord om potentiële cyberbeveiligingsevents op te sporen.</t>
@@ -12637,7 +12551,6 @@
           <t>L'environnement physique est surveillé pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J260" t="inlineStr"/>
       <c r="L260" s="16" t="inlineStr">
         <is>
           <t>De fysieke omgeving wordt bewaakt om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -12763,7 +12676,6 @@
           <t>L'activité du personnel est surveillée pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J263" t="inlineStr"/>
       <c r="L263" s="16" t="inlineStr">
         <is>
           <t>Personeelsactiviteiten worden gemonitord om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -12941,7 +12853,6 @@
           <t>Le code malveillant est détecté.</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr"/>
       <c r="L267" s="16" t="inlineStr">
         <is>
           <t>Kwaadaardige code wordt gedetecteerd.</t>
@@ -13073,7 +12984,6 @@
           <t>Un code mobile non autorisé est détecté.</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr"/>
       <c r="L270" s="16" t="inlineStr">
         <is>
           <t>Ongeoorloofde mobiele code is gedetecteerd.</t>
@@ -13152,7 +13062,6 @@
           <t>L'activité des prestataires de services externes est surveillée pour détecter les événements potentiels de cybersécurité.</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr"/>
       <c r="L272" s="16" t="inlineStr">
         <is>
           <t>De activiteit van externe dienstverleners wordt gemonitord om potentiële cyberbeveiligingsgebeurtenissen op te sporen.</t>
@@ -13278,7 +13187,6 @@
           <t>La surveillance du personnel, des connexions, des dispositifs et des logiciels non autorisés est effectuée.</t>
         </is>
       </c>
-      <c r="J275" t="inlineStr"/>
       <c r="L275" s="16" t="inlineStr">
         <is>
           <t>Monitoring op onbevoegd personeel, verbindingen, apparatuur en software wordt uitgevoerd.</t>
@@ -13410,7 +13318,6 @@
           <t>Les analyses de vulnérabilité sont effectuées.</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr"/>
       <c r="L278" s="16" t="inlineStr">
         <is>
           <t>Kwetsbaarheidsscans worden uitgevoerd.</t>
@@ -13546,7 +13453,6 @@
           <t>Les processus et procédures de détection sont maintenus et testés pour garantir la prise de conscience des événements anormaux.</t>
         </is>
       </c>
-      <c r="J281" t="inlineStr"/>
       <c r="K281" s="11" t="inlineStr">
         <is>
           <t>Opsporingsprocessen</t>
@@ -13577,7 +13483,6 @@
           <t>Les activités de détection sont conformes à toutes les exigences applicables.</t>
         </is>
       </c>
-      <c r="J282" t="inlineStr"/>
       <c r="L282" s="16" t="inlineStr">
         <is>
           <t>Detectie moet gebeuren conform alle toepasselijke eisen.</t>
@@ -13653,7 +13558,6 @@
           <t>Les processus de détection sont testés.</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr"/>
       <c r="L284" s="16" t="inlineStr">
         <is>
           <t>Detectieprocessen worden getest.</t>
@@ -13732,7 +13636,6 @@
           <t>Les informations relatives à la détection des événements sont communiquées.</t>
         </is>
       </c>
-      <c r="J286" t="inlineStr"/>
       <c r="L286" s="16" t="inlineStr">
         <is>
           <t>Informatie over gedetecteerde events wordt gecommuniceerd.</t>
@@ -13808,7 +13711,6 @@
           <t>Les processus de détection sont améliorés en permanence.</t>
         </is>
       </c>
-      <c r="J288" t="inlineStr"/>
       <c r="L288" s="16" t="inlineStr">
         <is>
           <t>De processen voor het detecteren van abnormale events worden voortdurend verbeterd.</t>
@@ -13937,8 +13839,6 @@
           <t>REPONDRE (RS)</t>
         </is>
       </c>
-      <c r="I291" t="inlineStr"/>
-      <c r="J291" t="inlineStr"/>
       <c r="K291" s="7" t="inlineStr">
         <is>
           <t>REAGEREN (RS)</t>
@@ -13974,7 +13874,6 @@
           <t>Les processus et procédures de réponse sont exécutés et maintenus, afin de garantir une réponse aux incidents de cybersécurité détectés.</t>
         </is>
       </c>
-      <c r="J292" t="inlineStr"/>
       <c r="K292" s="11" t="inlineStr">
         <is>
           <t>Responsplanning</t>
@@ -14005,7 +13904,6 @@
           <t xml:space="preserve"> Le plan de réponse est exécuté pendant ou après un incident.</t>
         </is>
       </c>
-      <c r="J293" t="inlineStr"/>
       <c r="L293" s="16" t="inlineStr">
         <is>
           <t>Het responsplan wordt uitgevoerd tijdens of na een incident.</t>
@@ -14097,7 +13995,6 @@
           <t>Les activités de réponse sont coordonnées avec les parties prenantes internes et externes (par exemple, le soutien externe des forces de l'ordre).</t>
         </is>
       </c>
-      <c r="J295" t="inlineStr"/>
       <c r="K295" s="11" t="inlineStr">
         <is>
           <t>Communicatie</t>
@@ -14128,7 +14025,6 @@
           <t>Le personnel connaît ses rôles et l'ordre des opérations lorsqu'une réponse est nécessaire.</t>
         </is>
       </c>
-      <c r="J296" t="inlineStr"/>
       <c r="L296" s="16" t="inlineStr">
         <is>
           <t>Het personeel kent zijn rol en volgorde van handelen wanneer een reactie nodig is.</t>
@@ -14204,7 +14100,6 @@
           <t>Les incidents sont signalés conformément aux critères établis.</t>
         </is>
       </c>
-      <c r="J298" t="inlineStr"/>
       <c r="L298" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden gemeld overeenkomstig de vastgestelde criteria.</t>
@@ -14330,7 +14225,6 @@
           <t>Les informations sont partagées conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J301" t="inlineStr"/>
       <c r="L301" s="16" t="inlineStr">
         <is>
           <t>Informatie wordt gedeeld in overeenstemming met de responsplannen.</t>
@@ -14456,7 +14350,6 @@
           <t>La coordination avec les parties prenantes se fait conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J304" t="inlineStr"/>
       <c r="L304" s="16" t="inlineStr">
         <is>
           <t>Coördinatie met belanghebbenden vindt plaats in overeenstemming met de responsplannen.</t>
@@ -14535,7 +14428,6 @@
           <t>Le partage volontaire d'informations se fait avec des parties prenantes externes afin d'obtenir une meilleure connaissance de la situation en matière de cybersécurité.</t>
         </is>
       </c>
-      <c r="J306" t="inlineStr"/>
       <c r="L306" s="16" t="inlineStr">
         <is>
           <t>Er vindt vrijwillige informatie-uitwisseling plaats met externe belanghebbenden om een breder situationeel bewustzijn over cyberbeveiliging te bereiken.</t>
@@ -14621,7 +14513,6 @@
           <t>Une analyse est effectuée pour garantir une réponse efficace et soutenir les activités de rétablissement.</t>
         </is>
       </c>
-      <c r="J308" t="inlineStr"/>
       <c r="K308" s="11" t="inlineStr">
         <is>
           <t>Analyse</t>
@@ -14652,7 +14543,6 @@
           <t>Les notifications des systèmes de détection sont examinées.</t>
         </is>
       </c>
-      <c r="J309" t="inlineStr"/>
       <c r="L309" s="16" t="inlineStr">
         <is>
           <t>RS.AN-1:  Meldingen van detectiesystemen worden onderzocht.</t>
@@ -14778,7 +14668,6 @@
           <t>L'impact de l'incident est compris.</t>
         </is>
       </c>
-      <c r="J312" t="inlineStr"/>
       <c r="L312" s="16" t="inlineStr">
         <is>
           <t>De gevolgen van het incident worden begrepen.</t>
@@ -14907,7 +14796,6 @@
           <t>L'analyse forensique est réalisée.</t>
         </is>
       </c>
-      <c r="J315" t="inlineStr"/>
       <c r="L315" s="16" t="inlineStr">
         <is>
           <t>Forensisch onderzoek wordt uitgevoerd.</t>
@@ -15033,7 +14921,6 @@
           <t>Les incidents sont classés par catégories conformément aux plans de réponse.</t>
         </is>
       </c>
-      <c r="J318" t="inlineStr"/>
       <c r="L318" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden in categorieën ingedeeld overeenkomstig de responsplannen.</t>
@@ -15114,7 +15001,6 @@
           <t>Des processus sont établis pour recevoir, analyser et répondre aux vulnérabilités divulguées à l'organisation par des sources internes et externes (par exemple, tests internes, bulletins de sécurité ou chercheurs en sécurité).</t>
         </is>
       </c>
-      <c r="J320" t="inlineStr"/>
       <c r="L320" s="16" t="inlineStr">
         <is>
           <t>Er zijn processen vastgesteld voor het ontvangen, analyseren en reageren op kwetsbaarheden die uit interne en externe bronnen (bv. interne tests, beveiligingsbulletins of beveiligingsonderzoekers) aan de organisatie bekend zijn gemaakt.</t>
@@ -15247,10 +15133,9 @@
       </c>
       <c r="I323" s="11" t="inlineStr">
         <is>
-          <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
-        </is>
-      </c>
-      <c r="J323" t="inlineStr"/>
+          <t>Des activités sont menées afin d'empêcher l'extension d'un événement, d'en atténuer les effets et de résoudre l'incident.</t>
+        </is>
+      </c>
       <c r="K323" s="11" t="inlineStr">
         <is>
           <t>Mitigatie</t>
@@ -15281,7 +15166,6 @@
           <t>Les incidents sont contenus.</t>
         </is>
       </c>
-      <c r="J324" t="inlineStr"/>
       <c r="L324" s="16" t="inlineStr">
         <is>
           <t>Incidenten worden beheerst.</t>
@@ -15307,74 +15191,149 @@
           <t>IMPORTANT_RS.MI-1.1</t>
         </is>
       </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>The organization shall implement an incident handling capability for information/cybersecurity incidents on its business critical systems that includes preparation, detection and analysis, containment, eradication, recovery and documented risk acceptance.</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>A documented risk acceptance deals with risks that the organisation assesses as not dangerous to the organisation's business critical systems and where the risk owner formally accepts the risk (related with the risk appetite of the organization)</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre en œuvre une capacité de traitement des incidents de sécurité de l'information/cybersécurité sur ses systèmes essentiels à l'activité, qui comprend la préparation, la détection et l'analyse, le confinement, l'éradication, le rétablissement et l'acceptation documentée des risques.</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>Une acceptation des risques documentée concerne les risques que l'organisation évalue comme non dangereux pour les systèmes critiques de l'organisation et pour lesquels le propriétaire du risque accepte formellement le risque (en relation avec l'appétit de l'organisation pour le risque).</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>De organisatie moet een capaciteit voor het afhandelen van informatie- /cyberbeveiligingsincidenten op haar bedrijfskritische systemen implementeren die de voorbereiding, detectie, analyse, insluiting (“containment”), uitroeiing, herstel en gedocumenteerde risicoaanvaarding omvat.</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>Een gedocumenteerde risicoaanvaarding heeft betrekking op risico's die volgens de organisatie niet gevaarlijk zijn voor de bedrijfskritische systemen van de organisatie en waarbij de eigenaar van het risico het risico formeel aanvaardt (gerelateerd aan de risicobereidheid, ”risk appetite”, van de organisatie).</t>
+        </is>
+      </c>
     </row>
     <row r="326">
-      <c r="B326" s="13" t="n">
+      <c r="B326" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D326" s="8" t="inlineStr">
+        <is>
+          <t>RS.IM</t>
+        </is>
+      </c>
+      <c r="E326" s="8" t="inlineStr">
+        <is>
+          <t>Improvements</t>
+        </is>
+      </c>
+      <c r="F326" s="9" t="inlineStr">
+        <is>
+          <t>Organizational response activities are improved by incorporating lessons learned from current and previous detection/response activities.</t>
+        </is>
+      </c>
+      <c r="H326" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Améliorations </t>
+        </is>
+      </c>
+      <c r="I326" s="11" t="inlineStr">
+        <is>
+          <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
+        </is>
+      </c>
+      <c r="K326" s="11" t="inlineStr">
+        <is>
+          <t>Verbeteringen</t>
+        </is>
+      </c>
+      <c r="L326" s="12" t="inlineStr">
+        <is>
+          <t>De responsactiviteiten van de organisatie worden verbeterd door lessen te trekken uit huidige en eerdere opsporings- en responsactiviteiten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="B327" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D326" s="13" t="inlineStr">
-        <is>
-          <t>RS.MI-2</t>
-        </is>
-      </c>
-      <c r="F326" s="14" t="inlineStr">
-        <is>
-          <t>Incidents are mitigated</t>
-        </is>
-      </c>
-      <c r="I326" s="15" t="inlineStr">
-        <is>
-          <t>Les incidents sont atténués.</t>
-        </is>
-      </c>
-      <c r="L326" s="16" t="inlineStr">
-        <is>
-          <t>Incidenten worden gemitigeerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B327" t="n">
-        <v>4</v>
-      </c>
-      <c r="C327" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D327" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RS.MI-2.1</t>
+      <c r="D327" s="13" t="inlineStr">
+        <is>
+          <t>RS.IM-1</t>
+        </is>
+      </c>
+      <c r="F327" s="14" t="inlineStr">
+        <is>
+          <t>Response plans incorporate lessons learned</t>
+        </is>
+      </c>
+      <c r="I327" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de réponse intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L327" s="16" t="inlineStr">
+        <is>
+          <t>In de responsplannen zijn de geleerde lessen verwerkt.</t>
         </is>
       </c>
     </row>
     <row r="328" ht="43.2" customHeight="1">
-      <c r="B328" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D328" s="13" t="inlineStr">
-        <is>
-          <t>RS.MI-3</t>
-        </is>
-      </c>
-      <c r="F328" s="14" t="inlineStr">
-        <is>
-          <t>Newly identified vulnerabilities are mitigated or documented as accepted risks</t>
-        </is>
-      </c>
-      <c r="I328" s="15" t="inlineStr">
-        <is>
-          <t>Les vulnérabilités nouvellement identifiées sont atténuées ou documentées comme des risques acceptés.</t>
-        </is>
-      </c>
-      <c r="L328" s="16" t="inlineStr">
-        <is>
-          <t>Nieuw vastgestelde kwetsbaarheden worden gemitigeerd of gedocumenteerd als aanvaarde risico's.</t>
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>4</v>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>B,I,E</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>BASIC_RS.IM-1.1</t>
+        </is>
+      </c>
+      <c r="F328" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall conduct post-incident evaluations to analyse lessons learned from incident response and recovery, and consequently improve processes / procedures / technologies to enhance its cyber resilience.</t>
+        </is>
+      </c>
+      <c r="G328" s="17" t="inlineStr">
+        <is>
+          <t>Consider bringing involved people together after each incident and reflect together on ways to improve what happened, how it happened, how we reacted, how it could have gone better, what should be done to prevent it from happening again, etc.</t>
+        </is>
+      </c>
+      <c r="I328" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit effectuer des évaluations post-incident afin d'analyser les enseignements tirés de la réponse à l'incident et du rétablissement, et par conséquent améliorer les processus / procédures / technologies pour renforcer sa cyber-résilience.</t>
+        </is>
+      </c>
+      <c r="J328" s="18" t="inlineStr">
+        <is>
+          <t>Envisagez de réunir les personnes concernées après chaque incident et réfléchissez ensemble aux moyens d'améliorer ce qui s'est passé, comment cela s'est passé, comment nous avons réagi, comment cela aurait pu mieux se passer, ce qui devrait être fait pour éviter que cela ne se reproduise, etc.</t>
+        </is>
+      </c>
+      <c r="L328" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet evaluaties uitvoeren na een incident om lessen te trekken uit de reactie op en het herstel van incidenten, en verbetert vervolgens de processen / procedures / technologieën om haar cyberweerbaarheid te vergroten.</t>
+        </is>
+      </c>
+      <c r="M328" s="18" t="inlineStr">
+        <is>
+          <t>Overweeg na elk incident de betrokkenen samen te brengen en samen na te denken over manieren om te verbeteren wat er is gebeurd, hoe het is gebeurd, hoe er is gereageerd, hoe het beter had kunnen gaan, wat er moet gebeuren om herhaling te voorkomen, enz.</t>
         </is>
       </c>
     </row>
@@ -15394,204 +15353,177 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>IMPORTANT_RS.MI-3.1</t>
+          <t>IMPORTANT_RS.IM-1.2</t>
         </is>
       </c>
       <c r="F329" s="17" t="inlineStr">
         <is>
-          <t>The organization shall implement an incident handling capability for information/cybersecurity incidents on its business critical systems that includes preparation, detection and analysis, containment, eradication, recovery and documented risk acceptance.</t>
+          <t>Lessons learned from incident handling shall be translated into updated or new incident handling procedures that shall be tested, approved and trained.</t>
         </is>
       </c>
       <c r="G329" s="17" t="inlineStr">
         <is>
-          <t>A documented risk acceptance deals with risks that the organisation assesses as not dangerous to the organisation's business critical systems and where the risk owner formally accepts the risk (related with the risk appetite of the organization)</t>
+          <t>No additional guidance on this topic.</t>
         </is>
       </c>
       <c r="I329" s="18" t="inlineStr">
         <is>
-          <t>L'organisation doit mettre en œuvre une capacité de traitement des incidents de sécurité de l'information/cybersécurité sur ses systèmes essentiels à l'activité, qui comprend la préparation, la détection et l'analyse, le confinement, l'éradication, le rétablissement et l'acceptation documentée des risques.</t>
+          <t>Les enseignements tirés du traitement des incidents sont traduits en procédures de traitement des incidents actualisées ou nouvelles qui sont testées, approuvées et enseignées.</t>
         </is>
       </c>
       <c r="J329" s="18" t="inlineStr">
         <is>
-          <t>Une acceptation des risques documentée concerne les risques que l'organisation évalue comme non dangereux pour les systèmes critiques de l'organisation et pour lesquels le propriétaire du risque accepte formellement le risque (en relation avec l'appétit de l'organisation pour le risque).</t>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
         </is>
       </c>
       <c r="L329" s="18" t="inlineStr">
         <is>
-          <t>De organisatie moet een capaciteit voor het afhandelen van informatie- /cyberbeveiligingsincidenten op haar bedrijfskritische systemen implementeren die de voorbereiding, detectie, analyse, insluiting (“containment”), uitroeiing, herstel en gedocumenteerde risicoaanvaarding omvat.</t>
+          <t>De uit de afhandeling van incidenten geleerde lessen moeten worden vertaald in bijgewerkte of nieuwe procedures voor de afhandeling van incidenten, die op hun beurt moeten worden getest, goedgekeurd en getraind.</t>
         </is>
       </c>
       <c r="M329" s="18" t="inlineStr">
         <is>
-          <t>Een gedocumenteerde risicoaanvaarding heeft betrekking op risico's die volgens de organisatie niet gevaarlijk zijn voor de bedrijfskritische systemen van de organisatie en waarbij de eigenaar van het risico het risico formeel aanvaardt (gerelateerd aan de risicobereidheid, ”risk appetite”, van de organisatie).</t>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
         </is>
       </c>
     </row>
     <row r="330" ht="57.6" customHeight="1">
-      <c r="B330" s="8" t="n">
+      <c r="B330" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D330" s="13" t="inlineStr">
+        <is>
+          <t>RS.IM-2</t>
+        </is>
+      </c>
+      <c r="F330" s="14" t="inlineStr">
+        <is>
+          <t>Response and Recovery strategies are updated</t>
+        </is>
+      </c>
+      <c r="I330" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de réponse intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L330" s="16" t="inlineStr">
+        <is>
+          <t>Reactie- en herstelstrategieën worden bijgewerkt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>4</v>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RS.IM-2.1</t>
+        </is>
+      </c>
+      <c r="F331" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall update the response and recovery  plans to address changes in its context.</t>
+        </is>
+      </c>
+      <c r="G331" s="17" t="inlineStr">
+        <is>
+          <t>The organization’s context relates to the organizational structure, its critical systems, attack vectors, new threats, improved technology, environment of operation, problems encountered during plan implementation/execution/testing and lessons learned.</t>
+        </is>
+      </c>
+      <c r="I331" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre à jour les plans de réponse et de rétablissement pour tenir compte des changements survenus dans son contexte.</t>
+        </is>
+      </c>
+      <c r="J331" s="18" t="inlineStr">
+        <is>
+          <t>Le contexte de l'organisation concerne la structure organisationnelle, ses systèmes critiques, les vecteurs d'attaque, les nouvelles menaces, les améliorations technologiques, l'environnement d'exploitation, les problèmes rencontrés lors de la mise en œuvre/exécution/test du plan et les enseignements tirés.</t>
+        </is>
+      </c>
+      <c r="L331" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de reactie- en herstelplannen aanpassen aan veranderingen in haar context.</t>
+        </is>
+      </c>
+      <c r="M331" s="18" t="inlineStr">
+        <is>
+          <t>De context van de organisatie heeft betrekking op de organisatiestructuur, haar kritieke systemen, aanvalsvectoren, nieuwe bedreigingen, verbeterde technologie, de bedrijfsomgeving, problemen die zich hebben voorgedaan tijdens de implementatie/uitvoering/testen van het plan en de lessen die zijn geleerd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="86.40000000000001" customHeight="1">
+      <c r="B332" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D332" s="5" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="E332" s="5" t="inlineStr">
+        <is>
+          <t>RECOVER (RC)</t>
+        </is>
+      </c>
+      <c r="H332" s="5" t="inlineStr">
+        <is>
+          <t>RETABLIR (RC)</t>
+        </is>
+      </c>
+      <c r="K332" s="7" t="inlineStr">
+        <is>
+          <t>HERSTELLEN (RC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="57.6" customHeight="1">
+      <c r="B333" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D330" s="8" t="inlineStr">
-        <is>
-          <t>RS.IM</t>
-        </is>
-      </c>
-      <c r="E330" s="8" t="inlineStr">
-        <is>
-          <t>Improvements</t>
-        </is>
-      </c>
-      <c r="F330" s="9" t="inlineStr">
-        <is>
-          <t>Organizational response activities are improved by incorporating lessons learned from current and previous detection/response activities.</t>
-        </is>
-      </c>
-      <c r="H330" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Améliorations </t>
-        </is>
-      </c>
-      <c r="I330" s="11" t="inlineStr">
-        <is>
-          <t>Les activités de réponse de l'organisation sont améliorées par l'intégration des enseignements tirés des activités de détection/réponse actuelles et précédentes.</t>
-        </is>
-      </c>
-      <c r="J330" t="inlineStr"/>
-      <c r="K330" s="11" t="inlineStr">
-        <is>
-          <t>Verbeteringen</t>
-        </is>
-      </c>
-      <c r="L330" s="12" t="inlineStr">
-        <is>
-          <t>De responsactiviteiten van de organisatie worden verbeterd door lessen te trekken uit huidige en eerdere opsporings- en responsactiviteiten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="331">
-      <c r="B331" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D331" s="13" t="inlineStr">
-        <is>
-          <t>RS.IM-1</t>
-        </is>
-      </c>
-      <c r="F331" s="14" t="inlineStr">
-        <is>
-          <t>Response plans incorporate lessons learned</t>
-        </is>
-      </c>
-      <c r="I331" s="15" t="inlineStr">
-        <is>
-          <t>Les plans de réponse intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J331" t="inlineStr"/>
-      <c r="L331" s="16" t="inlineStr">
-        <is>
-          <t>In de responsplannen zijn de geleerde lessen verwerkt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="332" ht="86.40000000000001" customHeight="1">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B332" t="n">
-        <v>4</v>
-      </c>
-      <c r="C332" t="inlineStr">
-        <is>
-          <t>B,I,E</t>
-        </is>
-      </c>
-      <c r="D332" t="inlineStr">
-        <is>
-          <t>BASIC_RS.IM-1.1</t>
-        </is>
-      </c>
-      <c r="F332" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall conduct post-incident evaluations to analyse lessons learned from incident response and recovery, and consequently improve processes / procedures / technologies to enhance its cyber resilience.</t>
-        </is>
-      </c>
-      <c r="G332" s="17" t="inlineStr">
-        <is>
-          <t>Consider bringing involved people together after each incident and reflect together on ways to improve what happened, how it happened, how we reacted, how it could have gone better, what should be done to prevent it from happening again, etc.</t>
-        </is>
-      </c>
-      <c r="I332" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit effectuer des évaluations post-incident afin d'analyser les enseignements tirés de la réponse à l'incident et du rétablissement, et par conséquent améliorer les processus / procédures / technologies pour renforcer sa cyber-résilience.</t>
-        </is>
-      </c>
-      <c r="J332" s="18" t="inlineStr">
-        <is>
-          <t>Envisagez de réunir les personnes concernées après chaque incident et réfléchissez ensemble aux moyens d'améliorer ce qui s'est passé, comment cela s'est passé, comment nous avons réagi, comment cela aurait pu mieux se passer, ce qui devrait être fait pour éviter que cela ne se reproduise, etc.</t>
-        </is>
-      </c>
-      <c r="L332" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet evaluaties uitvoeren na een incident om lessen te trekken uit de reactie op en het herstel van incidenten, en verbetert vervolgens de processen / procedures / technologieën om haar cyberweerbaarheid te vergroten.</t>
-        </is>
-      </c>
-      <c r="M332" s="18" t="inlineStr">
-        <is>
-          <t>Overweeg na elk incident de betrokkenen samen te brengen en samen na te denken over manieren om te verbeteren wat er is gebeurd, hoe het is gebeurd, hoe er is gereageerd, hoe het beter had kunnen gaan, wat er moet gebeuren om herhaling te voorkomen, enz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="333" ht="57.6" customHeight="1">
-      <c r="A333" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B333" t="n">
-        <v>4</v>
-      </c>
-      <c r="C333" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D333" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RS.IM-1.2</t>
-        </is>
-      </c>
-      <c r="F333" s="17" t="inlineStr">
-        <is>
-          <t>Lessons learned from incident handling shall be translated into updated or new incident handling procedures that shall be tested, approved and trained.</t>
-        </is>
-      </c>
-      <c r="G333" s="17" t="inlineStr">
-        <is>
-          <t>No additional guidance on this topic.</t>
-        </is>
-      </c>
-      <c r="I333" s="18" t="inlineStr">
-        <is>
-          <t>Les enseignements tirés du traitement des incidents sont traduits en procédures de traitement des incidents actualisées ou nouvelles qui sont testées, approuvées et enseignées.</t>
-        </is>
-      </c>
-      <c r="J333" s="18" t="inlineStr">
-        <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
-        </is>
-      </c>
-      <c r="L333" s="18" t="inlineStr">
-        <is>
-          <t>De uit de afhandeling van incidenten geleerde lessen moeten worden vertaald in bijgewerkte of nieuwe procedures voor de afhandeling van incidenten, die op hun beurt moeten worden getest, goedgekeurd en getraind.</t>
-        </is>
-      </c>
-      <c r="M333" s="18" t="inlineStr">
-        <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+      <c r="D333" s="8" t="inlineStr">
+        <is>
+          <t>RC.RP</t>
+        </is>
+      </c>
+      <c r="E333" s="8" t="inlineStr">
+        <is>
+          <t>Recovery Planning</t>
+        </is>
+      </c>
+      <c r="F333" s="9" t="inlineStr">
+        <is>
+          <t>Recovery processes and procedures are executed and maintained to ensure restoration of systems or assets affected by cybersecurity incidents.</t>
+        </is>
+      </c>
+      <c r="H333" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planification du rétablissement </t>
+        </is>
+      </c>
+      <c r="I333" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K333" s="11" t="inlineStr">
+        <is>
+          <t>Herstelplanning</t>
+        </is>
+      </c>
+      <c r="L333" s="12" t="inlineStr">
+        <is>
+          <t>Herstelprocessen en -procedures worden uitgevoerd en gehandhaafd om te zorgen voor herstel van systemen of activa die zijn getroffen door cyberbeveiligingsincidenten.</t>
         </is>
       </c>
     </row>
@@ -15601,23 +15533,22 @@
       </c>
       <c r="D334" s="13" t="inlineStr">
         <is>
-          <t>RS.IM-2</t>
+          <t>RC.RP-1</t>
         </is>
       </c>
       <c r="F334" s="14" t="inlineStr">
         <is>
-          <t>Response and Recovery strategies are updated</t>
+          <t xml:space="preserve">Recovery plan is executed during or after a cybersecurity incident </t>
         </is>
       </c>
       <c r="I334" s="15" t="inlineStr">
         <is>
-          <t>Les plans de réponse intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J334" t="inlineStr"/>
+          <t xml:space="preserve"> Le plan de reprise est exécuté pendant ou après un incident de cybersécurité.</t>
+        </is>
+      </c>
       <c r="L334" s="16" t="inlineStr">
         <is>
-          <t>Reactie- en herstelstrategieën worden bijgewerkt.</t>
+          <t>Het herstelplan wordt uitgevoerd tijdens of na een cyberbeveiligingsincident.</t>
         </is>
       </c>
     </row>
@@ -15632,164 +15563,20 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>I,E</t>
+          <t>B,I,E</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>IMPORTANT_RS.IM-2.1</t>
+          <t>BASIC_RC.RP-1.1</t>
         </is>
       </c>
       <c r="F335" s="17" t="inlineStr">
         <is>
-          <t>The organization shall update the response and recovery  plans to address changes in its context.</t>
+          <t>A recovery process for disasters and information/cybersecurity incidents shall be developed and executed as appropriate.</t>
         </is>
       </c>
       <c r="G335" s="17" t="inlineStr">
-        <is>
-          <t>The organization’s context relates to the organizational structure, its critical systems, attack vectors, new threats, improved technology, environment of operation, problems encountered during plan implementation/execution/testing and lessons learned.</t>
-        </is>
-      </c>
-      <c r="I335" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit mettre à jour les plans de réponse et de rétablissement pour tenir compte des changements survenus dans son contexte.</t>
-        </is>
-      </c>
-      <c r="J335" s="18" t="inlineStr">
-        <is>
-          <t>Le contexte de l'organisation concerne la structure organisationnelle, ses systèmes critiques, les vecteurs d'attaque, les nouvelles menaces, les améliorations technologiques, l'environnement d'exploitation, les problèmes rencontrés lors de la mise en œuvre/exécution/test du plan et les enseignements tirés.</t>
-        </is>
-      </c>
-      <c r="L335" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de reactie- en herstelplannen aanpassen aan veranderingen in haar context.</t>
-        </is>
-      </c>
-      <c r="M335" s="18" t="inlineStr">
-        <is>
-          <t>De context van de organisatie heeft betrekking op de organisatiestructuur, haar kritieke systemen, aanvalsvectoren, nieuwe bedreigingen, verbeterde technologie, de bedrijfsomgeving, problemen die zich hebben voorgedaan tijdens de implementatie/uitvoering/testen van het plan en de lessen die zijn geleerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="B336" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D336" s="5" t="inlineStr">
-        <is>
-          <t>RC</t>
-        </is>
-      </c>
-      <c r="E336" s="5" t="inlineStr">
-        <is>
-          <t>RECOVER (RC)</t>
-        </is>
-      </c>
-      <c r="H336" s="5" t="inlineStr">
-        <is>
-          <t>RETABLIR (RC)</t>
-        </is>
-      </c>
-      <c r="I336" t="inlineStr"/>
-      <c r="J336" t="inlineStr"/>
-      <c r="K336" s="7" t="inlineStr">
-        <is>
-          <t>HERSTELLEN (RC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="337" ht="57.6" customHeight="1">
-      <c r="B337" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D337" s="8" t="inlineStr">
-        <is>
-          <t>RC.RP</t>
-        </is>
-      </c>
-      <c r="E337" s="8" t="inlineStr">
-        <is>
-          <t>Recovery Planning</t>
-        </is>
-      </c>
-      <c r="F337" s="9" t="inlineStr">
-        <is>
-          <t>Recovery processes and procedures are executed and maintained to ensure restoration of systems or assets affected by cybersecurity incidents.</t>
-        </is>
-      </c>
-      <c r="H337" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Planification du rétablissement </t>
-        </is>
-      </c>
-      <c r="I337" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J337" t="inlineStr"/>
-      <c r="K337" s="11" t="inlineStr">
-        <is>
-          <t>Herstelplanning</t>
-        </is>
-      </c>
-      <c r="L337" s="12" t="inlineStr">
-        <is>
-          <t>Herstelprocessen en -procedures worden uitgevoerd en gehandhaafd om te zorgen voor herstel van systemen of activa die zijn getroffen door cyberbeveiligingsincidenten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="338" ht="28.8" customHeight="1">
-      <c r="B338" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D338" s="13" t="inlineStr">
-        <is>
-          <t>RC.RP-1</t>
-        </is>
-      </c>
-      <c r="F338" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recovery plan is executed during or after a cybersecurity incident </t>
-        </is>
-      </c>
-      <c r="I338" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Le plan de reprise est exécuté pendant ou après un incident de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J338" t="inlineStr"/>
-      <c r="L338" s="16" t="inlineStr">
-        <is>
-          <t>Het herstelplan wordt uitgevoerd tijdens of na een cyberbeveiligingsincident.</t>
-        </is>
-      </c>
-    </row>
-    <row r="339" ht="244.8" customHeight="1">
-      <c r="A339" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B339" t="n">
-        <v>4</v>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>B,I,E</t>
-        </is>
-      </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>BASIC_RC.RP-1.1</t>
-        </is>
-      </c>
-      <c r="F339" s="17" t="inlineStr">
-        <is>
-          <t>A recovery process for disasters and information/cybersecurity incidents shall be developed and executed as appropriate.</t>
-        </is>
-      </c>
-      <c r="G339" s="17" t="inlineStr">
         <is>
           <t>A process should be developed for what immediate actions will be taken in case of a fire, medical emergency, burglary, natural disaster, or  an information/cyber security incident.
 This process should consider:
@@ -15798,12 +15585,12 @@
 •	Who to call in case of an incident.</t>
         </is>
       </c>
-      <c r="I339" s="18" t="inlineStr">
+      <c r="I335" s="18" t="inlineStr">
         <is>
           <t>Un processus de rétablissement en cas de catastrophes et d'incidents liés à l'information et à la cybersécurité est élaboré et exécuté selon les besoins.</t>
         </is>
       </c>
-      <c r="J339" s="18" t="inlineStr">
+      <c r="J335" s="18" t="inlineStr">
         <is>
           <t>• Il convient qu’un processus soit élaboré pour déterminer les mesures immédiates à prendre en cas d'incendie, d'urgence médicale, de cambriolage, de catastrophe naturelle ou d'incident de sécurité informatique.
 • Il convient que ce processus prenne en compte : 
@@ -15812,12 +15599,12 @@
 	o Qui appeler en cas d'incident.</t>
         </is>
       </c>
-      <c r="L339" s="18" t="inlineStr">
+      <c r="L335" s="18" t="inlineStr">
         <is>
           <t>Er moet een herstelproces voor rampen en informatie-/cyberbeveiligingsincidenten worden ontwikkeld en zo nodig uitgevoerd.+L339</t>
         </is>
       </c>
-      <c r="M339" s="18" t="inlineStr">
+      <c r="M335" s="18" t="inlineStr">
         <is>
           <t>• Er zou een proces moeten worden ontwikkeld voor de onmiddellijke acties in geval van brand, medisch noodgeval, inbraak, natuurramp of een incident op het gebied van informatie-/cyberbeveiliging. 
 • Dit proces zou rekening moeten houden met: 
@@ -15827,120 +15614,283 @@
         </is>
       </c>
     </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>4</v>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>RC.RP-1.2</t>
+        </is>
+      </c>
+      <c r="F336" s="17" t="inlineStr">
+        <is>
+          <t>The essential organization’s functions and services shall be continued with little or no loss of operational continuity and continuity shall be sustained until full system restoration.</t>
+        </is>
+      </c>
+      <c r="G336" s="17" t="inlineStr">
+        <is>
+          <t>No additional guidance on this topic.</t>
+        </is>
+      </c>
+      <c r="I336" s="18" t="inlineStr">
+        <is>
+          <t>Les fonctions et services de l'organisation essentielle doivent être poursuivis avec peu ou pas de perte de continuité opérationnelle et la continuité doit être maintenue jusqu'à la restauration complète du système.</t>
+        </is>
+      </c>
+      <c r="J336" s="18" t="inlineStr">
+        <is>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+        </is>
+      </c>
+      <c r="L336" s="18" t="inlineStr">
+        <is>
+          <t>De essentiële functies en diensten van de organisatie moeten worden voortgezet met weinig of geen verlies van operationele continuïteit en de continuïteit moet worden gehandhaafd totdat het systeem volledig is hersteld.</t>
+        </is>
+      </c>
+      <c r="M336" s="18" t="inlineStr">
+        <is>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="57.6" customHeight="1">
+      <c r="B337" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D337" s="8" t="inlineStr">
+        <is>
+          <t>RC.IM</t>
+        </is>
+      </c>
+      <c r="E337" s="8" t="inlineStr">
+        <is>
+          <t>Improvements</t>
+        </is>
+      </c>
+      <c r="F337" s="9" t="inlineStr">
+        <is>
+          <t>Recovery planning and processes are improved by incorporating lessons learned into future activities.</t>
+        </is>
+      </c>
+      <c r="H337" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Améliorations </t>
+        </is>
+      </c>
+      <c r="I337" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K337" s="11" t="inlineStr">
+        <is>
+          <t>Verbeteringen</t>
+        </is>
+      </c>
+      <c r="L337" s="12" t="inlineStr">
+        <is>
+          <t>De herstelplanning en -processen worden verbeterd door in toekomstige activiteiten rekening te houden met de opgedane ervaring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="28.8" customHeight="1">
+      <c r="B338" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D338" s="13" t="inlineStr">
+        <is>
+          <t>RC.IM-1</t>
+        </is>
+      </c>
+      <c r="F338" s="14" t="inlineStr">
+        <is>
+          <t>Recovery plans incorporate lessons learned</t>
+        </is>
+      </c>
+      <c r="I338" s="15" t="inlineStr">
+        <is>
+          <t>Les plans de rétablissement intègrent les leçons apprises.</t>
+        </is>
+      </c>
+      <c r="L338" s="16" t="inlineStr">
+        <is>
+          <t>In de herstelplannen zijn de geleerde lessen verwerkt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="244.8" customHeight="1">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>4</v>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RC.IM-1.1</t>
+        </is>
+      </c>
+      <c r="F339" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall incorporate lessons learned from incident recovery activities into updated or new system recovery procedures and, after testing, frame this with appropriate training.</t>
+        </is>
+      </c>
+      <c r="G339" s="17" t="inlineStr">
+        <is>
+          <t>No additional guidance on this topic.</t>
+        </is>
+      </c>
+      <c r="I339" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit intégrer les enseignements tirés des activités de rétablissement des incidents dans les procédures de rétablissement du système, nouvelles ou mises à jour, et, après les avoir testées, les encadrer par une formation appropriée.</t>
+        </is>
+      </c>
+      <c r="J339" s="18" t="inlineStr">
+        <is>
+          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+        </is>
+      </c>
+      <c r="L339" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de lessen die zijn getrokken uit herstelactiviteiten bij incidenten verwerken in bijgewerkte of nieuwe herstelprocedures voor systemen en dit, na het testen, borgen met een passende opleiding.</t>
+        </is>
+      </c>
+      <c r="M339" s="18" t="inlineStr">
+        <is>
+          <t>Er zijn geen aanvullende richtsnoeren.</t>
+        </is>
+      </c>
+    </row>
     <row r="340" ht="72" customHeight="1">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B340" t="n">
-        <v>4</v>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>RC.RP-1.2</t>
-        </is>
-      </c>
-      <c r="F340" s="17" t="inlineStr">
-        <is>
-          <t>The essential organization’s functions and services shall be continued with little or no loss of operational continuity and continuity shall be sustained until full system restoration.</t>
-        </is>
-      </c>
-      <c r="G340" s="17" t="inlineStr">
-        <is>
-          <t>No additional guidance on this topic.</t>
-        </is>
-      </c>
-      <c r="I340" s="18" t="inlineStr">
-        <is>
-          <t>Les fonctions et services de l'organisation essentielle doivent être poursuivis avec peu ou pas de perte de continuité opérationnelle et la continuité doit être maintenue jusqu'à la restauration complète du système.</t>
-        </is>
-      </c>
-      <c r="J340" s="18" t="inlineStr">
-        <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
-        </is>
-      </c>
-      <c r="L340" s="18" t="inlineStr">
-        <is>
-          <t>De essentiële functies en diensten van de organisatie moeten worden voortgezet met weinig of geen verlies van operationele continuïteit en de continuïteit moet worden gehandhaafd totdat het systeem volledig is hersteld.</t>
-        </is>
-      </c>
-      <c r="M340" s="18" t="inlineStr">
-        <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+      <c r="B340" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D340" s="8" t="inlineStr">
+        <is>
+          <t>RC.CO</t>
+        </is>
+      </c>
+      <c r="E340" s="8" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="F340" s="9" t="inlineStr">
+        <is>
+          <t>Restoration activities are coordinated with internal and external parties (e.g.  coordinating centers, Internet Service Providers, owners of attacking systems, victims, other CSIRTs, and vendors).</t>
+        </is>
+      </c>
+      <c r="H340" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Communications </t>
+        </is>
+      </c>
+      <c r="I340" s="11" t="inlineStr">
+        <is>
+          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
+        </is>
+      </c>
+      <c r="K340" s="11" t="inlineStr">
+        <is>
+          <t>Communicatie</t>
+        </is>
+      </c>
+      <c r="L340" s="12" t="inlineStr">
+        <is>
+          <t>Herstelactiviteiten worden gecoördineerd met interne en externe partijen (bv. coördinatiecentra, internetproviders, eigenaars van aanvallende systemen, slachtoffers, andere CSIRT's en verkopers).</t>
         </is>
       </c>
     </row>
     <row r="341" ht="57.6" customHeight="1">
-      <c r="B341" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D341" s="8" t="inlineStr">
-        <is>
-          <t>RC.IM</t>
-        </is>
-      </c>
-      <c r="E341" s="8" t="inlineStr">
-        <is>
-          <t>Improvements</t>
-        </is>
-      </c>
-      <c r="F341" s="9" t="inlineStr">
-        <is>
-          <t>Recovery planning and processes are improved by incorporating lessons learned into future activities.</t>
-        </is>
-      </c>
-      <c r="H341" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Améliorations </t>
-        </is>
-      </c>
-      <c r="I341" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J341" t="inlineStr"/>
-      <c r="K341" s="11" t="inlineStr">
-        <is>
-          <t>Verbeteringen</t>
-        </is>
-      </c>
-      <c r="L341" s="12" t="inlineStr">
-        <is>
-          <t>De herstelplanning en -processen worden verbeterd door in toekomstige activiteiten rekening te houden met de opgedane ervaring.</t>
+      <c r="B341" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D341" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-1</t>
+        </is>
+      </c>
+      <c r="F341" s="14" t="inlineStr">
+        <is>
+          <t>Public relations are managed</t>
+        </is>
+      </c>
+      <c r="I341" s="15" t="inlineStr">
+        <is>
+          <t>Les relations publiques sont gérées.</t>
+        </is>
+      </c>
+      <c r="L341" s="16" t="inlineStr">
+        <is>
+          <t>De public relations worden beheerd.</t>
         </is>
       </c>
     </row>
     <row r="342" ht="28.8" customHeight="1">
-      <c r="B342" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D342" s="13" t="inlineStr">
-        <is>
-          <t>RC.IM-1</t>
-        </is>
-      </c>
-      <c r="F342" s="14" t="inlineStr">
-        <is>
-          <t>Recovery plans incorporate lessons learned</t>
-        </is>
-      </c>
-      <c r="I342" s="15" t="inlineStr">
-        <is>
-          <t>Les plans de rétablissement intègrent les leçons apprises.</t>
-        </is>
-      </c>
-      <c r="J342" t="inlineStr"/>
-      <c r="L342" s="16" t="inlineStr">
-        <is>
-          <t>In de herstelplannen zijn de geleerde lessen verwerkt.</t>
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B342" t="n">
+        <v>4</v>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>I,E</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>IMPORTANT_RC.CO-1.1</t>
+        </is>
+      </c>
+      <c r="F342" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall centralize and coordinate how information is disseminated and manage how the organization is presented to the public.</t>
+        </is>
+      </c>
+      <c r="G342" s="17" t="inlineStr">
+        <is>
+          <t>Public relations management may include, for example, managing media interactions, coordinating and logging all requests for interviews, handling and ‘triaging’ phone calls and e-mail requests, matching media requests with appropriate and available internal experts who are ready to be interviewed, screening all of information provided to the media, ensuring personnel are familiar with public relations and privacy policies.</t>
+        </is>
+      </c>
+      <c r="I342" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit centraliser et coordonner la manière dont les informations sont diffusées et gérer la manière dont l'organisation est présentée au public.</t>
+        </is>
+      </c>
+      <c r="J342" s="18" t="inlineStr">
+        <is>
+          <t>La gestion des relations publiques peut comprendre, par exemple, la gestion des interactions avec les médias, la coordination et l'enregistrement de toutes les demandes d'interviews, le traitement et le triage des appels téléphoniques et des demandes par e-mail, la mise en relation des demandes des médias avec les experts internes appropriés et disponibles qui sont prêts à être interviewés, le filtrage de toutes les informations fournies aux médias, l'assurance que le personnel connaît bien les politiques en matière de relations publiques et de confidentialité.</t>
+        </is>
+      </c>
+      <c r="L342" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
+        </is>
+      </c>
+      <c r="M342" s="18" t="inlineStr">
+        <is>
+          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
         </is>
       </c>
     </row>
@@ -15955,159 +15905,143 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>I,E</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>IMPORTANT_RC.IM-1.1</t>
+          <t>RC.CO-1.2</t>
         </is>
       </c>
       <c r="F343" s="17" t="inlineStr">
         <is>
-          <t>The organization shall incorporate lessons learned from incident recovery activities into updated or new system recovery procedures and, after testing, frame this with appropriate training.</t>
+          <t>A Public Relations Officer shall be assigned.</t>
         </is>
       </c>
       <c r="G343" s="17" t="inlineStr">
         <is>
-          <t>No additional guidance on this topic.</t>
+          <t>The Public Relations Officer should consider the use of pre-define external contacts 
+(e.g. press, regulators, interest groups).</t>
         </is>
       </c>
       <c r="I343" s="18" t="inlineStr">
         <is>
-          <t>L'organisation doit intégrer les enseignements tirés des activités de rétablissement des incidents dans les procédures de rétablissement du système, nouvelles ou mises à jour, et, après les avoir testées, les encadrer par une formation appropriée.</t>
+          <t>Un responsable des relations publiques est désigné.</t>
         </is>
       </c>
       <c r="J343" s="18" t="inlineStr">
         <is>
-          <t>Aucune orientation supplémentaire sur ce sujet.</t>
+          <t>Il convient que le responsable des relations publiques envisage l'utilisation de contacts externes prédéfinis (par exemple, la presse, les régulateurs, les groupes d'intérêt).</t>
         </is>
       </c>
       <c r="L343" s="18" t="inlineStr">
         <is>
-          <t>De organisatie moet de lessen die zijn getrokken uit herstelactiviteiten bij incidenten verwerken in bijgewerkte of nieuwe herstelprocedures voor systemen en dit, na het testen, borgen met een passende opleiding.</t>
+          <t>Er moet een Public Relations Officer worden aangesteld.</t>
         </is>
       </c>
       <c r="M343" s="18" t="inlineStr">
         <is>
-          <t>Er zijn geen aanvullende richtsnoeren.</t>
+          <t>De Public Relations Officer zou moeten overwegen gebruik te maken van vooraf bepaalde externe contacten (bijv. pers, regelgevers, belangengroepen).</t>
         </is>
       </c>
     </row>
     <row r="344" ht="57.6" customHeight="1">
-      <c r="B344" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D344" s="8" t="inlineStr">
-        <is>
-          <t>RC.CO</t>
-        </is>
-      </c>
-      <c r="E344" s="8" t="inlineStr">
-        <is>
-          <t>Communications</t>
-        </is>
-      </c>
-      <c r="F344" s="9" t="inlineStr">
-        <is>
-          <t>Restoration activities are coordinated with internal and external parties (e.g.  coordinating centers, Internet Service Providers, owners of attacking systems, victims, other CSIRTs, and vendors).</t>
-        </is>
-      </c>
-      <c r="H344" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Communications </t>
-        </is>
-      </c>
-      <c r="I344" s="11" t="inlineStr">
-        <is>
-          <t>Des processus et des procédures de rétablissement sont exécutés et maintenus pour assurer la restauration des systèmes ou des actifs touchés par des incidents de cybersécurité.</t>
-        </is>
-      </c>
-      <c r="J344" t="inlineStr"/>
-      <c r="K344" s="11" t="inlineStr">
-        <is>
-          <t>Communicatie</t>
-        </is>
-      </c>
-      <c r="L344" s="12" t="inlineStr">
-        <is>
-          <t>Herstelactiviteiten worden gecoördineerd met interne en externe partijen (bv. coördinatiecentra, internetproviders, eigenaars van aanvallende systemen, slachtoffers, andere CSIRT's en verkopers).</t>
+      <c r="B344" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D344" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-2</t>
+        </is>
+      </c>
+      <c r="F344" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reputation is repaired after an incident </t>
+        </is>
+      </c>
+      <c r="I344" s="15" t="inlineStr">
+        <is>
+          <t>La réputation est réparée après un incident.</t>
+        </is>
+      </c>
+      <c r="L344" s="16" t="inlineStr">
+        <is>
+          <t>Reputatie wordt hersteld na een incident.</t>
         </is>
       </c>
     </row>
     <row r="345">
-      <c r="B345" s="13" t="n">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>4</v>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>RC.CO-2.1</t>
+        </is>
+      </c>
+      <c r="F345" s="17" t="inlineStr">
+        <is>
+          <t>The organization shall implement a crisis response strategy to protect the organization from the negative consequences of a crisis and help restore its reputation.</t>
+        </is>
+      </c>
+      <c r="G345" s="17" t="inlineStr">
+        <is>
+          <t>Crisis response strategies include, for example, actions to shape attributions of the crisis, change perceptions of the organization in crisis, and reduce the negative effect generated by the crisis.</t>
+        </is>
+      </c>
+      <c r="I345" s="18" t="inlineStr">
+        <is>
+          <t>L'organisation doit mettre en œuvre une stratégie de réponse aux crises afin de protéger l'organisation des conséquences négatives d'une crise et de contribuer à restaurer sa réputation.</t>
+        </is>
+      </c>
+      <c r="J345" s="18" t="inlineStr">
+        <is>
+          <t>Les stratégies de réponse aux crises comprennent, par exemple, des actions visant à déterminer les attributions de la crise, à modifier les perceptions de l'organisation en crise et à réduire l'effet négatif généré par la crise.</t>
+        </is>
+      </c>
+      <c r="L345" s="18" t="inlineStr">
+        <is>
+          <t>Er moet een crisisbestrijdingsstrategie worden toegepast om de organisatie te beschermen tegen de negatieve gevolgen van een crisis en te helpen haar reputatie te herstellen.</t>
+        </is>
+      </c>
+      <c r="M345" s="18" t="inlineStr">
+        <is>
+          <t>Crisisbestrijdingsstrategieën omvatten bijvoorbeeld maatregelen om de beeldvorming over de crisis vorm te geven, de perceptie van de organisatie in crisis te veranderen, en het negatieve effect dat de crisis teweegbrengt te verminderen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="158.4" customHeight="1">
+      <c r="B346" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D345" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-1</t>
-        </is>
-      </c>
-      <c r="F345" s="14" t="inlineStr">
-        <is>
-          <t>Public relations are managed</t>
-        </is>
-      </c>
-      <c r="I345" s="15" t="inlineStr">
-        <is>
-          <t>Les relations publiques sont gérées.</t>
-        </is>
-      </c>
-      <c r="J345" t="inlineStr"/>
-      <c r="L345" s="16" t="inlineStr">
-        <is>
-          <t>De public relations worden beheerd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="346" ht="158.4" customHeight="1">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B346" t="n">
-        <v>4</v>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RC.CO-1.1</t>
-        </is>
-      </c>
-      <c r="F346" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall centralize and coordinate how information is disseminated and manage how the organization is presented to the public.</t>
-        </is>
-      </c>
-      <c r="G346" s="17" t="inlineStr">
-        <is>
-          <t>Public relations management may include, for example, managing media interactions, coordinating and logging all requests for interviews, handling and ‘triaging’ phone calls and e-mail requests, matching media requests with appropriate and available internal experts who are ready to be interviewed, screening all of information provided to the media, ensuring personnel are familiar with public relations and privacy policies.</t>
-        </is>
-      </c>
-      <c r="I346" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit centraliser et coordonner la manière dont les informations sont diffusées et gérer la manière dont l'organisation est présentée au public.</t>
-        </is>
-      </c>
-      <c r="J346" s="18" t="inlineStr">
-        <is>
-          <t>La gestion des relations publiques peut comprendre, par exemple, la gestion des interactions avec les médias, la coordination et l'enregistrement de toutes les demandes d'interviews, le traitement et le triage des appels téléphoniques et des demandes par e-mail, la mise en relation des demandes des médias avec les experts internes appropriés et disponibles qui sont prêts à être interviewés, le filtrage de toutes les informations fournies aux médias, l'assurance que le personnel connaît bien les politiques en matière de relations publiques et de confidentialité.</t>
-        </is>
-      </c>
-      <c r="L346" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
-        </is>
-      </c>
-      <c r="M346" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de wijze waarop informatie wordt verspreid centraliseren en coördineren, en beheert de wijze waarop de organisatie aan het publiek wordt gepresenteerd.</t>
+      <c r="D346" s="13" t="inlineStr">
+        <is>
+          <t>RC.CO-3</t>
+        </is>
+      </c>
+      <c r="F346" s="14" t="inlineStr">
+        <is>
+          <t>Recovery activities are communicated to internal and external stakeholders as well as executive and management teams</t>
+        </is>
+      </c>
+      <c r="I346" s="15" t="inlineStr">
+        <is>
+          <t>Les activités de rétablissement sont communiquées aux parties prenantes internes et externes, ainsi qu'aux équipes de direction et de gestion.</t>
+        </is>
+      </c>
+      <c r="L346" s="16" t="inlineStr">
+        <is>
+          <t>De herstelactiviteiten worden gecommuniceerd aan interne en externe belanghebbenden en aan directie- en managementteams.</t>
         </is>
       </c>
     </row>
@@ -16122,198 +16056,48 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>I,E</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>RC.CO-1.2</t>
+          <t>IMPORTANT_RC.CO-3.1</t>
         </is>
       </c>
       <c r="F347" s="17" t="inlineStr">
         <is>
-          <t>A Public Relations Officer shall be assigned.</t>
+          <t>The organization shall communicate recovery activities to predefined stakeholders, executive and management teams.</t>
         </is>
       </c>
       <c r="G347" s="17" t="inlineStr">
         <is>
-          <t>The Public Relations Officer should consider the use of pre-define external contacts 
-(e.g. press, regulators, interest groups).</t>
+          <t>Communication of recovery activities to all relevant stakeholders applies only to entities subject to the NIS legislation.</t>
         </is>
       </c>
       <c r="I347" s="18" t="inlineStr">
         <is>
-          <t>Un responsable des relations publiques est désigné.</t>
+          <t>L'organisation doit communiquer les activités de rétablissement aux parties prenantes prédéfinies, aux équipes de direction et de gestion.</t>
         </is>
       </c>
       <c r="J347" s="18" t="inlineStr">
         <is>
-          <t>Il convient que le responsable des relations publiques envisage l'utilisation de contacts externes prédéfinis (par exemple, la presse, les régulateurs, les groupes d'intérêt).</t>
+          <t>La communication des activités de rétablissement à toutes les parties prenantes concernées ne s'applique qu'aux entités soumises à la législation NIS.</t>
         </is>
       </c>
       <c r="L347" s="18" t="inlineStr">
         <is>
-          <t>Er moet een Public Relations Officer worden aangesteld.</t>
+          <t>De organisatie moet de herstelactiviteiten meedelen aan vooraf bepaalde belanghebbenden, directie- en managementteams.</t>
         </is>
       </c>
       <c r="M347" s="18" t="inlineStr">
         <is>
-          <t>De Public Relations Officer zou moeten overwegen gebruik te maken van vooraf bepaalde externe contacten (bijv. pers, regelgevers, belangengroepen).</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="B348" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D348" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-2</t>
-        </is>
-      </c>
-      <c r="F348" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reputation is repaired after an incident </t>
-        </is>
-      </c>
-      <c r="I348" s="15" t="inlineStr">
-        <is>
-          <t>La réputation est réparée après un incident.</t>
-        </is>
-      </c>
-      <c r="J348" t="inlineStr"/>
-      <c r="L348" s="16" t="inlineStr">
-        <is>
-          <t>Reputatie wordt hersteld na een incident.</t>
-        </is>
-      </c>
-    </row>
-    <row r="349" ht="72" customHeight="1">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B349" t="n">
-        <v>4</v>
-      </c>
-      <c r="C349" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D349" t="inlineStr">
-        <is>
-          <t>RC.CO-2.1</t>
-        </is>
-      </c>
-      <c r="F349" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall implement a crisis response strategy to protect the organization from the negative consequences of a crisis and help restore its reputation.</t>
-        </is>
-      </c>
-      <c r="G349" s="17" t="inlineStr">
-        <is>
-          <t>Crisis response strategies include, for example, actions to shape attributions of the crisis, change perceptions of the organization in crisis, and reduce the negative effect generated by the crisis.</t>
-        </is>
-      </c>
-      <c r="I349" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit mettre en œuvre une stratégie de réponse aux crises afin de protéger l'organisation des conséquences négatives d'une crise et de contribuer à restaurer sa réputation.</t>
-        </is>
-      </c>
-      <c r="J349" s="18" t="inlineStr">
-        <is>
-          <t>Les stratégies de réponse aux crises comprennent, par exemple, des actions visant à déterminer les attributions de la crise, à modifier les perceptions de l'organisation en crise et à réduire l'effet négatif généré par la crise.</t>
-        </is>
-      </c>
-      <c r="L349" s="18" t="inlineStr">
-        <is>
-          <t>Er moet een crisisbestrijdingsstrategie worden toegepast om de organisatie te beschermen tegen de negatieve gevolgen van een crisis en te helpen haar reputatie te herstellen.</t>
-        </is>
-      </c>
-      <c r="M349" s="18" t="inlineStr">
-        <is>
-          <t>Crisisbestrijdingsstrategieën omvatten bijvoorbeeld maatregelen om de beeldvorming over de crisis vorm te geven, de perceptie van de organisatie in crisis te veranderen, en het negatieve effect dat de crisis teweegbrengt te verminderen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="350" ht="43.2" customHeight="1">
-      <c r="B350" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D350" s="13" t="inlineStr">
-        <is>
-          <t>RC.CO-3</t>
-        </is>
-      </c>
-      <c r="F350" s="14" t="inlineStr">
-        <is>
-          <t>Recovery activities are communicated to internal and external stakeholders as well as executive and management teams</t>
-        </is>
-      </c>
-      <c r="I350" s="15" t="inlineStr">
-        <is>
-          <t>Les activités de rétablissement sont communiquées aux parties prenantes internes et externes, ainsi qu'aux équipes de direction et de gestion.</t>
-        </is>
-      </c>
-      <c r="J350" t="inlineStr"/>
-      <c r="L350" s="16" t="inlineStr">
-        <is>
-          <t>De herstelactiviteiten worden gecommuniceerd aan interne en externe belanghebbenden en aan directie- en managementteams.</t>
-        </is>
-      </c>
-    </row>
-    <row r="351" ht="57.6" customHeight="1">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B351" t="n">
-        <v>4</v>
-      </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>I,E</t>
-        </is>
-      </c>
-      <c r="D351" t="inlineStr">
-        <is>
-          <t>IMPORTANT_RC.CO-3.1</t>
-        </is>
-      </c>
-      <c r="F351" s="17" t="inlineStr">
-        <is>
-          <t>The organization shall communicate recovery activities to predefined stakeholders, executive and management teams.</t>
-        </is>
-      </c>
-      <c r="G351" s="17" t="inlineStr">
-        <is>
-          <t>Communication of recovery activities to all relevant stakeholders applies only to entities subject to the NIS legislation.</t>
-        </is>
-      </c>
-      <c r="I351" s="18" t="inlineStr">
-        <is>
-          <t>L'organisation doit communiquer les activités de rétablissement aux parties prenantes prédéfinies, aux équipes de direction et de gestion.</t>
-        </is>
-      </c>
-      <c r="J351" s="18" t="inlineStr">
-        <is>
-          <t>La communication des activités de rétablissement à toutes les parties prenantes concernées ne s'applique qu'aux entités soumises à la législation NIS.</t>
-        </is>
-      </c>
-      <c r="L351" s="18" t="inlineStr">
-        <is>
-          <t>De organisatie moet de herstelactiviteiten meedelen aan vooraf bepaalde belanghebbenden, directie- en managementteams.</t>
-        </is>
-      </c>
-      <c r="M351" s="18" t="inlineStr">
-        <is>
           <t>Communicatie van herstelactiviteiten aan belanghebbenden geldt alleen voor entiteiten die onder de NIS- wetgeving vallen.</t>
         </is>
       </c>
     </row>
+    <row r="349" ht="72" customHeight="1"/>
+    <row r="350" ht="43.2" customHeight="1"/>
+    <row r="351" ht="57.6" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>